<commit_message>
Public Rail + Tech Frac Fixes
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{12930437-8380-4A20-BC55-0F37E67B4891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1B8D76C-00D5-4846-BCB1-A43933AB5893}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{EE2E0D63-B56C-4BDE-BCAD-5F60909CE8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7CC7D6-F03E-4234-BF37-5810BC20243F}"/>
   <bookViews>
-    <workbookView xWindow="29070" yWindow="-14715" windowWidth="16440" windowHeight="29040" tabRatio="821" activeTab="1" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="821" firstSheet="14" activeTab="18" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -26,13 +26,17 @@
     <sheet name="Transit_Costs" sheetId="16" r:id="rId11"/>
     <sheet name="NTD_Service" sheetId="12" r:id="rId12"/>
     <sheet name="Fuel_Factors" sheetId="14" r:id="rId13"/>
-    <sheet name="Fuel_Factors_Revision" sheetId="22" r:id="rId14"/>
-    <sheet name="Warming_Potential" sheetId="17" r:id="rId15"/>
+    <sheet name="Fuel_Factors_Baselines" sheetId="27" r:id="rId14"/>
+    <sheet name="Fuel_Factors_Revision" sheetId="22" r:id="rId15"/>
+    <sheet name="Warming_Potential" sheetId="17" r:id="rId16"/>
+    <sheet name="EV_Forecast" sheetId="23" r:id="rId17"/>
+    <sheet name="Passenger_Rail_State_Mileage" sheetId="24" r:id="rId18"/>
+    <sheet name="Passenger_Rail_FuelFactors" sheetId="25" r:id="rId19"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId16"/>
-    <externalReference r:id="rId17"/>
-    <externalReference r:id="rId18"/>
+    <externalReference r:id="rId20"/>
+    <externalReference r:id="rId21"/>
+    <externalReference r:id="rId22"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">AEO_VMT_Base!$A$1:$C$1</definedName>
@@ -87,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8384" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8606" uniqueCount="333">
   <si>
     <t>state</t>
   </si>
@@ -1009,6 +1013,84 @@
   <si>
     <t>CO2eq_g_kWh</t>
   </si>
+  <si>
+    <t>percEVstock_AEO</t>
+  </si>
+  <si>
+    <t>percEVstock_ACCII</t>
+  </si>
+  <si>
+    <t>percEVstock_ACC</t>
+  </si>
+  <si>
+    <t>percEVstock_ACCACT</t>
+  </si>
+  <si>
+    <t>percEVstock_ACCIIACT</t>
+  </si>
+  <si>
+    <t>Heavy Duty Truck</t>
+  </si>
+  <si>
+    <t>Light Duty Truck</t>
+  </si>
+  <si>
+    <t>Medium Duty Truck</t>
+  </si>
+  <si>
+    <t>Passenger Car</t>
+  </si>
+  <si>
+    <t>amtrak_riders</t>
+  </si>
+  <si>
+    <t>commuterrail_miles</t>
+  </si>
+  <si>
+    <t>heavyrail_miles</t>
+  </si>
+  <si>
+    <t>lightrail_miles</t>
+  </si>
+  <si>
+    <t>amtrak_Energy_Intensity_BTUPerPaxMil</t>
+  </si>
+  <si>
+    <t>CR_Energy_Intensity_BTUPerPaxMil</t>
+  </si>
+  <si>
+    <t>HR_Energy_Intensity_BTUPerPaxMil</t>
+  </si>
+  <si>
+    <t>LR_Energy_Intensity_BTUPerPaxMil</t>
+  </si>
+  <si>
+    <t>Propane</t>
+  </si>
+  <si>
+    <t>units</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>upstream_life_cycle_Factor</t>
+  </si>
+  <si>
+    <t>electricity</t>
+  </si>
+  <si>
+    <t>fuel_conversion_gasoline_equivalent</t>
+  </si>
+  <si>
+    <t>fuel_conversion_BTU</t>
+  </si>
+  <si>
+    <t>energy_efficiency_ratio</t>
+  </si>
+  <si>
+    <t>CNG to Diesel</t>
+  </si>
 </sst>
 </file>
 
@@ -1118,7 +1200,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1141,6 +1223,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2807,6 +2890,18 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{518D259B-7CFD-40C9-852E-5504E1166921}" name="Fuel_Factors_Baseline" displayName="Fuel_Factors_Baseline" ref="A1:C16" totalsRowShown="0">
+  <autoFilter ref="A1:C16" xr:uid="{518D259B-7CFD-40C9-852E-5504E1166921}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{CEC5F72C-E366-45EB-B906-60DFE2C20A8F}" name="fuel_type"/>
+    <tableColumn id="2" xr3:uid="{C607764C-F28E-4CFA-8C1F-C3427D0186D8}" name="units"/>
+    <tableColumn id="3" xr3:uid="{2CEB8B5E-0AE4-47CF-ADC1-6A60B25483AE}" name="value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{03AFADD4-FAEA-41F7-A128-A44DAF1E827F}" name="Fuel_Factors_Revision" displayName="Fuel_Factors_Revision" ref="A1:K39" totalsRowShown="0">
   <autoFilter ref="A1:K39" xr:uid="{03AFADD4-FAEA-41F7-A128-A44DAF1E827F}"/>
   <tableColumns count="11">
@@ -2826,12 +2921,57 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6DFCB0CB-F0C1-406B-8BC4-DBF1C6DEF1BD}" name="GWP" displayName="GWP" ref="A1:B3" totalsRowShown="0">
   <autoFilter ref="A1:B3" xr:uid="{6DFCB0CB-F0C1-406B-8BC4-DBF1C6DEF1BD}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C7571F8A-FAEB-418D-B890-7F650F2EC67E}" name="Gas"/>
     <tableColumn id="2" xr3:uid="{0A2C010A-79AE-435E-98A7-45ED8AF3EA48}" name="GWP"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{3D4BD3A3-7756-49E2-B00A-144DD3C0AB84}" name="EV_Forecast" displayName="EV_Forecast" ref="A1:G121" totalsRowShown="0">
+  <autoFilter ref="A1:G121" xr:uid="{3D4BD3A3-7756-49E2-B00A-144DD3C0AB84}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{98339C45-1FB4-4A31-A342-8A18C9D17CBF}" name="veh_type"/>
+    <tableColumn id="2" xr3:uid="{5448A7A5-8D60-4DB5-9002-C1C331D0B9BD}" name="year"/>
+    <tableColumn id="3" xr3:uid="{6C87E9A0-5979-4F0A-AEC0-A63C0F93051B}" name="percEVstock_AEO"/>
+    <tableColumn id="4" xr3:uid="{1AEA079B-7185-4543-8E7E-17320AB65398}" name="percEVstock_ACCII"/>
+    <tableColumn id="5" xr3:uid="{C201EFA0-9EE7-44A0-911D-38D56E3B907B}" name="percEVstock_ACC"/>
+    <tableColumn id="6" xr3:uid="{941DD455-3F84-44FE-BE56-FB8C7695A3F6}" name="percEVstock_ACCACT"/>
+    <tableColumn id="7" xr3:uid="{C571AE9D-EDC5-441E-BD86-18F36763A9BA}" name="percEVstock_ACCIIACT"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C9ACDE8-AAE2-4347-8072-D2D12BA0A2E5}" name="Passenger_Rail_State_Mileage" displayName="Passenger_Rail_State_Mileage" ref="A1:F52" totalsRowShown="0">
+  <autoFilter ref="A1:F52" xr:uid="{3C9ACDE8-AAE2-4347-8072-D2D12BA0A2E5}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{BDBC3F5C-D408-43E1-81EC-95C50C377D64}" name="state"/>
+    <tableColumn id="2" xr3:uid="{36E465BC-AC57-462E-8C5F-2264EACFA55C}" name="year"/>
+    <tableColumn id="3" xr3:uid="{469EDCC2-4A35-4A7D-AA02-B7FC795193D0}" name="amtrak_riders"/>
+    <tableColumn id="4" xr3:uid="{C72C4CFA-8DBF-437E-B532-4E876AF07824}" name="commuterrail_miles"/>
+    <tableColumn id="5" xr3:uid="{A69FEAF6-C35E-44ED-9457-60BCB7A154FD}" name="heavyrail_miles"/>
+    <tableColumn id="6" xr3:uid="{40439AC9-0C67-414F-A72A-182AB961EF72}" name="lightrail_miles"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}" name="Passenger_Rail_FuelFactors" displayName="Passenger_Rail_FuelFactors" ref="A1:E33" totalsRowShown="0">
+  <autoFilter ref="A1:E33" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{E1F2670B-316B-4194-A86B-8536CC6E5F6A}" name="year"/>
+    <tableColumn id="2" xr3:uid="{B177438D-BB65-4F5B-B9B2-4F2ACFB89EBB}" name="amtrak_Energy_Intensity_BTUPerPaxMil"/>
+    <tableColumn id="3" xr3:uid="{145EDF5A-67AC-4FBD-8747-BD532DBD07D2}" name="CR_Energy_Intensity_BTUPerPaxMil"/>
+    <tableColumn id="4" xr3:uid="{FABA830F-9553-48B4-B4E7-CA28DF0F2168}" name="HR_Energy_Intensity_BTUPerPaxMil"/>
+    <tableColumn id="5" xr3:uid="{5411A020-667E-4006-86A4-6CBDBC158F0A}" name="LR_Energy_Intensity_BTUPerPaxMil"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -19536,6 +19676,199 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFD11A43-B943-40FD-8C75-39E96A18C306}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" s="20">
+        <v>7.94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C3">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>289</v>
+      </c>
+      <c r="C4">
+        <v>5.4399999999999997E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C5">
+        <v>5.72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" t="s">
+        <v>327</v>
+      </c>
+      <c r="C6">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C7">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" t="s">
+        <v>327</v>
+      </c>
+      <c r="C8">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B9" t="s">
+        <v>329</v>
+      </c>
+      <c r="C9">
+        <v>33.977738722905684</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" t="s">
+        <v>329</v>
+      </c>
+      <c r="C10">
+        <v>0.89285714285714279</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>324</v>
+      </c>
+      <c r="B11" t="s">
+        <v>329</v>
+      </c>
+      <c r="C11">
+        <v>1.3513513513513513</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>329</v>
+      </c>
+      <c r="C12">
+        <v>123.57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" t="s">
+        <v>330</v>
+      </c>
+      <c r="C13">
+        <v>3414</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" t="s">
+        <v>330</v>
+      </c>
+      <c r="C14">
+        <v>116000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" t="s">
+        <v>330</v>
+      </c>
+      <c r="C15">
+        <v>128500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>332</v>
+      </c>
+      <c r="B16" t="s">
+        <v>331</v>
+      </c>
+      <c r="C16">
+        <v>0.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B8B760-61E2-4C3C-B734-67EBC38A98CD}">
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -20926,7 +21259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF48310-0F86-4489-96AB-7F1DA3A7B2B6}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -20953,6 +21286,4449 @@
       </c>
       <c r="B3">
         <v>298</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{241E29C4-5664-445C-AFC0-25E977A29D94}">
+  <dimension ref="A1:G121"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.6328125" customWidth="1"/>
+    <col min="4" max="4" width="18.54296875" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="6" max="6" width="20.7265625" customWidth="1"/>
+    <col min="7" max="7" width="21.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D1" t="s">
+        <v>308</v>
+      </c>
+      <c r="E1" t="s">
+        <v>309</v>
+      </c>
+      <c r="F1" t="s">
+        <v>310</v>
+      </c>
+      <c r="G1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>312</v>
+      </c>
+      <c r="B2">
+        <v>2021</v>
+      </c>
+      <c r="C2">
+        <v>1.7833599999999999E-4</v>
+      </c>
+      <c r="D2">
+        <v>1.7833599999999999E-4</v>
+      </c>
+      <c r="E2">
+        <v>1.7833599999999999E-4</v>
+      </c>
+      <c r="F2">
+        <v>1.7833599999999999E-4</v>
+      </c>
+      <c r="G2">
+        <v>1.7833599999999999E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B3">
+        <v>2022</v>
+      </c>
+      <c r="C3">
+        <v>3.3397599999999999E-4</v>
+      </c>
+      <c r="D3">
+        <v>3.3397599999999999E-4</v>
+      </c>
+      <c r="E3">
+        <v>3.3397599999999999E-4</v>
+      </c>
+      <c r="F3">
+        <v>3.3397599999999999E-4</v>
+      </c>
+      <c r="G3">
+        <v>3.3397599999999999E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B4">
+        <v>2023</v>
+      </c>
+      <c r="C4">
+        <v>4.9029200000000003E-4</v>
+      </c>
+      <c r="D4">
+        <v>4.9029200000000003E-4</v>
+      </c>
+      <c r="E4">
+        <v>4.9029200000000003E-4</v>
+      </c>
+      <c r="F4">
+        <v>4.9029200000000003E-4</v>
+      </c>
+      <c r="G4">
+        <v>4.9029200000000003E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5">
+        <v>2024</v>
+      </c>
+      <c r="C5">
+        <v>6.4432900000000002E-4</v>
+      </c>
+      <c r="D5">
+        <v>6.4432900000000002E-4</v>
+      </c>
+      <c r="E5">
+        <v>6.4432900000000002E-4</v>
+      </c>
+      <c r="F5">
+        <v>2.8879320000000002E-3</v>
+      </c>
+      <c r="G5">
+        <v>2.8879320000000002E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B6">
+        <v>2025</v>
+      </c>
+      <c r="C6">
+        <v>7.96417E-4</v>
+      </c>
+      <c r="D6">
+        <v>7.96417E-4</v>
+      </c>
+      <c r="E6">
+        <v>7.96417E-4</v>
+      </c>
+      <c r="F6">
+        <v>6.3800389999999997E-3</v>
+      </c>
+      <c r="G6">
+        <v>6.3800389999999997E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>312</v>
+      </c>
+      <c r="B7">
+        <v>2026</v>
+      </c>
+      <c r="C7">
+        <v>9.4634700000000005E-4</v>
+      </c>
+      <c r="D7">
+        <v>9.4634700000000005E-4</v>
+      </c>
+      <c r="E7">
+        <v>9.4634700000000005E-4</v>
+      </c>
+      <c r="F7">
+        <v>1.0761928E-2</v>
+      </c>
+      <c r="G7">
+        <v>1.0761928E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8">
+        <v>2027</v>
+      </c>
+      <c r="C8">
+        <v>1.0917800000000001E-3</v>
+      </c>
+      <c r="D8">
+        <v>1.0917800000000001E-3</v>
+      </c>
+      <c r="E8">
+        <v>1.0917800000000001E-3</v>
+      </c>
+      <c r="F8">
+        <v>1.6864591000000002E-2</v>
+      </c>
+      <c r="G8">
+        <v>1.6864591000000002E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>312</v>
+      </c>
+      <c r="B9">
+        <v>2028</v>
+      </c>
+      <c r="C9">
+        <v>1.234576E-3</v>
+      </c>
+      <c r="D9">
+        <v>1.234576E-3</v>
+      </c>
+      <c r="E9">
+        <v>1.234576E-3</v>
+      </c>
+      <c r="F9">
+        <v>2.5187912999999999E-2</v>
+      </c>
+      <c r="G9">
+        <v>2.5187912999999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>312</v>
+      </c>
+      <c r="B10">
+        <v>2029</v>
+      </c>
+      <c r="C10">
+        <v>1.377184E-3</v>
+      </c>
+      <c r="D10">
+        <v>1.377184E-3</v>
+      </c>
+      <c r="E10">
+        <v>1.377184E-3</v>
+      </c>
+      <c r="F10">
+        <v>3.5627709E-2</v>
+      </c>
+      <c r="G10">
+        <v>3.5627709E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B11">
+        <v>2030</v>
+      </c>
+      <c r="C11">
+        <v>1.5188409999999999E-3</v>
+      </c>
+      <c r="D11">
+        <v>1.5188409999999999E-3</v>
+      </c>
+      <c r="E11">
+        <v>1.5188409999999999E-3</v>
+      </c>
+      <c r="F11">
+        <v>4.7980977000000001E-2</v>
+      </c>
+      <c r="G11">
+        <v>4.7980977000000001E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>312</v>
+      </c>
+      <c r="B12">
+        <v>2031</v>
+      </c>
+      <c r="C12">
+        <v>1.6599869999999999E-3</v>
+      </c>
+      <c r="D12">
+        <v>1.6599869999999999E-3</v>
+      </c>
+      <c r="E12">
+        <v>1.6599869999999999E-3</v>
+      </c>
+      <c r="F12">
+        <v>6.1868593999999999E-2</v>
+      </c>
+      <c r="G12">
+        <v>6.1868593999999999E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>312</v>
+      </c>
+      <c r="B13">
+        <v>2032</v>
+      </c>
+      <c r="C13">
+        <v>1.8000679999999999E-3</v>
+      </c>
+      <c r="D13">
+        <v>1.8000679999999999E-3</v>
+      </c>
+      <c r="E13">
+        <v>1.8000679999999999E-3</v>
+      </c>
+      <c r="F13">
+        <v>7.6526794999999995E-2</v>
+      </c>
+      <c r="G13">
+        <v>7.6526794999999995E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>312</v>
+      </c>
+      <c r="B14">
+        <v>2033</v>
+      </c>
+      <c r="C14">
+        <v>1.9408330000000001E-3</v>
+      </c>
+      <c r="D14">
+        <v>1.9408330000000001E-3</v>
+      </c>
+      <c r="E14">
+        <v>1.9408330000000001E-3</v>
+      </c>
+      <c r="F14">
+        <v>9.1638549E-2</v>
+      </c>
+      <c r="G14">
+        <v>9.1638549E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>312</v>
+      </c>
+      <c r="B15">
+        <v>2034</v>
+      </c>
+      <c r="C15">
+        <v>2.0840559999999999E-3</v>
+      </c>
+      <c r="D15">
+        <v>2.0840559999999999E-3</v>
+      </c>
+      <c r="E15">
+        <v>2.0840559999999999E-3</v>
+      </c>
+      <c r="F15">
+        <v>0.106988207</v>
+      </c>
+      <c r="G15">
+        <v>0.106988207</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>312</v>
+      </c>
+      <c r="B16">
+        <v>2035</v>
+      </c>
+      <c r="C16">
+        <v>2.2269479999999999E-3</v>
+      </c>
+      <c r="D16">
+        <v>2.2269479999999999E-3</v>
+      </c>
+      <c r="E16">
+        <v>2.2269479999999999E-3</v>
+      </c>
+      <c r="F16">
+        <v>0.12328299600000001</v>
+      </c>
+      <c r="G16">
+        <v>0.12328299600000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>312</v>
+      </c>
+      <c r="B17">
+        <v>2036</v>
+      </c>
+      <c r="C17">
+        <v>2.3683300000000001E-3</v>
+      </c>
+      <c r="D17">
+        <v>2.3683300000000001E-3</v>
+      </c>
+      <c r="E17">
+        <v>2.3683300000000001E-3</v>
+      </c>
+      <c r="F17">
+        <v>0.13350161599999999</v>
+      </c>
+      <c r="G17">
+        <v>0.13350161599999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B18">
+        <v>2037</v>
+      </c>
+      <c r="C18">
+        <v>2.5096810000000002E-3</v>
+      </c>
+      <c r="D18">
+        <v>2.5096810000000002E-3</v>
+      </c>
+      <c r="E18">
+        <v>2.5096810000000002E-3</v>
+      </c>
+      <c r="F18">
+        <v>0.14717171300000001</v>
+      </c>
+      <c r="G18">
+        <v>0.14717171300000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>312</v>
+      </c>
+      <c r="B19">
+        <v>2038</v>
+      </c>
+      <c r="C19">
+        <v>2.6516360000000002E-3</v>
+      </c>
+      <c r="D19">
+        <v>2.6516360000000002E-3</v>
+      </c>
+      <c r="E19">
+        <v>2.6516360000000002E-3</v>
+      </c>
+      <c r="F19">
+        <v>0.159999847</v>
+      </c>
+      <c r="G19">
+        <v>0.159999847</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>312</v>
+      </c>
+      <c r="B20">
+        <v>2039</v>
+      </c>
+      <c r="C20">
+        <v>2.7978980000000001E-3</v>
+      </c>
+      <c r="D20">
+        <v>2.7978980000000001E-3</v>
+      </c>
+      <c r="E20">
+        <v>2.7978980000000001E-3</v>
+      </c>
+      <c r="F20">
+        <v>0.17197367399999999</v>
+      </c>
+      <c r="G20">
+        <v>0.17197367399999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>312</v>
+      </c>
+      <c r="B21">
+        <v>2040</v>
+      </c>
+      <c r="C21">
+        <v>2.9475489999999998E-3</v>
+      </c>
+      <c r="D21">
+        <v>2.9475489999999998E-3</v>
+      </c>
+      <c r="E21">
+        <v>2.9475489999999998E-3</v>
+      </c>
+      <c r="F21">
+        <v>0.18306308800000001</v>
+      </c>
+      <c r="G21">
+        <v>0.18306308800000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>312</v>
+      </c>
+      <c r="B22">
+        <v>2041</v>
+      </c>
+      <c r="C22">
+        <v>3.1025660000000002E-3</v>
+      </c>
+      <c r="D22">
+        <v>3.1025660000000002E-3</v>
+      </c>
+      <c r="E22">
+        <v>3.1025660000000002E-3</v>
+      </c>
+      <c r="F22">
+        <v>0.19322018599999999</v>
+      </c>
+      <c r="G22">
+        <v>0.19322018599999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>312</v>
+      </c>
+      <c r="B23">
+        <v>2042</v>
+      </c>
+      <c r="C23">
+        <v>3.2548310000000001E-3</v>
+      </c>
+      <c r="D23">
+        <v>3.2548310000000001E-3</v>
+      </c>
+      <c r="E23">
+        <v>3.2548310000000001E-3</v>
+      </c>
+      <c r="F23">
+        <v>0.20237197600000001</v>
+      </c>
+      <c r="G23">
+        <v>0.20237197600000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>312</v>
+      </c>
+      <c r="B24">
+        <v>2043</v>
+      </c>
+      <c r="C24">
+        <v>3.4059329999999999E-3</v>
+      </c>
+      <c r="D24">
+        <v>3.4059329999999999E-3</v>
+      </c>
+      <c r="E24">
+        <v>3.4059329999999999E-3</v>
+      </c>
+      <c r="F24">
+        <v>0.21056287000000001</v>
+      </c>
+      <c r="G24">
+        <v>0.21056287000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>312</v>
+      </c>
+      <c r="B25">
+        <v>2044</v>
+      </c>
+      <c r="C25">
+        <v>3.5547740000000001E-3</v>
+      </c>
+      <c r="D25">
+        <v>3.5547740000000001E-3</v>
+      </c>
+      <c r="E25">
+        <v>3.5547740000000001E-3</v>
+      </c>
+      <c r="F25">
+        <v>0.21777566700000001</v>
+      </c>
+      <c r="G25">
+        <v>0.21777566700000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>312</v>
+      </c>
+      <c r="B26">
+        <v>2045</v>
+      </c>
+      <c r="C26">
+        <v>3.702253E-3</v>
+      </c>
+      <c r="D26">
+        <v>3.702253E-3</v>
+      </c>
+      <c r="E26">
+        <v>3.702253E-3</v>
+      </c>
+      <c r="F26">
+        <v>0.224084228</v>
+      </c>
+      <c r="G26">
+        <v>0.224084228</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>312</v>
+      </c>
+      <c r="B27">
+        <v>2046</v>
+      </c>
+      <c r="C27">
+        <v>3.8532660000000002E-3</v>
+      </c>
+      <c r="D27">
+        <v>3.8532660000000002E-3</v>
+      </c>
+      <c r="E27">
+        <v>3.8532660000000002E-3</v>
+      </c>
+      <c r="F27">
+        <v>0.229570676</v>
+      </c>
+      <c r="G27">
+        <v>0.229570676</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>312</v>
+      </c>
+      <c r="B28">
+        <v>2047</v>
+      </c>
+      <c r="C28">
+        <v>4.0069169999999996E-3</v>
+      </c>
+      <c r="D28">
+        <v>4.0069169999999996E-3</v>
+      </c>
+      <c r="E28">
+        <v>4.0069169999999996E-3</v>
+      </c>
+      <c r="F28">
+        <v>0.23429806</v>
+      </c>
+      <c r="G28">
+        <v>0.23429806</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>312</v>
+      </c>
+      <c r="B29">
+        <v>2048</v>
+      </c>
+      <c r="C29">
+        <v>4.1629220000000003E-3</v>
+      </c>
+      <c r="D29">
+        <v>4.1629220000000003E-3</v>
+      </c>
+      <c r="E29">
+        <v>4.1629220000000003E-3</v>
+      </c>
+      <c r="F29">
+        <v>0.23831492700000001</v>
+      </c>
+      <c r="G29">
+        <v>0.23831492700000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>312</v>
+      </c>
+      <c r="B30">
+        <v>2049</v>
+      </c>
+      <c r="C30">
+        <v>4.3251549999999998E-3</v>
+      </c>
+      <c r="D30">
+        <v>4.3251549999999998E-3</v>
+      </c>
+      <c r="E30">
+        <v>4.3251549999999998E-3</v>
+      </c>
+      <c r="F30">
+        <v>0.241681439</v>
+      </c>
+      <c r="G30">
+        <v>0.241681439</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>312</v>
+      </c>
+      <c r="B31">
+        <v>2050</v>
+      </c>
+      <c r="C31">
+        <v>4.495321E-3</v>
+      </c>
+      <c r="D31">
+        <v>4.495321E-3</v>
+      </c>
+      <c r="E31">
+        <v>4.495321E-3</v>
+      </c>
+      <c r="F31">
+        <v>0.24449030199999999</v>
+      </c>
+      <c r="G31">
+        <v>0.24449030199999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>313</v>
+      </c>
+      <c r="B32">
+        <v>2021</v>
+      </c>
+      <c r="C32">
+        <v>2.7681490000000001E-3</v>
+      </c>
+      <c r="D32">
+        <v>2.7681490000000001E-3</v>
+      </c>
+      <c r="E32">
+        <v>2.7681490000000001E-3</v>
+      </c>
+      <c r="F32">
+        <v>2.7681490000000001E-3</v>
+      </c>
+      <c r="G32">
+        <v>2.7681490000000001E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>313</v>
+      </c>
+      <c r="B33">
+        <v>2022</v>
+      </c>
+      <c r="C33">
+        <v>5.506319E-3</v>
+      </c>
+      <c r="D33">
+        <v>8.2696799999999997E-3</v>
+      </c>
+      <c r="E33">
+        <v>6.8879989999999997E-3</v>
+      </c>
+      <c r="F33">
+        <v>6.8879989999999997E-3</v>
+      </c>
+      <c r="G33">
+        <v>8.2696799999999997E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>313</v>
+      </c>
+      <c r="B34">
+        <v>2023</v>
+      </c>
+      <c r="C34">
+        <v>8.604024E-3</v>
+      </c>
+      <c r="D34">
+        <v>1.3771211E-2</v>
+      </c>
+      <c r="E34">
+        <v>1.1187618E-2</v>
+      </c>
+      <c r="F34">
+        <v>1.1187618E-2</v>
+      </c>
+      <c r="G34">
+        <v>1.3771211E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>313</v>
+      </c>
+      <c r="B35">
+        <v>2024</v>
+      </c>
+      <c r="C35">
+        <v>1.1780479999999999E-2</v>
+      </c>
+      <c r="D35">
+        <v>1.9272741999999999E-2</v>
+      </c>
+      <c r="E35">
+        <v>1.5526610999999999E-2</v>
+      </c>
+      <c r="F35">
+        <v>1.5526610999999999E-2</v>
+      </c>
+      <c r="G35">
+        <v>1.9272741999999999E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>313</v>
+      </c>
+      <c r="B36">
+        <v>2025</v>
+      </c>
+      <c r="C36">
+        <v>1.4880427E-2</v>
+      </c>
+      <c r="D36">
+        <v>2.4774272999999999E-2</v>
+      </c>
+      <c r="E36">
+        <v>1.9827350000000001E-2</v>
+      </c>
+      <c r="F36">
+        <v>1.9827350000000001E-2</v>
+      </c>
+      <c r="G36">
+        <v>2.4774272999999999E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>313</v>
+      </c>
+      <c r="B37">
+        <v>2026</v>
+      </c>
+      <c r="C37">
+        <v>1.7896786000000001E-2</v>
+      </c>
+      <c r="D37">
+        <v>3.7774355000000003E-2</v>
+      </c>
+      <c r="E37">
+        <v>2.783557E-2</v>
+      </c>
+      <c r="F37">
+        <v>2.783557E-2</v>
+      </c>
+      <c r="G37">
+        <v>3.7774355000000003E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>313</v>
+      </c>
+      <c r="B38">
+        <v>2027</v>
+      </c>
+      <c r="C38">
+        <v>2.0805857000000001E-2</v>
+      </c>
+      <c r="D38">
+        <v>5.7356055000000003E-2</v>
+      </c>
+      <c r="E38">
+        <v>3.9080956E-2</v>
+      </c>
+      <c r="F38">
+        <v>3.9080956E-2</v>
+      </c>
+      <c r="G38">
+        <v>5.7356055000000003E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>313</v>
+      </c>
+      <c r="B39">
+        <v>2028</v>
+      </c>
+      <c r="C39">
+        <v>2.3611013E-2</v>
+      </c>
+      <c r="D39">
+        <v>8.4760910999999994E-2</v>
+      </c>
+      <c r="E39">
+        <v>5.4185961999999997E-2</v>
+      </c>
+      <c r="F39">
+        <v>5.4185961999999997E-2</v>
+      </c>
+      <c r="G39">
+        <v>8.4760910999999994E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>313</v>
+      </c>
+      <c r="B40">
+        <v>2029</v>
+      </c>
+      <c r="C40">
+        <v>2.6362935000000001E-2</v>
+      </c>
+      <c r="D40">
+        <v>0.110267067</v>
+      </c>
+      <c r="E40">
+        <v>6.8315001E-2</v>
+      </c>
+      <c r="F40">
+        <v>6.8315001E-2</v>
+      </c>
+      <c r="G40">
+        <v>0.110267067</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>313</v>
+      </c>
+      <c r="B41">
+        <v>2030</v>
+      </c>
+      <c r="C41">
+        <v>2.9098506E-2</v>
+      </c>
+      <c r="D41">
+        <v>0.13976050100000001</v>
+      </c>
+      <c r="E41">
+        <v>8.4429504000000002E-2</v>
+      </c>
+      <c r="F41">
+        <v>8.4429504000000002E-2</v>
+      </c>
+      <c r="G41">
+        <v>0.13976050100000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>313</v>
+      </c>
+      <c r="B42">
+        <v>2031</v>
+      </c>
+      <c r="C42">
+        <v>3.1850912000000002E-2</v>
+      </c>
+      <c r="D42">
+        <v>0.16977555799999999</v>
+      </c>
+      <c r="E42">
+        <v>0.100813235</v>
+      </c>
+      <c r="F42">
+        <v>0.100813235</v>
+      </c>
+      <c r="G42">
+        <v>0.16977555799999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>313</v>
+      </c>
+      <c r="B43">
+        <v>2032</v>
+      </c>
+      <c r="C43">
+        <v>3.4619206E-2</v>
+      </c>
+      <c r="D43">
+        <v>0.20474008699999999</v>
+      </c>
+      <c r="E43">
+        <v>0.119679647</v>
+      </c>
+      <c r="F43">
+        <v>0.119679647</v>
+      </c>
+      <c r="G43">
+        <v>0.20474008699999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>313</v>
+      </c>
+      <c r="B44">
+        <v>2033</v>
+      </c>
+      <c r="C44">
+        <v>3.7401094000000003E-2</v>
+      </c>
+      <c r="D44">
+        <v>0.24537620900000001</v>
+      </c>
+      <c r="E44">
+        <v>0.141388651</v>
+      </c>
+      <c r="F44">
+        <v>0.141388651</v>
+      </c>
+      <c r="G44">
+        <v>0.24537620900000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>313</v>
+      </c>
+      <c r="B45">
+        <v>2034</v>
+      </c>
+      <c r="C45">
+        <v>4.0196467999999999E-2</v>
+      </c>
+      <c r="D45">
+        <v>0.292219018</v>
+      </c>
+      <c r="E45">
+        <v>0.16620774299999999</v>
+      </c>
+      <c r="F45">
+        <v>0.16620774299999999</v>
+      </c>
+      <c r="G45">
+        <v>0.292219018</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>313</v>
+      </c>
+      <c r="B46">
+        <v>2035</v>
+      </c>
+      <c r="C46">
+        <v>4.2987719000000001E-2</v>
+      </c>
+      <c r="D46">
+        <v>0.34549044600000001</v>
+      </c>
+      <c r="E46">
+        <v>0.19423908200000001</v>
+      </c>
+      <c r="F46">
+        <v>0.19423908200000001</v>
+      </c>
+      <c r="G46">
+        <v>0.34549044600000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>313</v>
+      </c>
+      <c r="B47">
+        <v>2036</v>
+      </c>
+      <c r="C47">
+        <v>4.5770973E-2</v>
+      </c>
+      <c r="D47">
+        <v>0.39619227099999998</v>
+      </c>
+      <c r="E47">
+        <v>0.22098162199999999</v>
+      </c>
+      <c r="F47">
+        <v>0.22098162199999999</v>
+      </c>
+      <c r="G47">
+        <v>0.39619227099999998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>313</v>
+      </c>
+      <c r="B48">
+        <v>2037</v>
+      </c>
+      <c r="C48">
+        <v>4.8543924000000002E-2</v>
+      </c>
+      <c r="D48">
+        <v>0.444968113</v>
+      </c>
+      <c r="E48">
+        <v>0.24675601899999999</v>
+      </c>
+      <c r="F48">
+        <v>0.24675601899999999</v>
+      </c>
+      <c r="G48">
+        <v>0.444968113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>313</v>
+      </c>
+      <c r="B49">
+        <v>2038</v>
+      </c>
+      <c r="C49">
+        <v>5.1304790000000003E-2</v>
+      </c>
+      <c r="D49">
+        <v>0.49169161900000002</v>
+      </c>
+      <c r="E49">
+        <v>0.27149820400000002</v>
+      </c>
+      <c r="F49">
+        <v>0.27149820400000002</v>
+      </c>
+      <c r="G49">
+        <v>0.49169161900000002</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>313</v>
+      </c>
+      <c r="B50">
+        <v>2039</v>
+      </c>
+      <c r="C50">
+        <v>5.40186E-2</v>
+      </c>
+      <c r="D50">
+        <v>0.53644918200000002</v>
+      </c>
+      <c r="E50">
+        <v>0.29523389100000003</v>
+      </c>
+      <c r="F50">
+        <v>0.29523389100000003</v>
+      </c>
+      <c r="G50">
+        <v>0.53644918200000002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>313</v>
+      </c>
+      <c r="B51">
+        <v>2040</v>
+      </c>
+      <c r="C51">
+        <v>5.6696666E-2</v>
+      </c>
+      <c r="D51">
+        <v>0.57897244699999995</v>
+      </c>
+      <c r="E51">
+        <v>0.31783455599999999</v>
+      </c>
+      <c r="F51">
+        <v>0.31783455599999999</v>
+      </c>
+      <c r="G51">
+        <v>0.57897244699999995</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>313</v>
+      </c>
+      <c r="B52">
+        <v>2041</v>
+      </c>
+      <c r="C52">
+        <v>5.9316059999999997E-2</v>
+      </c>
+      <c r="D52">
+        <v>0.61912640799999996</v>
+      </c>
+      <c r="E52">
+        <v>0.33922123399999998</v>
+      </c>
+      <c r="F52">
+        <v>0.33922123399999998</v>
+      </c>
+      <c r="G52">
+        <v>0.61912640799999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>313</v>
+      </c>
+      <c r="B53">
+        <v>2042</v>
+      </c>
+      <c r="C53">
+        <v>6.1865734999999998E-2</v>
+      </c>
+      <c r="D53">
+        <v>0.657095557</v>
+      </c>
+      <c r="E53">
+        <v>0.35948064600000001</v>
+      </c>
+      <c r="F53">
+        <v>0.35948064600000001</v>
+      </c>
+      <c r="G53">
+        <v>0.657095557</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>313</v>
+      </c>
+      <c r="B54">
+        <v>2043</v>
+      </c>
+      <c r="C54">
+        <v>6.4368699000000001E-2</v>
+      </c>
+      <c r="D54">
+        <v>0.69262306100000004</v>
+      </c>
+      <c r="E54">
+        <v>0.37849588000000001</v>
+      </c>
+      <c r="F54">
+        <v>0.37849588000000001</v>
+      </c>
+      <c r="G54">
+        <v>0.69262306100000004</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>313</v>
+      </c>
+      <c r="B55">
+        <v>2044</v>
+      </c>
+      <c r="C55">
+        <v>6.6828560999999995E-2</v>
+      </c>
+      <c r="D55">
+        <v>0.72576428699999995</v>
+      </c>
+      <c r="E55">
+        <v>0.39629642399999998</v>
+      </c>
+      <c r="F55">
+        <v>0.39629642399999998</v>
+      </c>
+      <c r="G55">
+        <v>0.72576428699999995</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>313</v>
+      </c>
+      <c r="B56">
+        <v>2045</v>
+      </c>
+      <c r="C56">
+        <v>6.9255160999999996E-2</v>
+      </c>
+      <c r="D56">
+        <v>0.75643987199999996</v>
+      </c>
+      <c r="E56">
+        <v>0.41284751600000003</v>
+      </c>
+      <c r="F56">
+        <v>0.41284751600000003</v>
+      </c>
+      <c r="G56">
+        <v>0.75643987199999996</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>313</v>
+      </c>
+      <c r="B57">
+        <v>2046</v>
+      </c>
+      <c r="C57">
+        <v>7.1660583E-2</v>
+      </c>
+      <c r="D57">
+        <v>0.78459593599999999</v>
+      </c>
+      <c r="E57">
+        <v>0.42812825900000001</v>
+      </c>
+      <c r="F57">
+        <v>0.42812825900000001</v>
+      </c>
+      <c r="G57">
+        <v>0.78459593599999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>313</v>
+      </c>
+      <c r="B58">
+        <v>2047</v>
+      </c>
+      <c r="C58">
+        <v>7.4023167000000001E-2</v>
+      </c>
+      <c r="D58">
+        <v>0.81016510900000005</v>
+      </c>
+      <c r="E58">
+        <v>0.44209413800000003</v>
+      </c>
+      <c r="F58">
+        <v>0.44209413800000003</v>
+      </c>
+      <c r="G58">
+        <v>0.81016510900000005</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>313</v>
+      </c>
+      <c r="B59">
+        <v>2048</v>
+      </c>
+      <c r="C59">
+        <v>7.6331019E-2</v>
+      </c>
+      <c r="D59">
+        <v>0.83324370199999997</v>
+      </c>
+      <c r="E59">
+        <v>0.454787361</v>
+      </c>
+      <c r="F59">
+        <v>0.454787361</v>
+      </c>
+      <c r="G59">
+        <v>0.83324370199999997</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>313</v>
+      </c>
+      <c r="B60">
+        <v>2049</v>
+      </c>
+      <c r="C60">
+        <v>7.8599206000000005E-2</v>
+      </c>
+      <c r="D60">
+        <v>0.85401336000000005</v>
+      </c>
+      <c r="E60">
+        <v>0.46630628299999999</v>
+      </c>
+      <c r="F60">
+        <v>0.46630628299999999</v>
+      </c>
+      <c r="G60">
+        <v>0.85401336000000005</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>313</v>
+      </c>
+      <c r="B61">
+        <v>2050</v>
+      </c>
+      <c r="C61">
+        <v>8.0826548999999998E-2</v>
+      </c>
+      <c r="D61">
+        <v>0.87233277799999998</v>
+      </c>
+      <c r="E61">
+        <v>0.47657966400000001</v>
+      </c>
+      <c r="F61">
+        <v>0.47657966400000001</v>
+      </c>
+      <c r="G61">
+        <v>0.87233277799999998</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>314</v>
+      </c>
+      <c r="B62">
+        <v>2021</v>
+      </c>
+      <c r="C62">
+        <v>2.69208E-4</v>
+      </c>
+      <c r="D62">
+        <v>2.69208E-4</v>
+      </c>
+      <c r="E62">
+        <v>2.69208E-4</v>
+      </c>
+      <c r="F62">
+        <v>2.69208E-4</v>
+      </c>
+      <c r="G62">
+        <v>2.69208E-4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>314</v>
+      </c>
+      <c r="B63">
+        <v>2022</v>
+      </c>
+      <c r="C63">
+        <v>5.1113500000000002E-4</v>
+      </c>
+      <c r="D63">
+        <v>5.1113500000000002E-4</v>
+      </c>
+      <c r="E63">
+        <v>5.1113500000000002E-4</v>
+      </c>
+      <c r="F63">
+        <v>5.1113500000000002E-4</v>
+      </c>
+      <c r="G63">
+        <v>5.1113500000000002E-4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>314</v>
+      </c>
+      <c r="B64">
+        <v>2023</v>
+      </c>
+      <c r="C64">
+        <v>7.5173000000000004E-4</v>
+      </c>
+      <c r="D64">
+        <v>7.5173000000000004E-4</v>
+      </c>
+      <c r="E64">
+        <v>7.5173000000000004E-4</v>
+      </c>
+      <c r="F64">
+        <v>7.5173000000000004E-4</v>
+      </c>
+      <c r="G64">
+        <v>7.5173000000000004E-4</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>314</v>
+      </c>
+      <c r="B65">
+        <v>2024</v>
+      </c>
+      <c r="C65">
+        <v>9.8721599999999996E-4</v>
+      </c>
+      <c r="D65">
+        <v>9.8721599999999996E-4</v>
+      </c>
+      <c r="E65">
+        <v>9.8721599999999996E-4</v>
+      </c>
+      <c r="F65">
+        <v>2.2232290000000002E-3</v>
+      </c>
+      <c r="G65">
+        <v>2.2232290000000002E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>314</v>
+      </c>
+      <c r="B66">
+        <v>2025</v>
+      </c>
+      <c r="C66">
+        <v>1.2173970000000001E-3</v>
+      </c>
+      <c r="D66">
+        <v>1.2173970000000001E-3</v>
+      </c>
+      <c r="E66">
+        <v>1.2173970000000001E-3</v>
+      </c>
+      <c r="F66">
+        <v>6.3453590000000001E-3</v>
+      </c>
+      <c r="G66">
+        <v>6.3453590000000001E-3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>314</v>
+      </c>
+      <c r="B67">
+        <v>2026</v>
+      </c>
+      <c r="C67">
+        <v>1.4441510000000001E-3</v>
+      </c>
+      <c r="D67">
+        <v>1.4441510000000001E-3</v>
+      </c>
+      <c r="E67">
+        <v>1.4441510000000001E-3</v>
+      </c>
+      <c r="F67">
+        <v>1.1845461999999999E-2</v>
+      </c>
+      <c r="G67">
+        <v>1.1845461999999999E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>314</v>
+      </c>
+      <c r="B68">
+        <v>2027</v>
+      </c>
+      <c r="C68">
+        <v>1.664706E-3</v>
+      </c>
+      <c r="D68">
+        <v>1.664706E-3</v>
+      </c>
+      <c r="E68">
+        <v>1.664706E-3</v>
+      </c>
+      <c r="F68">
+        <v>1.9948430999999999E-2</v>
+      </c>
+      <c r="G68">
+        <v>1.9948430999999999E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>314</v>
+      </c>
+      <c r="B69">
+        <v>2028</v>
+      </c>
+      <c r="C69">
+        <v>1.879225E-3</v>
+      </c>
+      <c r="D69">
+        <v>1.879225E-3</v>
+      </c>
+      <c r="E69">
+        <v>1.879225E-3</v>
+      </c>
+      <c r="F69">
+        <v>3.1568299000000001E-2</v>
+      </c>
+      <c r="G69">
+        <v>3.1568299000000001E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>314</v>
+      </c>
+      <c r="B70">
+        <v>2029</v>
+      </c>
+      <c r="C70">
+        <v>2.0915529999999999E-3</v>
+      </c>
+      <c r="D70">
+        <v>2.0915529999999999E-3</v>
+      </c>
+      <c r="E70">
+        <v>2.0915529999999999E-3</v>
+      </c>
+      <c r="F70">
+        <v>4.6924004999999998E-2</v>
+      </c>
+      <c r="G70">
+        <v>4.6924004999999998E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>314</v>
+      </c>
+      <c r="B71">
+        <v>2030</v>
+      </c>
+      <c r="C71">
+        <v>2.3018520000000001E-3</v>
+      </c>
+      <c r="D71">
+        <v>2.3018520000000001E-3</v>
+      </c>
+      <c r="E71">
+        <v>2.3018520000000001E-3</v>
+      </c>
+      <c r="F71">
+        <v>6.5785700000000003E-2</v>
+      </c>
+      <c r="G71">
+        <v>6.5785700000000003E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>314</v>
+      </c>
+      <c r="B72">
+        <v>2031</v>
+      </c>
+      <c r="C72">
+        <v>2.5109339999999998E-3</v>
+      </c>
+      <c r="D72">
+        <v>2.5109339999999998E-3</v>
+      </c>
+      <c r="E72">
+        <v>2.5109339999999998E-3</v>
+      </c>
+      <c r="F72">
+        <v>8.8363822999999994E-2</v>
+      </c>
+      <c r="G72">
+        <v>8.8363822999999994E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>314</v>
+      </c>
+      <c r="B73">
+        <v>2032</v>
+      </c>
+      <c r="C73">
+        <v>2.7175649999999999E-3</v>
+      </c>
+      <c r="D73">
+        <v>2.7175649999999999E-3</v>
+      </c>
+      <c r="E73">
+        <v>2.7175649999999999E-3</v>
+      </c>
+      <c r="F73">
+        <v>0.112572854</v>
+      </c>
+      <c r="G73">
+        <v>0.112572854</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>314</v>
+      </c>
+      <c r="B74">
+        <v>2033</v>
+      </c>
+      <c r="C74">
+        <v>2.927851E-3</v>
+      </c>
+      <c r="D74">
+        <v>2.927851E-3</v>
+      </c>
+      <c r="E74">
+        <v>2.927851E-3</v>
+      </c>
+      <c r="F74">
+        <v>0.13861931199999999</v>
+      </c>
+      <c r="G74">
+        <v>0.13861931199999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>314</v>
+      </c>
+      <c r="B75">
+        <v>2034</v>
+      </c>
+      <c r="C75">
+        <v>3.1403939999999999E-3</v>
+      </c>
+      <c r="D75">
+        <v>3.1403939999999999E-3</v>
+      </c>
+      <c r="E75">
+        <v>3.1403939999999999E-3</v>
+      </c>
+      <c r="F75">
+        <v>0.16646481900000001</v>
+      </c>
+      <c r="G75">
+        <v>0.16646481900000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>314</v>
+      </c>
+      <c r="B76">
+        <v>2035</v>
+      </c>
+      <c r="C76">
+        <v>3.3537770000000001E-3</v>
+      </c>
+      <c r="D76">
+        <v>3.3537770000000001E-3</v>
+      </c>
+      <c r="E76">
+        <v>3.3537770000000001E-3</v>
+      </c>
+      <c r="F76">
+        <v>0.19560739399999999</v>
+      </c>
+      <c r="G76">
+        <v>0.19560739399999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>314</v>
+      </c>
+      <c r="B77">
+        <v>2036</v>
+      </c>
+      <c r="C77">
+        <v>3.5669400000000002E-3</v>
+      </c>
+      <c r="D77">
+        <v>3.5669400000000002E-3</v>
+      </c>
+      <c r="E77">
+        <v>3.5669400000000002E-3</v>
+      </c>
+      <c r="F77">
+        <v>0.224213724</v>
+      </c>
+      <c r="G77">
+        <v>0.224213724</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>314</v>
+      </c>
+      <c r="B78">
+        <v>2037</v>
+      </c>
+      <c r="C78">
+        <v>3.7814290000000002E-3</v>
+      </c>
+      <c r="D78">
+        <v>3.7814290000000002E-3</v>
+      </c>
+      <c r="E78">
+        <v>3.7814290000000002E-3</v>
+      </c>
+      <c r="F78">
+        <v>0.251758013</v>
+      </c>
+      <c r="G78">
+        <v>0.251758013</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>314</v>
+      </c>
+      <c r="B79">
+        <v>2038</v>
+      </c>
+      <c r="C79">
+        <v>3.9981180000000002E-3</v>
+      </c>
+      <c r="D79">
+        <v>3.9981180000000002E-3</v>
+      </c>
+      <c r="E79">
+        <v>3.9981180000000002E-3</v>
+      </c>
+      <c r="F79">
+        <v>0.27830375000000002</v>
+      </c>
+      <c r="G79">
+        <v>0.27830375000000002</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>314</v>
+      </c>
+      <c r="B80">
+        <v>2039</v>
+      </c>
+      <c r="C80">
+        <v>4.2198260000000003E-3</v>
+      </c>
+      <c r="D80">
+        <v>4.2198260000000003E-3</v>
+      </c>
+      <c r="E80">
+        <v>4.2198260000000003E-3</v>
+      </c>
+      <c r="F80">
+        <v>0.30357849199999998</v>
+      </c>
+      <c r="G80">
+        <v>0.30357849199999998</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>314</v>
+      </c>
+      <c r="B81">
+        <v>2040</v>
+      </c>
+      <c r="C81">
+        <v>4.448624E-3</v>
+      </c>
+      <c r="D81">
+        <v>4.448624E-3</v>
+      </c>
+      <c r="E81">
+        <v>4.448624E-3</v>
+      </c>
+      <c r="F81">
+        <v>0.32763684900000001</v>
+      </c>
+      <c r="G81">
+        <v>0.32763684900000001</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>314</v>
+      </c>
+      <c r="B82">
+        <v>2041</v>
+      </c>
+      <c r="C82">
+        <v>4.678415E-3</v>
+      </c>
+      <c r="D82">
+        <v>4.678415E-3</v>
+      </c>
+      <c r="E82">
+        <v>4.678415E-3</v>
+      </c>
+      <c r="F82">
+        <v>0.35042086</v>
+      </c>
+      <c r="G82">
+        <v>0.35042086</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>314</v>
+      </c>
+      <c r="B83">
+        <v>2042</v>
+      </c>
+      <c r="C83">
+        <v>4.910925E-3</v>
+      </c>
+      <c r="D83">
+        <v>4.910925E-3</v>
+      </c>
+      <c r="E83">
+        <v>4.910925E-3</v>
+      </c>
+      <c r="F83">
+        <v>0.371888357</v>
+      </c>
+      <c r="G83">
+        <v>0.371888357</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>314</v>
+      </c>
+      <c r="B84">
+        <v>2043</v>
+      </c>
+      <c r="C84">
+        <v>5.1371760000000002E-3</v>
+      </c>
+      <c r="D84">
+        <v>5.1371760000000002E-3</v>
+      </c>
+      <c r="E84">
+        <v>5.1371760000000002E-3</v>
+      </c>
+      <c r="F84">
+        <v>0.39163393099999999</v>
+      </c>
+      <c r="G84">
+        <v>0.39163393099999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>314</v>
+      </c>
+      <c r="B85">
+        <v>2044</v>
+      </c>
+      <c r="C85">
+        <v>5.3573889999999997E-3</v>
+      </c>
+      <c r="D85">
+        <v>5.3573889999999997E-3</v>
+      </c>
+      <c r="E85">
+        <v>5.3573889999999997E-3</v>
+      </c>
+      <c r="F85">
+        <v>0.41053531700000001</v>
+      </c>
+      <c r="G85">
+        <v>0.41053531700000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>314</v>
+      </c>
+      <c r="B86">
+        <v>2045</v>
+      </c>
+      <c r="C86">
+        <v>5.5812450000000003E-3</v>
+      </c>
+      <c r="D86">
+        <v>5.5812450000000003E-3</v>
+      </c>
+      <c r="E86">
+        <v>5.5812450000000003E-3</v>
+      </c>
+      <c r="F86">
+        <v>0.427685765</v>
+      </c>
+      <c r="G86">
+        <v>0.427685765</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>314</v>
+      </c>
+      <c r="B87">
+        <v>2046</v>
+      </c>
+      <c r="C87">
+        <v>5.811709E-3</v>
+      </c>
+      <c r="D87">
+        <v>5.811709E-3</v>
+      </c>
+      <c r="E87">
+        <v>5.811709E-3</v>
+      </c>
+      <c r="F87">
+        <v>0.443591191</v>
+      </c>
+      <c r="G87">
+        <v>0.443591191</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>314</v>
+      </c>
+      <c r="B88">
+        <v>2047</v>
+      </c>
+      <c r="C88">
+        <v>6.0421320000000004E-3</v>
+      </c>
+      <c r="D88">
+        <v>6.0421320000000004E-3</v>
+      </c>
+      <c r="E88">
+        <v>6.0421320000000004E-3</v>
+      </c>
+      <c r="F88">
+        <v>0.45792830099999998</v>
+      </c>
+      <c r="G88">
+        <v>0.45792830099999998</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>314</v>
+      </c>
+      <c r="B89">
+        <v>2048</v>
+      </c>
+      <c r="C89">
+        <v>6.2732539999999998E-3</v>
+      </c>
+      <c r="D89">
+        <v>6.2732539999999998E-3</v>
+      </c>
+      <c r="E89">
+        <v>6.2732539999999998E-3</v>
+      </c>
+      <c r="F89">
+        <v>0.47101606299999998</v>
+      </c>
+      <c r="G89">
+        <v>0.47101606299999998</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>314</v>
+      </c>
+      <c r="B90">
+        <v>2049</v>
+      </c>
+      <c r="C90">
+        <v>6.5150909999999998E-3</v>
+      </c>
+      <c r="D90">
+        <v>6.5150909999999998E-3</v>
+      </c>
+      <c r="E90">
+        <v>6.5150909999999998E-3</v>
+      </c>
+      <c r="F90">
+        <v>0.48289326799999999</v>
+      </c>
+      <c r="G90">
+        <v>0.48289326799999999</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>314</v>
+      </c>
+      <c r="B91">
+        <v>2050</v>
+      </c>
+      <c r="C91">
+        <v>6.767019E-3</v>
+      </c>
+      <c r="D91">
+        <v>6.767019E-3</v>
+      </c>
+      <c r="E91">
+        <v>6.767019E-3</v>
+      </c>
+      <c r="F91">
+        <v>0.49398055200000002</v>
+      </c>
+      <c r="G91">
+        <v>0.49398055200000002</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>315</v>
+      </c>
+      <c r="B92">
+        <v>2021</v>
+      </c>
+      <c r="C92">
+        <v>1.2819571E-2</v>
+      </c>
+      <c r="D92">
+        <v>1.2819571E-2</v>
+      </c>
+      <c r="E92">
+        <v>1.2819571E-2</v>
+      </c>
+      <c r="F92">
+        <v>1.2819571E-2</v>
+      </c>
+      <c r="G92">
+        <v>1.2819571E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>315</v>
+      </c>
+      <c r="B93">
+        <v>2022</v>
+      </c>
+      <c r="C93">
+        <v>1.4978317E-2</v>
+      </c>
+      <c r="D93">
+        <v>3.2432076999999997E-2</v>
+      </c>
+      <c r="E93">
+        <v>2.3705197000000001E-2</v>
+      </c>
+      <c r="F93">
+        <v>2.3705197000000001E-2</v>
+      </c>
+      <c r="G93">
+        <v>3.2432076999999997E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>315</v>
+      </c>
+      <c r="B94">
+        <v>2023</v>
+      </c>
+      <c r="C94">
+        <v>1.7291666000000001E-2</v>
+      </c>
+      <c r="D94">
+        <v>5.2044582999999998E-2</v>
+      </c>
+      <c r="E94">
+        <v>3.4668124000000002E-2</v>
+      </c>
+      <c r="F94">
+        <v>3.4668124000000002E-2</v>
+      </c>
+      <c r="G94">
+        <v>5.2044582999999998E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>315</v>
+      </c>
+      <c r="B95">
+        <v>2024</v>
+      </c>
+      <c r="C95">
+        <v>1.9724051999999999E-2</v>
+      </c>
+      <c r="D95">
+        <v>7.1657088999999993E-2</v>
+      </c>
+      <c r="E95">
+        <v>4.5690570999999999E-2</v>
+      </c>
+      <c r="F95">
+        <v>4.5690570999999999E-2</v>
+      </c>
+      <c r="G95">
+        <v>7.1657088999999993E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>315</v>
+      </c>
+      <c r="B96">
+        <v>2025</v>
+      </c>
+      <c r="C96">
+        <v>2.2165526000000001E-2</v>
+      </c>
+      <c r="D96">
+        <v>9.1269594999999995E-2</v>
+      </c>
+      <c r="E96">
+        <v>5.671756E-2</v>
+      </c>
+      <c r="F96">
+        <v>5.671756E-2</v>
+      </c>
+      <c r="G96">
+        <v>9.1269594999999995E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>315</v>
+      </c>
+      <c r="B97">
+        <v>2026</v>
+      </c>
+      <c r="C97">
+        <v>2.4657855999999999E-2</v>
+      </c>
+      <c r="D97">
+        <v>0.12079788800000001</v>
+      </c>
+      <c r="E97">
+        <v>7.2727871999999999E-2</v>
+      </c>
+      <c r="F97">
+        <v>7.2727871999999999E-2</v>
+      </c>
+      <c r="G97">
+        <v>0.12079788800000001</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>315</v>
+      </c>
+      <c r="B98">
+        <v>2027</v>
+      </c>
+      <c r="C98">
+        <v>2.7184686999999999E-2</v>
+      </c>
+      <c r="D98">
+        <v>0.151904497</v>
+      </c>
+      <c r="E98">
+        <v>8.9544592000000006E-2</v>
+      </c>
+      <c r="F98">
+        <v>8.9544592000000006E-2</v>
+      </c>
+      <c r="G98">
+        <v>0.151904497</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>315</v>
+      </c>
+      <c r="B99">
+        <v>2028</v>
+      </c>
+      <c r="C99">
+        <v>2.9742540000000001E-2</v>
+      </c>
+      <c r="D99">
+        <v>0.18432768499999999</v>
+      </c>
+      <c r="E99">
+        <v>0.107035112</v>
+      </c>
+      <c r="F99">
+        <v>0.107035112</v>
+      </c>
+      <c r="G99">
+        <v>0.18432768499999999</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>315</v>
+      </c>
+      <c r="B100">
+        <v>2029</v>
+      </c>
+      <c r="C100">
+        <v>3.2380491999999997E-2</v>
+      </c>
+      <c r="D100">
+        <v>0.22622346600000001</v>
+      </c>
+      <c r="E100">
+        <v>0.12930197900000001</v>
+      </c>
+      <c r="F100">
+        <v>0.12930197900000001</v>
+      </c>
+      <c r="G100">
+        <v>0.22622346600000001</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>315</v>
+      </c>
+      <c r="B101">
+        <v>2030</v>
+      </c>
+      <c r="C101">
+        <v>3.5179580000000002E-2</v>
+      </c>
+      <c r="D101">
+        <v>0.27353129100000001</v>
+      </c>
+      <c r="E101">
+        <v>0.15435543600000001</v>
+      </c>
+      <c r="F101">
+        <v>0.15435543600000001</v>
+      </c>
+      <c r="G101">
+        <v>0.27353129100000001</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>315</v>
+      </c>
+      <c r="B102">
+        <v>2031</v>
+      </c>
+      <c r="C102">
+        <v>3.8168565000000002E-2</v>
+      </c>
+      <c r="D102">
+        <v>0.32771400000000001</v>
+      </c>
+      <c r="E102">
+        <v>0.18294128300000001</v>
+      </c>
+      <c r="F102">
+        <v>0.18294128300000001</v>
+      </c>
+      <c r="G102">
+        <v>0.32771400000000001</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>315</v>
+      </c>
+      <c r="B103">
+        <v>2032</v>
+      </c>
+      <c r="C103">
+        <v>4.1333373999999999E-2</v>
+      </c>
+      <c r="D103">
+        <v>0.38171043300000002</v>
+      </c>
+      <c r="E103">
+        <v>0.21152190400000001</v>
+      </c>
+      <c r="F103">
+        <v>0.21152190400000001</v>
+      </c>
+      <c r="G103">
+        <v>0.38171043300000002</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>315</v>
+      </c>
+      <c r="B104">
+        <v>2033</v>
+      </c>
+      <c r="C104">
+        <v>4.4657994999999999E-2</v>
+      </c>
+      <c r="D104">
+        <v>0.43484204300000001</v>
+      </c>
+      <c r="E104">
+        <v>0.23975001900000001</v>
+      </c>
+      <c r="F104">
+        <v>0.23975001900000001</v>
+      </c>
+      <c r="G104">
+        <v>0.43484204300000001</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>315</v>
+      </c>
+      <c r="B105">
+        <v>2034</v>
+      </c>
+      <c r="C105">
+        <v>4.8126879999999997E-2</v>
+      </c>
+      <c r="D105">
+        <v>0.48654755500000002</v>
+      </c>
+      <c r="E105">
+        <v>0.26733721799999999</v>
+      </c>
+      <c r="F105">
+        <v>0.26733721799999999</v>
+      </c>
+      <c r="G105">
+        <v>0.48654755500000002</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>315</v>
+      </c>
+      <c r="B106">
+        <v>2035</v>
+      </c>
+      <c r="C106">
+        <v>5.1706859000000001E-2</v>
+      </c>
+      <c r="D106">
+        <v>0.53597180700000002</v>
+      </c>
+      <c r="E106">
+        <v>0.29383933299999998</v>
+      </c>
+      <c r="F106">
+        <v>0.29383933299999998</v>
+      </c>
+      <c r="G106">
+        <v>0.53597180700000002</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>315</v>
+      </c>
+      <c r="B107">
+        <v>2036</v>
+      </c>
+      <c r="C107">
+        <v>5.5368675999999999E-2</v>
+      </c>
+      <c r="D107">
+        <v>0.58298080299999999</v>
+      </c>
+      <c r="E107">
+        <v>0.31917473899999999</v>
+      </c>
+      <c r="F107">
+        <v>0.31917473899999999</v>
+      </c>
+      <c r="G107">
+        <v>0.58298080299999999</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>315</v>
+      </c>
+      <c r="B108">
+        <v>2037</v>
+      </c>
+      <c r="C108">
+        <v>5.9080055999999999E-2</v>
+      </c>
+      <c r="D108">
+        <v>0.62722744100000005</v>
+      </c>
+      <c r="E108">
+        <v>0.34315374799999998</v>
+      </c>
+      <c r="F108">
+        <v>0.34315374799999998</v>
+      </c>
+      <c r="G108">
+        <v>0.62722744100000005</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>315</v>
+      </c>
+      <c r="B109">
+        <v>2038</v>
+      </c>
+      <c r="C109">
+        <v>6.2828703E-2</v>
+      </c>
+      <c r="D109">
+        <v>0.66866269899999997</v>
+      </c>
+      <c r="E109">
+        <v>0.36574570099999998</v>
+      </c>
+      <c r="F109">
+        <v>0.36574570099999998</v>
+      </c>
+      <c r="G109">
+        <v>0.66866269899999997</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>315</v>
+      </c>
+      <c r="B110">
+        <v>2039</v>
+      </c>
+      <c r="C110">
+        <v>6.6573137000000004E-2</v>
+      </c>
+      <c r="D110">
+        <v>0.70719917499999996</v>
+      </c>
+      <c r="E110">
+        <v>0.38688615599999998</v>
+      </c>
+      <c r="F110">
+        <v>0.38688615599999998</v>
+      </c>
+      <c r="G110">
+        <v>0.70719917499999996</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>315</v>
+      </c>
+      <c r="B111">
+        <v>2040</v>
+      </c>
+      <c r="C111">
+        <v>7.0318973000000007E-2</v>
+      </c>
+      <c r="D111">
+        <v>0.74286130100000003</v>
+      </c>
+      <c r="E111">
+        <v>0.40659013700000002</v>
+      </c>
+      <c r="F111">
+        <v>0.40659013700000002</v>
+      </c>
+      <c r="G111">
+        <v>0.74286130100000003</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>315</v>
+      </c>
+      <c r="B112">
+        <v>2041</v>
+      </c>
+      <c r="C112">
+        <v>7.4044963000000005E-2</v>
+      </c>
+      <c r="D112">
+        <v>0.77541419899999997</v>
+      </c>
+      <c r="E112">
+        <v>0.42472958100000002</v>
+      </c>
+      <c r="F112">
+        <v>0.42472958100000002</v>
+      </c>
+      <c r="G112">
+        <v>0.77541419899999997</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>315</v>
+      </c>
+      <c r="B113">
+        <v>2042</v>
+      </c>
+      <c r="C113">
+        <v>7.7742975000000006E-2</v>
+      </c>
+      <c r="D113">
+        <v>0.80508984299999997</v>
+      </c>
+      <c r="E113">
+        <v>0.44141640900000001</v>
+      </c>
+      <c r="F113">
+        <v>0.44141640900000001</v>
+      </c>
+      <c r="G113">
+        <v>0.80508984299999997</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>315</v>
+      </c>
+      <c r="B114">
+        <v>2043</v>
+      </c>
+      <c r="C114">
+        <v>8.1487271E-2</v>
+      </c>
+      <c r="D114">
+        <v>0.83183468400000005</v>
+      </c>
+      <c r="E114">
+        <v>0.456660978</v>
+      </c>
+      <c r="F114">
+        <v>0.456660978</v>
+      </c>
+      <c r="G114">
+        <v>0.83183468400000005</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>315</v>
+      </c>
+      <c r="B115">
+        <v>2044</v>
+      </c>
+      <c r="C115">
+        <v>8.5272758000000004E-2</v>
+      </c>
+      <c r="D115">
+        <v>0.85566570900000005</v>
+      </c>
+      <c r="E115">
+        <v>0.47046923400000001</v>
+      </c>
+      <c r="F115">
+        <v>0.47046923400000001</v>
+      </c>
+      <c r="G115">
+        <v>0.85566570900000005</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>315</v>
+      </c>
+      <c r="B116">
+        <v>2045</v>
+      </c>
+      <c r="C116">
+        <v>8.9111153999999998E-2</v>
+      </c>
+      <c r="D116">
+        <v>0.87680356800000003</v>
+      </c>
+      <c r="E116">
+        <v>0.48295736099999997</v>
+      </c>
+      <c r="F116">
+        <v>0.48295736099999997</v>
+      </c>
+      <c r="G116">
+        <v>0.87680356800000003</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>315</v>
+      </c>
+      <c r="B117">
+        <v>2046</v>
+      </c>
+      <c r="C117">
+        <v>9.3001159E-2</v>
+      </c>
+      <c r="D117">
+        <v>0.89522190400000001</v>
+      </c>
+      <c r="E117">
+        <v>0.49411153099999999</v>
+      </c>
+      <c r="F117">
+        <v>0.49411153099999999</v>
+      </c>
+      <c r="G117">
+        <v>0.89522190400000001</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>315</v>
+      </c>
+      <c r="B118">
+        <v>2047</v>
+      </c>
+      <c r="C118">
+        <v>9.6893360999999997E-2</v>
+      </c>
+      <c r="D118">
+        <v>0.91109814099999997</v>
+      </c>
+      <c r="E118">
+        <v>0.50399575100000005</v>
+      </c>
+      <c r="F118">
+        <v>0.50399575100000005</v>
+      </c>
+      <c r="G118">
+        <v>0.91109814099999997</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>315</v>
+      </c>
+      <c r="B119">
+        <v>2048</v>
+      </c>
+      <c r="C119">
+        <v>0.100758687</v>
+      </c>
+      <c r="D119">
+        <v>0.92468582899999996</v>
+      </c>
+      <c r="E119">
+        <v>0.51272225800000004</v>
+      </c>
+      <c r="F119">
+        <v>0.51272225800000004</v>
+      </c>
+      <c r="G119">
+        <v>0.92468582899999996</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>315</v>
+      </c>
+      <c r="B120">
+        <v>2049</v>
+      </c>
+      <c r="C120">
+        <v>0.104609438</v>
+      </c>
+      <c r="D120">
+        <v>0.93609858000000001</v>
+      </c>
+      <c r="E120">
+        <v>0.52035400899999995</v>
+      </c>
+      <c r="F120">
+        <v>0.52035400899999995</v>
+      </c>
+      <c r="G120">
+        <v>0.93609858000000001</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>315</v>
+      </c>
+      <c r="B121">
+        <v>2050</v>
+      </c>
+      <c r="C121">
+        <v>0.108448247</v>
+      </c>
+      <c r="D121">
+        <v>0.94575257999999995</v>
+      </c>
+      <c r="E121">
+        <v>0.52710000000000001</v>
+      </c>
+      <c r="F121">
+        <v>0.52710041399999996</v>
+      </c>
+      <c r="G121">
+        <v>0.94575257999999995</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4DD4AF-DD0C-4218-BC59-541B179F4B4B}">
+  <dimension ref="A1:F52"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="14.6328125" customWidth="1"/>
+    <col min="4" max="4" width="19.90625" customWidth="1"/>
+    <col min="5" max="5" width="16.26953125" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D1" t="s">
+        <v>317</v>
+      </c>
+      <c r="E1" t="s">
+        <v>318</v>
+      </c>
+      <c r="F1" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>2019</v>
+      </c>
+      <c r="C2">
+        <v>10150210</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>2019</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>2019</v>
+      </c>
+      <c r="C4">
+        <v>19763274</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>108918663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>2019</v>
+      </c>
+      <c r="C5">
+        <v>6032563</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>2019</v>
+      </c>
+      <c r="C6">
+        <v>2272320341</v>
+      </c>
+      <c r="D6">
+        <v>923680643</v>
+      </c>
+      <c r="E6">
+        <v>1964029505</v>
+      </c>
+      <c r="F6">
+        <v>931495117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>2019</v>
+      </c>
+      <c r="C7">
+        <v>53601802</v>
+      </c>
+      <c r="D7">
+        <v>121331394</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>178266835</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>2019</v>
+      </c>
+      <c r="C8">
+        <v>362943581</v>
+      </c>
+      <c r="D8">
+        <v>16002355</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>2019</v>
+      </c>
+      <c r="C9">
+        <v>142291569</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>2019</v>
+      </c>
+      <c r="C10">
+        <v>179525732</v>
+      </c>
+      <c r="D10">
+        <v>143756233</v>
+      </c>
+      <c r="E10">
+        <v>136546053</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>2019</v>
+      </c>
+      <c r="C11">
+        <v>28108257</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>450023139</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>2019</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>2019</v>
+      </c>
+      <c r="C13">
+        <v>1334134</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>2019</v>
+      </c>
+      <c r="C14">
+        <v>936800351</v>
+      </c>
+      <c r="D14">
+        <v>1365137921</v>
+      </c>
+      <c r="E14">
+        <v>1378128437</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>2019</v>
+      </c>
+      <c r="C15">
+        <v>23368372</v>
+      </c>
+      <c r="D15">
+        <v>108385897</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16">
+        <v>2019</v>
+      </c>
+      <c r="C16">
+        <v>10215072</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17">
+        <v>2019</v>
+      </c>
+      <c r="C17">
+        <v>9219926</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>2019</v>
+      </c>
+      <c r="C18">
+        <v>1659634</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19">
+        <v>2019</v>
+      </c>
+      <c r="C19">
+        <v>34941975</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20">
+        <v>2019</v>
+      </c>
+      <c r="C20">
+        <v>66584121</v>
+      </c>
+      <c r="D20">
+        <v>44297074</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21">
+        <v>2019</v>
+      </c>
+      <c r="C21">
+        <v>403051904</v>
+      </c>
+      <c r="D21">
+        <v>271391388</v>
+      </c>
+      <c r="E21">
+        <v>32470539</v>
+      </c>
+      <c r="F21">
+        <v>39816955</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22">
+        <v>2019</v>
+      </c>
+      <c r="C22">
+        <v>686323124</v>
+      </c>
+      <c r="D22">
+        <v>653570994</v>
+      </c>
+      <c r="E22">
+        <v>572046325</v>
+      </c>
+      <c r="F22">
+        <v>137719112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23">
+        <v>2019</v>
+      </c>
+      <c r="C23">
+        <v>167317988</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24">
+        <v>2019</v>
+      </c>
+      <c r="C24">
+        <v>26177472</v>
+      </c>
+      <c r="D24">
+        <v>18965595</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>100499405</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25">
+        <v>2019</v>
+      </c>
+      <c r="C25">
+        <v>24330591</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26">
+        <v>2019</v>
+      </c>
+      <c r="C26">
+        <v>137330320</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>89068641</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27">
+        <v>2019</v>
+      </c>
+      <c r="C27">
+        <v>24070350</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28">
+        <v>2019</v>
+      </c>
+      <c r="C28">
+        <v>9853074</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29">
+        <v>2019</v>
+      </c>
+      <c r="C29">
+        <v>17645639</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30">
+        <v>2019</v>
+      </c>
+      <c r="C30">
+        <v>85722975</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31">
+        <v>2019</v>
+      </c>
+      <c r="C31">
+        <v>347590724</v>
+      </c>
+      <c r="D31">
+        <v>2006197776</v>
+      </c>
+      <c r="E31">
+        <v>546353547</v>
+      </c>
+      <c r="F31">
+        <v>73704102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32">
+        <v>2019</v>
+      </c>
+      <c r="C32">
+        <v>23165058</v>
+      </c>
+      <c r="D32">
+        <v>35411192</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33">
+        <v>2019</v>
+      </c>
+      <c r="C33">
+        <v>2583207104</v>
+      </c>
+      <c r="D33">
+        <v>5964349570</v>
+      </c>
+      <c r="E33">
+        <v>10511005234</v>
+      </c>
+      <c r="F33">
+        <v>11971472</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>256</v>
+      </c>
+      <c r="B34">
+        <v>2019</v>
+      </c>
+      <c r="C34">
+        <v>184838466</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>45024652</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35">
+        <v>2019</v>
+      </c>
+      <c r="C35">
+        <v>20057435</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36">
+        <v>2019</v>
+      </c>
+      <c r="C36">
+        <v>26201671</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>36529680</v>
+      </c>
+      <c r="F36">
+        <v>8974467</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37">
+        <v>2019</v>
+      </c>
+      <c r="C37">
+        <v>13968539</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38">
+        <v>2019</v>
+      </c>
+      <c r="C38">
+        <v>161077351</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>207967836</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39">
+        <v>2019</v>
+      </c>
+      <c r="C39">
+        <v>1321007165</v>
+      </c>
+      <c r="D39">
+        <v>603541707</v>
+      </c>
+      <c r="E39">
+        <v>399537395</v>
+      </c>
+      <c r="F39">
+        <v>28888028</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40">
+        <v>2019</v>
+      </c>
+      <c r="C40">
+        <v>195839815</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>257</v>
+      </c>
+      <c r="B41">
+        <v>2019</v>
+      </c>
+      <c r="C41">
+        <v>35517998</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42">
+        <v>2019</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43">
+        <v>2019</v>
+      </c>
+      <c r="C43">
+        <v>12774245</v>
+      </c>
+      <c r="D43">
+        <v>4544152</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44">
+        <v>2019</v>
+      </c>
+      <c r="C44">
+        <v>72175940</v>
+      </c>
+      <c r="D44">
+        <v>41940297</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>279333373</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>45</v>
+      </c>
+      <c r="B45">
+        <v>2019</v>
+      </c>
+      <c r="C45">
+        <v>11341330</v>
+      </c>
+      <c r="D45">
+        <v>133685517</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>83098538</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46">
+        <v>2019</v>
+      </c>
+      <c r="C46">
+        <v>18429934</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>47</v>
+      </c>
+      <c r="B47">
+        <v>2019</v>
+      </c>
+      <c r="C47">
+        <v>306024295</v>
+      </c>
+      <c r="D47">
+        <v>135051068</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>4798117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48">
+        <v>2019</v>
+      </c>
+      <c r="C48">
+        <v>258175574</v>
+      </c>
+      <c r="D48">
+        <v>116066343</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>163463700</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>11</v>
+      </c>
+      <c r="B49">
+        <v>2019</v>
+      </c>
+      <c r="C49">
+        <v>1032877444</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>1313511151</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>2019</v>
+      </c>
+      <c r="C50">
+        <v>10228758</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>2019</v>
+      </c>
+      <c r="C51">
+        <v>192765515</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>2019</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8190302C-E34C-4DC7-B5A5-3449292AAE8F}">
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="37" customWidth="1"/>
+    <col min="3" max="3" width="33.26953125" customWidth="1"/>
+    <col min="4" max="4" width="33.453125" customWidth="1"/>
+    <col min="5" max="5" width="33" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C1" t="s">
+        <v>321</v>
+      </c>
+      <c r="D1" t="s">
+        <v>322</v>
+      </c>
+      <c r="E1" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>2019</v>
+      </c>
+      <c r="B2">
+        <v>1506</v>
+      </c>
+      <c r="C2">
+        <v>1583</v>
+      </c>
+      <c r="D2">
+        <v>851</v>
+      </c>
+      <c r="E2">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2020</v>
+      </c>
+      <c r="B3">
+        <v>1506</v>
+      </c>
+      <c r="C3">
+        <v>1583</v>
+      </c>
+      <c r="D3">
+        <v>851</v>
+      </c>
+      <c r="E3">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2021</v>
+      </c>
+      <c r="B4">
+        <v>1506</v>
+      </c>
+      <c r="C4">
+        <v>1583</v>
+      </c>
+      <c r="D4">
+        <v>851</v>
+      </c>
+      <c r="E4">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>2022</v>
+      </c>
+      <c r="B5">
+        <v>1506</v>
+      </c>
+      <c r="C5">
+        <v>1583</v>
+      </c>
+      <c r="D5">
+        <v>851</v>
+      </c>
+      <c r="E5">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>2023</v>
+      </c>
+      <c r="B6">
+        <v>1506</v>
+      </c>
+      <c r="C6">
+        <v>1583</v>
+      </c>
+      <c r="D6">
+        <v>851</v>
+      </c>
+      <c r="E6">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>2024</v>
+      </c>
+      <c r="B7">
+        <v>1506</v>
+      </c>
+      <c r="C7">
+        <v>1583</v>
+      </c>
+      <c r="D7">
+        <v>851</v>
+      </c>
+      <c r="E7">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>2025</v>
+      </c>
+      <c r="B8">
+        <v>1506</v>
+      </c>
+      <c r="C8">
+        <v>1583</v>
+      </c>
+      <c r="D8">
+        <v>851</v>
+      </c>
+      <c r="E8">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>2026</v>
+      </c>
+      <c r="B9">
+        <v>1506</v>
+      </c>
+      <c r="C9">
+        <v>1583</v>
+      </c>
+      <c r="D9">
+        <v>851</v>
+      </c>
+      <c r="E9">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>2027</v>
+      </c>
+      <c r="B10">
+        <v>1506</v>
+      </c>
+      <c r="C10">
+        <v>1583</v>
+      </c>
+      <c r="D10">
+        <v>851</v>
+      </c>
+      <c r="E10">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>2028</v>
+      </c>
+      <c r="B11">
+        <v>1506</v>
+      </c>
+      <c r="C11">
+        <v>1583</v>
+      </c>
+      <c r="D11">
+        <v>851</v>
+      </c>
+      <c r="E11">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>2029</v>
+      </c>
+      <c r="B12">
+        <v>1506</v>
+      </c>
+      <c r="C12">
+        <v>1583</v>
+      </c>
+      <c r="D12">
+        <v>851</v>
+      </c>
+      <c r="E12">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>2030</v>
+      </c>
+      <c r="B13">
+        <v>1506</v>
+      </c>
+      <c r="C13">
+        <v>1583</v>
+      </c>
+      <c r="D13">
+        <v>851</v>
+      </c>
+      <c r="E13">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>2031</v>
+      </c>
+      <c r="B14">
+        <v>1506</v>
+      </c>
+      <c r="C14">
+        <v>1583</v>
+      </c>
+      <c r="D14">
+        <v>851</v>
+      </c>
+      <c r="E14">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>2032</v>
+      </c>
+      <c r="B15">
+        <v>1506</v>
+      </c>
+      <c r="C15">
+        <v>1583</v>
+      </c>
+      <c r="D15">
+        <v>851</v>
+      </c>
+      <c r="E15">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>2033</v>
+      </c>
+      <c r="B16">
+        <v>1506</v>
+      </c>
+      <c r="C16">
+        <v>1583</v>
+      </c>
+      <c r="D16">
+        <v>851</v>
+      </c>
+      <c r="E16">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>2034</v>
+      </c>
+      <c r="B17">
+        <v>1506</v>
+      </c>
+      <c r="C17">
+        <v>1583</v>
+      </c>
+      <c r="D17">
+        <v>851</v>
+      </c>
+      <c r="E17">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>2035</v>
+      </c>
+      <c r="B18">
+        <v>1506</v>
+      </c>
+      <c r="C18">
+        <v>1583</v>
+      </c>
+      <c r="D18">
+        <v>851</v>
+      </c>
+      <c r="E18">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>2036</v>
+      </c>
+      <c r="B19">
+        <v>1506</v>
+      </c>
+      <c r="C19">
+        <v>1583</v>
+      </c>
+      <c r="D19">
+        <v>851</v>
+      </c>
+      <c r="E19">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>2037</v>
+      </c>
+      <c r="B20">
+        <v>1506</v>
+      </c>
+      <c r="C20">
+        <v>1583</v>
+      </c>
+      <c r="D20">
+        <v>851</v>
+      </c>
+      <c r="E20">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>2038</v>
+      </c>
+      <c r="B21">
+        <v>1506</v>
+      </c>
+      <c r="C21">
+        <v>1583</v>
+      </c>
+      <c r="D21">
+        <v>851</v>
+      </c>
+      <c r="E21">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>2039</v>
+      </c>
+      <c r="B22">
+        <v>1506</v>
+      </c>
+      <c r="C22">
+        <v>1583</v>
+      </c>
+      <c r="D22">
+        <v>851</v>
+      </c>
+      <c r="E22">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>2040</v>
+      </c>
+      <c r="B23">
+        <v>1506</v>
+      </c>
+      <c r="C23">
+        <v>1583</v>
+      </c>
+      <c r="D23">
+        <v>851</v>
+      </c>
+      <c r="E23">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>2041</v>
+      </c>
+      <c r="B24">
+        <v>1506</v>
+      </c>
+      <c r="C24">
+        <v>1583</v>
+      </c>
+      <c r="D24">
+        <v>851</v>
+      </c>
+      <c r="E24">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>2042</v>
+      </c>
+      <c r="B25">
+        <v>1506</v>
+      </c>
+      <c r="C25">
+        <v>1583</v>
+      </c>
+      <c r="D25">
+        <v>851</v>
+      </c>
+      <c r="E25">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>2043</v>
+      </c>
+      <c r="B26">
+        <v>1506</v>
+      </c>
+      <c r="C26">
+        <v>1583</v>
+      </c>
+      <c r="D26">
+        <v>851</v>
+      </c>
+      <c r="E26">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>2044</v>
+      </c>
+      <c r="B27">
+        <v>1506</v>
+      </c>
+      <c r="C27">
+        <v>1583</v>
+      </c>
+      <c r="D27">
+        <v>851</v>
+      </c>
+      <c r="E27">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>2045</v>
+      </c>
+      <c r="B28">
+        <v>1506</v>
+      </c>
+      <c r="C28">
+        <v>1583</v>
+      </c>
+      <c r="D28">
+        <v>851</v>
+      </c>
+      <c r="E28">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>2046</v>
+      </c>
+      <c r="B29">
+        <v>1506</v>
+      </c>
+      <c r="C29">
+        <v>1583</v>
+      </c>
+      <c r="D29">
+        <v>851</v>
+      </c>
+      <c r="E29">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>2047</v>
+      </c>
+      <c r="B30">
+        <v>1506</v>
+      </c>
+      <c r="C30">
+        <v>1583</v>
+      </c>
+      <c r="D30">
+        <v>851</v>
+      </c>
+      <c r="E30">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>2048</v>
+      </c>
+      <c r="B31">
+        <v>1506</v>
+      </c>
+      <c r="C31">
+        <v>1583</v>
+      </c>
+      <c r="D31">
+        <v>851</v>
+      </c>
+      <c r="E31">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>2049</v>
+      </c>
+      <c r="B32">
+        <v>1506</v>
+      </c>
+      <c r="C32">
+        <v>1583</v>
+      </c>
+      <c r="D32">
+        <v>851</v>
+      </c>
+      <c r="E32">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>2050</v>
+      </c>
+      <c r="B33">
+        <v>1506</v>
+      </c>
+      <c r="C33">
+        <v>1583</v>
+      </c>
+      <c r="D33">
+        <v>851</v>
+      </c>
+      <c r="E33">
+        <v>851</v>
       </c>
     </row>
   </sheetData>
@@ -59221,12 +63997,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>259</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
       <c r="G2" s="17">
         <f>SUM([1]AEO_VMT_Base!$B$6:$B$7)/[1]AEO_VMT_Base!$B$10</f>
         <v>0.90535164725664219</v>
@@ -82254,15 +87030,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -82444,6 +87211,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -82451,14 +87227,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -82476,6 +87244,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
-Fixing a Merge Issue I Created :angel:
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -87039,12 +87039,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -87226,6 +87220,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
   <ds:schemaRefs>
@@ -87235,15 +87235,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -87259,4 +87250,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "-Fixing a Merge Issue I Created :angel:"
This reverts commit 00adbe134ae213b117e0d83284fe85015e551b65.
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -87039,6 +87039,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -87220,12 +87226,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
   <ds:schemaRefs>
@@ -87235,6 +87235,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -87250,13 +87259,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "Merge branch 'main' of https://github.com/camsys/TEACART"
This reverts commit 983e74fc48447816ae2ac47e9b6617e1ff3a19f3, reversing
changes made to 4f793bf8efdad635772b05a989597d178ef3c11b.
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -87030,21 +87030,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -87226,24 +87211,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -87259,4 +87242,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "Public Rail + Tech Frac Fixes"
This reverts commit 4f793bf8efdad635772b05a989597d178ef3c11b.
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{EE2E0D63-B56C-4BDE-BCAD-5F60909CE8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A7CC7D6-F03E-4234-BF37-5810BC20243F}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{12930437-8380-4A20-BC55-0F37E67B4891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1B8D76C-00D5-4846-BCB1-A43933AB5893}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="821" firstSheet="14" activeTab="18" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="29070" yWindow="-14715" windowWidth="16440" windowHeight="29040" tabRatio="821" activeTab="1" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -26,17 +26,13 @@
     <sheet name="Transit_Costs" sheetId="16" r:id="rId11"/>
     <sheet name="NTD_Service" sheetId="12" r:id="rId12"/>
     <sheet name="Fuel_Factors" sheetId="14" r:id="rId13"/>
-    <sheet name="Fuel_Factors_Baselines" sheetId="27" r:id="rId14"/>
-    <sheet name="Fuel_Factors_Revision" sheetId="22" r:id="rId15"/>
-    <sheet name="Warming_Potential" sheetId="17" r:id="rId16"/>
-    <sheet name="EV_Forecast" sheetId="23" r:id="rId17"/>
-    <sheet name="Passenger_Rail_State_Mileage" sheetId="24" r:id="rId18"/>
-    <sheet name="Passenger_Rail_FuelFactors" sheetId="25" r:id="rId19"/>
+    <sheet name="Fuel_Factors_Revision" sheetId="22" r:id="rId14"/>
+    <sheet name="Warming_Potential" sheetId="17" r:id="rId15"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId20"/>
-    <externalReference r:id="rId21"/>
-    <externalReference r:id="rId22"/>
+    <externalReference r:id="rId16"/>
+    <externalReference r:id="rId17"/>
+    <externalReference r:id="rId18"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">AEO_VMT_Base!$A$1:$C$1</definedName>
@@ -91,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8606" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8384" uniqueCount="307">
   <si>
     <t>state</t>
   </si>
@@ -1013,84 +1009,6 @@
   <si>
     <t>CO2eq_g_kWh</t>
   </si>
-  <si>
-    <t>percEVstock_AEO</t>
-  </si>
-  <si>
-    <t>percEVstock_ACCII</t>
-  </si>
-  <si>
-    <t>percEVstock_ACC</t>
-  </si>
-  <si>
-    <t>percEVstock_ACCACT</t>
-  </si>
-  <si>
-    <t>percEVstock_ACCIIACT</t>
-  </si>
-  <si>
-    <t>Heavy Duty Truck</t>
-  </si>
-  <si>
-    <t>Light Duty Truck</t>
-  </si>
-  <si>
-    <t>Medium Duty Truck</t>
-  </si>
-  <si>
-    <t>Passenger Car</t>
-  </si>
-  <si>
-    <t>amtrak_riders</t>
-  </si>
-  <si>
-    <t>commuterrail_miles</t>
-  </si>
-  <si>
-    <t>heavyrail_miles</t>
-  </si>
-  <si>
-    <t>lightrail_miles</t>
-  </si>
-  <si>
-    <t>amtrak_Energy_Intensity_BTUPerPaxMil</t>
-  </si>
-  <si>
-    <t>CR_Energy_Intensity_BTUPerPaxMil</t>
-  </si>
-  <si>
-    <t>HR_Energy_Intensity_BTUPerPaxMil</t>
-  </si>
-  <si>
-    <t>LR_Energy_Intensity_BTUPerPaxMil</t>
-  </si>
-  <si>
-    <t>Propane</t>
-  </si>
-  <si>
-    <t>units</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>upstream_life_cycle_Factor</t>
-  </si>
-  <si>
-    <t>electricity</t>
-  </si>
-  <si>
-    <t>fuel_conversion_gasoline_equivalent</t>
-  </si>
-  <si>
-    <t>fuel_conversion_BTU</t>
-  </si>
-  <si>
-    <t>energy_efficiency_ratio</t>
-  </si>
-  <si>
-    <t>CNG to Diesel</t>
-  </si>
 </sst>
 </file>
 
@@ -1200,7 +1118,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1223,7 +1141,6 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2890,18 +2807,6 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{518D259B-7CFD-40C9-852E-5504E1166921}" name="Fuel_Factors_Baseline" displayName="Fuel_Factors_Baseline" ref="A1:C16" totalsRowShown="0">
-  <autoFilter ref="A1:C16" xr:uid="{518D259B-7CFD-40C9-852E-5504E1166921}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CEC5F72C-E366-45EB-B906-60DFE2C20A8F}" name="fuel_type"/>
-    <tableColumn id="2" xr3:uid="{C607764C-F28E-4CFA-8C1F-C3427D0186D8}" name="units"/>
-    <tableColumn id="3" xr3:uid="{2CEB8B5E-0AE4-47CF-ADC1-6A60B25483AE}" name="value"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{03AFADD4-FAEA-41F7-A128-A44DAF1E827F}" name="Fuel_Factors_Revision" displayName="Fuel_Factors_Revision" ref="A1:K39" totalsRowShown="0">
   <autoFilter ref="A1:K39" xr:uid="{03AFADD4-FAEA-41F7-A128-A44DAF1E827F}"/>
   <tableColumns count="11">
@@ -2921,57 +2826,12 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6DFCB0CB-F0C1-406B-8BC4-DBF1C6DEF1BD}" name="GWP" displayName="GWP" ref="A1:B3" totalsRowShown="0">
   <autoFilter ref="A1:B3" xr:uid="{6DFCB0CB-F0C1-406B-8BC4-DBF1C6DEF1BD}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{C7571F8A-FAEB-418D-B890-7F650F2EC67E}" name="Gas"/>
     <tableColumn id="2" xr3:uid="{0A2C010A-79AE-435E-98A7-45ED8AF3EA48}" name="GWP"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{3D4BD3A3-7756-49E2-B00A-144DD3C0AB84}" name="EV_Forecast" displayName="EV_Forecast" ref="A1:G121" totalsRowShown="0">
-  <autoFilter ref="A1:G121" xr:uid="{3D4BD3A3-7756-49E2-B00A-144DD3C0AB84}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{98339C45-1FB4-4A31-A342-8A18C9D17CBF}" name="veh_type"/>
-    <tableColumn id="2" xr3:uid="{5448A7A5-8D60-4DB5-9002-C1C331D0B9BD}" name="year"/>
-    <tableColumn id="3" xr3:uid="{6C87E9A0-5979-4F0A-AEC0-A63C0F93051B}" name="percEVstock_AEO"/>
-    <tableColumn id="4" xr3:uid="{1AEA079B-7185-4543-8E7E-17320AB65398}" name="percEVstock_ACCII"/>
-    <tableColumn id="5" xr3:uid="{C201EFA0-9EE7-44A0-911D-38D56E3B907B}" name="percEVstock_ACC"/>
-    <tableColumn id="6" xr3:uid="{941DD455-3F84-44FE-BE56-FB8C7695A3F6}" name="percEVstock_ACCACT"/>
-    <tableColumn id="7" xr3:uid="{C571AE9D-EDC5-441E-BD86-18F36763A9BA}" name="percEVstock_ACCIIACT"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{3C9ACDE8-AAE2-4347-8072-D2D12BA0A2E5}" name="Passenger_Rail_State_Mileage" displayName="Passenger_Rail_State_Mileage" ref="A1:F52" totalsRowShown="0">
-  <autoFilter ref="A1:F52" xr:uid="{3C9ACDE8-AAE2-4347-8072-D2D12BA0A2E5}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{BDBC3F5C-D408-43E1-81EC-95C50C377D64}" name="state"/>
-    <tableColumn id="2" xr3:uid="{36E465BC-AC57-462E-8C5F-2264EACFA55C}" name="year"/>
-    <tableColumn id="3" xr3:uid="{469EDCC2-4A35-4A7D-AA02-B7FC795193D0}" name="amtrak_riders"/>
-    <tableColumn id="4" xr3:uid="{C72C4CFA-8DBF-437E-B532-4E876AF07824}" name="commuterrail_miles"/>
-    <tableColumn id="5" xr3:uid="{A69FEAF6-C35E-44ED-9457-60BCB7A154FD}" name="heavyrail_miles"/>
-    <tableColumn id="6" xr3:uid="{40439AC9-0C67-414F-A72A-182AB961EF72}" name="lightrail_miles"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}" name="Passenger_Rail_FuelFactors" displayName="Passenger_Rail_FuelFactors" ref="A1:E33" totalsRowShown="0">
-  <autoFilter ref="A1:E33" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E1F2670B-316B-4194-A86B-8536CC6E5F6A}" name="year"/>
-    <tableColumn id="2" xr3:uid="{B177438D-BB65-4F5B-B9B2-4F2ACFB89EBB}" name="amtrak_Energy_Intensity_BTUPerPaxMil"/>
-    <tableColumn id="3" xr3:uid="{145EDF5A-67AC-4FBD-8747-BD532DBD07D2}" name="CR_Energy_Intensity_BTUPerPaxMil"/>
-    <tableColumn id="4" xr3:uid="{FABA830F-9553-48B4-B4E7-CA28DF0F2168}" name="HR_Energy_Intensity_BTUPerPaxMil"/>
-    <tableColumn id="5" xr3:uid="{5411A020-667E-4006-86A4-6CBDBC158F0A}" name="LR_Energy_Intensity_BTUPerPaxMil"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -19676,199 +19536,6 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFD11A43-B943-40FD-8C75-39E96A18C306}">
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" t="s">
-        <v>325</v>
-      </c>
-      <c r="C1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B2" t="s">
-        <v>289</v>
-      </c>
-      <c r="C2" s="20">
-        <v>7.94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C3">
-        <v>9.4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" t="s">
-        <v>289</v>
-      </c>
-      <c r="C4">
-        <v>5.4399999999999997E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>324</v>
-      </c>
-      <c r="B5" t="s">
-        <v>289</v>
-      </c>
-      <c r="C5">
-        <v>5.72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B6" t="s">
-        <v>327</v>
-      </c>
-      <c r="C6">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" t="s">
-        <v>327</v>
-      </c>
-      <c r="C7">
-        <v>0.21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" t="s">
-        <v>327</v>
-      </c>
-      <c r="C8">
-        <v>0.28999999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>328</v>
-      </c>
-      <c r="B9" t="s">
-        <v>329</v>
-      </c>
-      <c r="C9">
-        <v>33.977738722905684</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>156</v>
-      </c>
-      <c r="B10" t="s">
-        <v>329</v>
-      </c>
-      <c r="C10">
-        <v>0.89285714285714279</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>324</v>
-      </c>
-      <c r="B11" t="s">
-        <v>329</v>
-      </c>
-      <c r="C11">
-        <v>1.3513513513513513</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" t="s">
-        <v>329</v>
-      </c>
-      <c r="C12">
-        <v>123.57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>328</v>
-      </c>
-      <c r="B13" t="s">
-        <v>330</v>
-      </c>
-      <c r="C13">
-        <v>3414</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>182</v>
-      </c>
-      <c r="B14" t="s">
-        <v>330</v>
-      </c>
-      <c r="C14">
-        <v>116000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>156</v>
-      </c>
-      <c r="B15" t="s">
-        <v>330</v>
-      </c>
-      <c r="C15">
-        <v>128500</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>332</v>
-      </c>
-      <c r="B16" t="s">
-        <v>331</v>
-      </c>
-      <c r="C16">
-        <v>0.9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B8B760-61E2-4C3C-B734-67EBC38A98CD}">
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -21259,7 +20926,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EF48310-0F86-4489-96AB-7F1DA3A7B2B6}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -21286,4449 +20953,6 @@
       </c>
       <c r="B3">
         <v>298</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{241E29C4-5664-445C-AFC0-25E977A29D94}">
-  <dimension ref="A1:G121"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="10.81640625" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" customWidth="1"/>
-    <col min="5" max="5" width="17.453125" customWidth="1"/>
-    <col min="6" max="6" width="20.7265625" customWidth="1"/>
-    <col min="7" max="7" width="21.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>307</v>
-      </c>
-      <c r="D1" t="s">
-        <v>308</v>
-      </c>
-      <c r="E1" t="s">
-        <v>309</v>
-      </c>
-      <c r="F1" t="s">
-        <v>310</v>
-      </c>
-      <c r="G1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>312</v>
-      </c>
-      <c r="B2">
-        <v>2021</v>
-      </c>
-      <c r="C2">
-        <v>1.7833599999999999E-4</v>
-      </c>
-      <c r="D2">
-        <v>1.7833599999999999E-4</v>
-      </c>
-      <c r="E2">
-        <v>1.7833599999999999E-4</v>
-      </c>
-      <c r="F2">
-        <v>1.7833599999999999E-4</v>
-      </c>
-      <c r="G2">
-        <v>1.7833599999999999E-4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>312</v>
-      </c>
-      <c r="B3">
-        <v>2022</v>
-      </c>
-      <c r="C3">
-        <v>3.3397599999999999E-4</v>
-      </c>
-      <c r="D3">
-        <v>3.3397599999999999E-4</v>
-      </c>
-      <c r="E3">
-        <v>3.3397599999999999E-4</v>
-      </c>
-      <c r="F3">
-        <v>3.3397599999999999E-4</v>
-      </c>
-      <c r="G3">
-        <v>3.3397599999999999E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>312</v>
-      </c>
-      <c r="B4">
-        <v>2023</v>
-      </c>
-      <c r="C4">
-        <v>4.9029200000000003E-4</v>
-      </c>
-      <c r="D4">
-        <v>4.9029200000000003E-4</v>
-      </c>
-      <c r="E4">
-        <v>4.9029200000000003E-4</v>
-      </c>
-      <c r="F4">
-        <v>4.9029200000000003E-4</v>
-      </c>
-      <c r="G4">
-        <v>4.9029200000000003E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>312</v>
-      </c>
-      <c r="B5">
-        <v>2024</v>
-      </c>
-      <c r="C5">
-        <v>6.4432900000000002E-4</v>
-      </c>
-      <c r="D5">
-        <v>6.4432900000000002E-4</v>
-      </c>
-      <c r="E5">
-        <v>6.4432900000000002E-4</v>
-      </c>
-      <c r="F5">
-        <v>2.8879320000000002E-3</v>
-      </c>
-      <c r="G5">
-        <v>2.8879320000000002E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>312</v>
-      </c>
-      <c r="B6">
-        <v>2025</v>
-      </c>
-      <c r="C6">
-        <v>7.96417E-4</v>
-      </c>
-      <c r="D6">
-        <v>7.96417E-4</v>
-      </c>
-      <c r="E6">
-        <v>7.96417E-4</v>
-      </c>
-      <c r="F6">
-        <v>6.3800389999999997E-3</v>
-      </c>
-      <c r="G6">
-        <v>6.3800389999999997E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>312</v>
-      </c>
-      <c r="B7">
-        <v>2026</v>
-      </c>
-      <c r="C7">
-        <v>9.4634700000000005E-4</v>
-      </c>
-      <c r="D7">
-        <v>9.4634700000000005E-4</v>
-      </c>
-      <c r="E7">
-        <v>9.4634700000000005E-4</v>
-      </c>
-      <c r="F7">
-        <v>1.0761928E-2</v>
-      </c>
-      <c r="G7">
-        <v>1.0761928E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>312</v>
-      </c>
-      <c r="B8">
-        <v>2027</v>
-      </c>
-      <c r="C8">
-        <v>1.0917800000000001E-3</v>
-      </c>
-      <c r="D8">
-        <v>1.0917800000000001E-3</v>
-      </c>
-      <c r="E8">
-        <v>1.0917800000000001E-3</v>
-      </c>
-      <c r="F8">
-        <v>1.6864591000000002E-2</v>
-      </c>
-      <c r="G8">
-        <v>1.6864591000000002E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>312</v>
-      </c>
-      <c r="B9">
-        <v>2028</v>
-      </c>
-      <c r="C9">
-        <v>1.234576E-3</v>
-      </c>
-      <c r="D9">
-        <v>1.234576E-3</v>
-      </c>
-      <c r="E9">
-        <v>1.234576E-3</v>
-      </c>
-      <c r="F9">
-        <v>2.5187912999999999E-2</v>
-      </c>
-      <c r="G9">
-        <v>2.5187912999999999E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>312</v>
-      </c>
-      <c r="B10">
-        <v>2029</v>
-      </c>
-      <c r="C10">
-        <v>1.377184E-3</v>
-      </c>
-      <c r="D10">
-        <v>1.377184E-3</v>
-      </c>
-      <c r="E10">
-        <v>1.377184E-3</v>
-      </c>
-      <c r="F10">
-        <v>3.5627709E-2</v>
-      </c>
-      <c r="G10">
-        <v>3.5627709E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>312</v>
-      </c>
-      <c r="B11">
-        <v>2030</v>
-      </c>
-      <c r="C11">
-        <v>1.5188409999999999E-3</v>
-      </c>
-      <c r="D11">
-        <v>1.5188409999999999E-3</v>
-      </c>
-      <c r="E11">
-        <v>1.5188409999999999E-3</v>
-      </c>
-      <c r="F11">
-        <v>4.7980977000000001E-2</v>
-      </c>
-      <c r="G11">
-        <v>4.7980977000000001E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>312</v>
-      </c>
-      <c r="B12">
-        <v>2031</v>
-      </c>
-      <c r="C12">
-        <v>1.6599869999999999E-3</v>
-      </c>
-      <c r="D12">
-        <v>1.6599869999999999E-3</v>
-      </c>
-      <c r="E12">
-        <v>1.6599869999999999E-3</v>
-      </c>
-      <c r="F12">
-        <v>6.1868593999999999E-2</v>
-      </c>
-      <c r="G12">
-        <v>6.1868593999999999E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>312</v>
-      </c>
-      <c r="B13">
-        <v>2032</v>
-      </c>
-      <c r="C13">
-        <v>1.8000679999999999E-3</v>
-      </c>
-      <c r="D13">
-        <v>1.8000679999999999E-3</v>
-      </c>
-      <c r="E13">
-        <v>1.8000679999999999E-3</v>
-      </c>
-      <c r="F13">
-        <v>7.6526794999999995E-2</v>
-      </c>
-      <c r="G13">
-        <v>7.6526794999999995E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>312</v>
-      </c>
-      <c r="B14">
-        <v>2033</v>
-      </c>
-      <c r="C14">
-        <v>1.9408330000000001E-3</v>
-      </c>
-      <c r="D14">
-        <v>1.9408330000000001E-3</v>
-      </c>
-      <c r="E14">
-        <v>1.9408330000000001E-3</v>
-      </c>
-      <c r="F14">
-        <v>9.1638549E-2</v>
-      </c>
-      <c r="G14">
-        <v>9.1638549E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>312</v>
-      </c>
-      <c r="B15">
-        <v>2034</v>
-      </c>
-      <c r="C15">
-        <v>2.0840559999999999E-3</v>
-      </c>
-      <c r="D15">
-        <v>2.0840559999999999E-3</v>
-      </c>
-      <c r="E15">
-        <v>2.0840559999999999E-3</v>
-      </c>
-      <c r="F15">
-        <v>0.106988207</v>
-      </c>
-      <c r="G15">
-        <v>0.106988207</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>312</v>
-      </c>
-      <c r="B16">
-        <v>2035</v>
-      </c>
-      <c r="C16">
-        <v>2.2269479999999999E-3</v>
-      </c>
-      <c r="D16">
-        <v>2.2269479999999999E-3</v>
-      </c>
-      <c r="E16">
-        <v>2.2269479999999999E-3</v>
-      </c>
-      <c r="F16">
-        <v>0.12328299600000001</v>
-      </c>
-      <c r="G16">
-        <v>0.12328299600000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>312</v>
-      </c>
-      <c r="B17">
-        <v>2036</v>
-      </c>
-      <c r="C17">
-        <v>2.3683300000000001E-3</v>
-      </c>
-      <c r="D17">
-        <v>2.3683300000000001E-3</v>
-      </c>
-      <c r="E17">
-        <v>2.3683300000000001E-3</v>
-      </c>
-      <c r="F17">
-        <v>0.13350161599999999</v>
-      </c>
-      <c r="G17">
-        <v>0.13350161599999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>312</v>
-      </c>
-      <c r="B18">
-        <v>2037</v>
-      </c>
-      <c r="C18">
-        <v>2.5096810000000002E-3</v>
-      </c>
-      <c r="D18">
-        <v>2.5096810000000002E-3</v>
-      </c>
-      <c r="E18">
-        <v>2.5096810000000002E-3</v>
-      </c>
-      <c r="F18">
-        <v>0.14717171300000001</v>
-      </c>
-      <c r="G18">
-        <v>0.14717171300000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>312</v>
-      </c>
-      <c r="B19">
-        <v>2038</v>
-      </c>
-      <c r="C19">
-        <v>2.6516360000000002E-3</v>
-      </c>
-      <c r="D19">
-        <v>2.6516360000000002E-3</v>
-      </c>
-      <c r="E19">
-        <v>2.6516360000000002E-3</v>
-      </c>
-      <c r="F19">
-        <v>0.159999847</v>
-      </c>
-      <c r="G19">
-        <v>0.159999847</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>312</v>
-      </c>
-      <c r="B20">
-        <v>2039</v>
-      </c>
-      <c r="C20">
-        <v>2.7978980000000001E-3</v>
-      </c>
-      <c r="D20">
-        <v>2.7978980000000001E-3</v>
-      </c>
-      <c r="E20">
-        <v>2.7978980000000001E-3</v>
-      </c>
-      <c r="F20">
-        <v>0.17197367399999999</v>
-      </c>
-      <c r="G20">
-        <v>0.17197367399999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>312</v>
-      </c>
-      <c r="B21">
-        <v>2040</v>
-      </c>
-      <c r="C21">
-        <v>2.9475489999999998E-3</v>
-      </c>
-      <c r="D21">
-        <v>2.9475489999999998E-3</v>
-      </c>
-      <c r="E21">
-        <v>2.9475489999999998E-3</v>
-      </c>
-      <c r="F21">
-        <v>0.18306308800000001</v>
-      </c>
-      <c r="G21">
-        <v>0.18306308800000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>312</v>
-      </c>
-      <c r="B22">
-        <v>2041</v>
-      </c>
-      <c r="C22">
-        <v>3.1025660000000002E-3</v>
-      </c>
-      <c r="D22">
-        <v>3.1025660000000002E-3</v>
-      </c>
-      <c r="E22">
-        <v>3.1025660000000002E-3</v>
-      </c>
-      <c r="F22">
-        <v>0.19322018599999999</v>
-      </c>
-      <c r="G22">
-        <v>0.19322018599999999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>312</v>
-      </c>
-      <c r="B23">
-        <v>2042</v>
-      </c>
-      <c r="C23">
-        <v>3.2548310000000001E-3</v>
-      </c>
-      <c r="D23">
-        <v>3.2548310000000001E-3</v>
-      </c>
-      <c r="E23">
-        <v>3.2548310000000001E-3</v>
-      </c>
-      <c r="F23">
-        <v>0.20237197600000001</v>
-      </c>
-      <c r="G23">
-        <v>0.20237197600000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>312</v>
-      </c>
-      <c r="B24">
-        <v>2043</v>
-      </c>
-      <c r="C24">
-        <v>3.4059329999999999E-3</v>
-      </c>
-      <c r="D24">
-        <v>3.4059329999999999E-3</v>
-      </c>
-      <c r="E24">
-        <v>3.4059329999999999E-3</v>
-      </c>
-      <c r="F24">
-        <v>0.21056287000000001</v>
-      </c>
-      <c r="G24">
-        <v>0.21056287000000001</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>312</v>
-      </c>
-      <c r="B25">
-        <v>2044</v>
-      </c>
-      <c r="C25">
-        <v>3.5547740000000001E-3</v>
-      </c>
-      <c r="D25">
-        <v>3.5547740000000001E-3</v>
-      </c>
-      <c r="E25">
-        <v>3.5547740000000001E-3</v>
-      </c>
-      <c r="F25">
-        <v>0.21777566700000001</v>
-      </c>
-      <c r="G25">
-        <v>0.21777566700000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>312</v>
-      </c>
-      <c r="B26">
-        <v>2045</v>
-      </c>
-      <c r="C26">
-        <v>3.702253E-3</v>
-      </c>
-      <c r="D26">
-        <v>3.702253E-3</v>
-      </c>
-      <c r="E26">
-        <v>3.702253E-3</v>
-      </c>
-      <c r="F26">
-        <v>0.224084228</v>
-      </c>
-      <c r="G26">
-        <v>0.224084228</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>312</v>
-      </c>
-      <c r="B27">
-        <v>2046</v>
-      </c>
-      <c r="C27">
-        <v>3.8532660000000002E-3</v>
-      </c>
-      <c r="D27">
-        <v>3.8532660000000002E-3</v>
-      </c>
-      <c r="E27">
-        <v>3.8532660000000002E-3</v>
-      </c>
-      <c r="F27">
-        <v>0.229570676</v>
-      </c>
-      <c r="G27">
-        <v>0.229570676</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>312</v>
-      </c>
-      <c r="B28">
-        <v>2047</v>
-      </c>
-      <c r="C28">
-        <v>4.0069169999999996E-3</v>
-      </c>
-      <c r="D28">
-        <v>4.0069169999999996E-3</v>
-      </c>
-      <c r="E28">
-        <v>4.0069169999999996E-3</v>
-      </c>
-      <c r="F28">
-        <v>0.23429806</v>
-      </c>
-      <c r="G28">
-        <v>0.23429806</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>312</v>
-      </c>
-      <c r="B29">
-        <v>2048</v>
-      </c>
-      <c r="C29">
-        <v>4.1629220000000003E-3</v>
-      </c>
-      <c r="D29">
-        <v>4.1629220000000003E-3</v>
-      </c>
-      <c r="E29">
-        <v>4.1629220000000003E-3</v>
-      </c>
-      <c r="F29">
-        <v>0.23831492700000001</v>
-      </c>
-      <c r="G29">
-        <v>0.23831492700000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>312</v>
-      </c>
-      <c r="B30">
-        <v>2049</v>
-      </c>
-      <c r="C30">
-        <v>4.3251549999999998E-3</v>
-      </c>
-      <c r="D30">
-        <v>4.3251549999999998E-3</v>
-      </c>
-      <c r="E30">
-        <v>4.3251549999999998E-3</v>
-      </c>
-      <c r="F30">
-        <v>0.241681439</v>
-      </c>
-      <c r="G30">
-        <v>0.241681439</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>312</v>
-      </c>
-      <c r="B31">
-        <v>2050</v>
-      </c>
-      <c r="C31">
-        <v>4.495321E-3</v>
-      </c>
-      <c r="D31">
-        <v>4.495321E-3</v>
-      </c>
-      <c r="E31">
-        <v>4.495321E-3</v>
-      </c>
-      <c r="F31">
-        <v>0.24449030199999999</v>
-      </c>
-      <c r="G31">
-        <v>0.24449030199999999</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>313</v>
-      </c>
-      <c r="B32">
-        <v>2021</v>
-      </c>
-      <c r="C32">
-        <v>2.7681490000000001E-3</v>
-      </c>
-      <c r="D32">
-        <v>2.7681490000000001E-3</v>
-      </c>
-      <c r="E32">
-        <v>2.7681490000000001E-3</v>
-      </c>
-      <c r="F32">
-        <v>2.7681490000000001E-3</v>
-      </c>
-      <c r="G32">
-        <v>2.7681490000000001E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>313</v>
-      </c>
-      <c r="B33">
-        <v>2022</v>
-      </c>
-      <c r="C33">
-        <v>5.506319E-3</v>
-      </c>
-      <c r="D33">
-        <v>8.2696799999999997E-3</v>
-      </c>
-      <c r="E33">
-        <v>6.8879989999999997E-3</v>
-      </c>
-      <c r="F33">
-        <v>6.8879989999999997E-3</v>
-      </c>
-      <c r="G33">
-        <v>8.2696799999999997E-3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>313</v>
-      </c>
-      <c r="B34">
-        <v>2023</v>
-      </c>
-      <c r="C34">
-        <v>8.604024E-3</v>
-      </c>
-      <c r="D34">
-        <v>1.3771211E-2</v>
-      </c>
-      <c r="E34">
-        <v>1.1187618E-2</v>
-      </c>
-      <c r="F34">
-        <v>1.1187618E-2</v>
-      </c>
-      <c r="G34">
-        <v>1.3771211E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>313</v>
-      </c>
-      <c r="B35">
-        <v>2024</v>
-      </c>
-      <c r="C35">
-        <v>1.1780479999999999E-2</v>
-      </c>
-      <c r="D35">
-        <v>1.9272741999999999E-2</v>
-      </c>
-      <c r="E35">
-        <v>1.5526610999999999E-2</v>
-      </c>
-      <c r="F35">
-        <v>1.5526610999999999E-2</v>
-      </c>
-      <c r="G35">
-        <v>1.9272741999999999E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>313</v>
-      </c>
-      <c r="B36">
-        <v>2025</v>
-      </c>
-      <c r="C36">
-        <v>1.4880427E-2</v>
-      </c>
-      <c r="D36">
-        <v>2.4774272999999999E-2</v>
-      </c>
-      <c r="E36">
-        <v>1.9827350000000001E-2</v>
-      </c>
-      <c r="F36">
-        <v>1.9827350000000001E-2</v>
-      </c>
-      <c r="G36">
-        <v>2.4774272999999999E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>313</v>
-      </c>
-      <c r="B37">
-        <v>2026</v>
-      </c>
-      <c r="C37">
-        <v>1.7896786000000001E-2</v>
-      </c>
-      <c r="D37">
-        <v>3.7774355000000003E-2</v>
-      </c>
-      <c r="E37">
-        <v>2.783557E-2</v>
-      </c>
-      <c r="F37">
-        <v>2.783557E-2</v>
-      </c>
-      <c r="G37">
-        <v>3.7774355000000003E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>313</v>
-      </c>
-      <c r="B38">
-        <v>2027</v>
-      </c>
-      <c r="C38">
-        <v>2.0805857000000001E-2</v>
-      </c>
-      <c r="D38">
-        <v>5.7356055000000003E-2</v>
-      </c>
-      <c r="E38">
-        <v>3.9080956E-2</v>
-      </c>
-      <c r="F38">
-        <v>3.9080956E-2</v>
-      </c>
-      <c r="G38">
-        <v>5.7356055000000003E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>313</v>
-      </c>
-      <c r="B39">
-        <v>2028</v>
-      </c>
-      <c r="C39">
-        <v>2.3611013E-2</v>
-      </c>
-      <c r="D39">
-        <v>8.4760910999999994E-2</v>
-      </c>
-      <c r="E39">
-        <v>5.4185961999999997E-2</v>
-      </c>
-      <c r="F39">
-        <v>5.4185961999999997E-2</v>
-      </c>
-      <c r="G39">
-        <v>8.4760910999999994E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>313</v>
-      </c>
-      <c r="B40">
-        <v>2029</v>
-      </c>
-      <c r="C40">
-        <v>2.6362935000000001E-2</v>
-      </c>
-      <c r="D40">
-        <v>0.110267067</v>
-      </c>
-      <c r="E40">
-        <v>6.8315001E-2</v>
-      </c>
-      <c r="F40">
-        <v>6.8315001E-2</v>
-      </c>
-      <c r="G40">
-        <v>0.110267067</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>313</v>
-      </c>
-      <c r="B41">
-        <v>2030</v>
-      </c>
-      <c r="C41">
-        <v>2.9098506E-2</v>
-      </c>
-      <c r="D41">
-        <v>0.13976050100000001</v>
-      </c>
-      <c r="E41">
-        <v>8.4429504000000002E-2</v>
-      </c>
-      <c r="F41">
-        <v>8.4429504000000002E-2</v>
-      </c>
-      <c r="G41">
-        <v>0.13976050100000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>313</v>
-      </c>
-      <c r="B42">
-        <v>2031</v>
-      </c>
-      <c r="C42">
-        <v>3.1850912000000002E-2</v>
-      </c>
-      <c r="D42">
-        <v>0.16977555799999999</v>
-      </c>
-      <c r="E42">
-        <v>0.100813235</v>
-      </c>
-      <c r="F42">
-        <v>0.100813235</v>
-      </c>
-      <c r="G42">
-        <v>0.16977555799999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>313</v>
-      </c>
-      <c r="B43">
-        <v>2032</v>
-      </c>
-      <c r="C43">
-        <v>3.4619206E-2</v>
-      </c>
-      <c r="D43">
-        <v>0.20474008699999999</v>
-      </c>
-      <c r="E43">
-        <v>0.119679647</v>
-      </c>
-      <c r="F43">
-        <v>0.119679647</v>
-      </c>
-      <c r="G43">
-        <v>0.20474008699999999</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>313</v>
-      </c>
-      <c r="B44">
-        <v>2033</v>
-      </c>
-      <c r="C44">
-        <v>3.7401094000000003E-2</v>
-      </c>
-      <c r="D44">
-        <v>0.24537620900000001</v>
-      </c>
-      <c r="E44">
-        <v>0.141388651</v>
-      </c>
-      <c r="F44">
-        <v>0.141388651</v>
-      </c>
-      <c r="G44">
-        <v>0.24537620900000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>313</v>
-      </c>
-      <c r="B45">
-        <v>2034</v>
-      </c>
-      <c r="C45">
-        <v>4.0196467999999999E-2</v>
-      </c>
-      <c r="D45">
-        <v>0.292219018</v>
-      </c>
-      <c r="E45">
-        <v>0.16620774299999999</v>
-      </c>
-      <c r="F45">
-        <v>0.16620774299999999</v>
-      </c>
-      <c r="G45">
-        <v>0.292219018</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>313</v>
-      </c>
-      <c r="B46">
-        <v>2035</v>
-      </c>
-      <c r="C46">
-        <v>4.2987719000000001E-2</v>
-      </c>
-      <c r="D46">
-        <v>0.34549044600000001</v>
-      </c>
-      <c r="E46">
-        <v>0.19423908200000001</v>
-      </c>
-      <c r="F46">
-        <v>0.19423908200000001</v>
-      </c>
-      <c r="G46">
-        <v>0.34549044600000001</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>313</v>
-      </c>
-      <c r="B47">
-        <v>2036</v>
-      </c>
-      <c r="C47">
-        <v>4.5770973E-2</v>
-      </c>
-      <c r="D47">
-        <v>0.39619227099999998</v>
-      </c>
-      <c r="E47">
-        <v>0.22098162199999999</v>
-      </c>
-      <c r="F47">
-        <v>0.22098162199999999</v>
-      </c>
-      <c r="G47">
-        <v>0.39619227099999998</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>313</v>
-      </c>
-      <c r="B48">
-        <v>2037</v>
-      </c>
-      <c r="C48">
-        <v>4.8543924000000002E-2</v>
-      </c>
-      <c r="D48">
-        <v>0.444968113</v>
-      </c>
-      <c r="E48">
-        <v>0.24675601899999999</v>
-      </c>
-      <c r="F48">
-        <v>0.24675601899999999</v>
-      </c>
-      <c r="G48">
-        <v>0.444968113</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>313</v>
-      </c>
-      <c r="B49">
-        <v>2038</v>
-      </c>
-      <c r="C49">
-        <v>5.1304790000000003E-2</v>
-      </c>
-      <c r="D49">
-        <v>0.49169161900000002</v>
-      </c>
-      <c r="E49">
-        <v>0.27149820400000002</v>
-      </c>
-      <c r="F49">
-        <v>0.27149820400000002</v>
-      </c>
-      <c r="G49">
-        <v>0.49169161900000002</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>313</v>
-      </c>
-      <c r="B50">
-        <v>2039</v>
-      </c>
-      <c r="C50">
-        <v>5.40186E-2</v>
-      </c>
-      <c r="D50">
-        <v>0.53644918200000002</v>
-      </c>
-      <c r="E50">
-        <v>0.29523389100000003</v>
-      </c>
-      <c r="F50">
-        <v>0.29523389100000003</v>
-      </c>
-      <c r="G50">
-        <v>0.53644918200000002</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>313</v>
-      </c>
-      <c r="B51">
-        <v>2040</v>
-      </c>
-      <c r="C51">
-        <v>5.6696666E-2</v>
-      </c>
-      <c r="D51">
-        <v>0.57897244699999995</v>
-      </c>
-      <c r="E51">
-        <v>0.31783455599999999</v>
-      </c>
-      <c r="F51">
-        <v>0.31783455599999999</v>
-      </c>
-      <c r="G51">
-        <v>0.57897244699999995</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>313</v>
-      </c>
-      <c r="B52">
-        <v>2041</v>
-      </c>
-      <c r="C52">
-        <v>5.9316059999999997E-2</v>
-      </c>
-      <c r="D52">
-        <v>0.61912640799999996</v>
-      </c>
-      <c r="E52">
-        <v>0.33922123399999998</v>
-      </c>
-      <c r="F52">
-        <v>0.33922123399999998</v>
-      </c>
-      <c r="G52">
-        <v>0.61912640799999996</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>313</v>
-      </c>
-      <c r="B53">
-        <v>2042</v>
-      </c>
-      <c r="C53">
-        <v>6.1865734999999998E-2</v>
-      </c>
-      <c r="D53">
-        <v>0.657095557</v>
-      </c>
-      <c r="E53">
-        <v>0.35948064600000001</v>
-      </c>
-      <c r="F53">
-        <v>0.35948064600000001</v>
-      </c>
-      <c r="G53">
-        <v>0.657095557</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>313</v>
-      </c>
-      <c r="B54">
-        <v>2043</v>
-      </c>
-      <c r="C54">
-        <v>6.4368699000000001E-2</v>
-      </c>
-      <c r="D54">
-        <v>0.69262306100000004</v>
-      </c>
-      <c r="E54">
-        <v>0.37849588000000001</v>
-      </c>
-      <c r="F54">
-        <v>0.37849588000000001</v>
-      </c>
-      <c r="G54">
-        <v>0.69262306100000004</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>313</v>
-      </c>
-      <c r="B55">
-        <v>2044</v>
-      </c>
-      <c r="C55">
-        <v>6.6828560999999995E-2</v>
-      </c>
-      <c r="D55">
-        <v>0.72576428699999995</v>
-      </c>
-      <c r="E55">
-        <v>0.39629642399999998</v>
-      </c>
-      <c r="F55">
-        <v>0.39629642399999998</v>
-      </c>
-      <c r="G55">
-        <v>0.72576428699999995</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>313</v>
-      </c>
-      <c r="B56">
-        <v>2045</v>
-      </c>
-      <c r="C56">
-        <v>6.9255160999999996E-2</v>
-      </c>
-      <c r="D56">
-        <v>0.75643987199999996</v>
-      </c>
-      <c r="E56">
-        <v>0.41284751600000003</v>
-      </c>
-      <c r="F56">
-        <v>0.41284751600000003</v>
-      </c>
-      <c r="G56">
-        <v>0.75643987199999996</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>313</v>
-      </c>
-      <c r="B57">
-        <v>2046</v>
-      </c>
-      <c r="C57">
-        <v>7.1660583E-2</v>
-      </c>
-      <c r="D57">
-        <v>0.78459593599999999</v>
-      </c>
-      <c r="E57">
-        <v>0.42812825900000001</v>
-      </c>
-      <c r="F57">
-        <v>0.42812825900000001</v>
-      </c>
-      <c r="G57">
-        <v>0.78459593599999999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>313</v>
-      </c>
-      <c r="B58">
-        <v>2047</v>
-      </c>
-      <c r="C58">
-        <v>7.4023167000000001E-2</v>
-      </c>
-      <c r="D58">
-        <v>0.81016510900000005</v>
-      </c>
-      <c r="E58">
-        <v>0.44209413800000003</v>
-      </c>
-      <c r="F58">
-        <v>0.44209413800000003</v>
-      </c>
-      <c r="G58">
-        <v>0.81016510900000005</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>313</v>
-      </c>
-      <c r="B59">
-        <v>2048</v>
-      </c>
-      <c r="C59">
-        <v>7.6331019E-2</v>
-      </c>
-      <c r="D59">
-        <v>0.83324370199999997</v>
-      </c>
-      <c r="E59">
-        <v>0.454787361</v>
-      </c>
-      <c r="F59">
-        <v>0.454787361</v>
-      </c>
-      <c r="G59">
-        <v>0.83324370199999997</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>313</v>
-      </c>
-      <c r="B60">
-        <v>2049</v>
-      </c>
-      <c r="C60">
-        <v>7.8599206000000005E-2</v>
-      </c>
-      <c r="D60">
-        <v>0.85401336000000005</v>
-      </c>
-      <c r="E60">
-        <v>0.46630628299999999</v>
-      </c>
-      <c r="F60">
-        <v>0.46630628299999999</v>
-      </c>
-      <c r="G60">
-        <v>0.85401336000000005</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>313</v>
-      </c>
-      <c r="B61">
-        <v>2050</v>
-      </c>
-      <c r="C61">
-        <v>8.0826548999999998E-2</v>
-      </c>
-      <c r="D61">
-        <v>0.87233277799999998</v>
-      </c>
-      <c r="E61">
-        <v>0.47657966400000001</v>
-      </c>
-      <c r="F61">
-        <v>0.47657966400000001</v>
-      </c>
-      <c r="G61">
-        <v>0.87233277799999998</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>314</v>
-      </c>
-      <c r="B62">
-        <v>2021</v>
-      </c>
-      <c r="C62">
-        <v>2.69208E-4</v>
-      </c>
-      <c r="D62">
-        <v>2.69208E-4</v>
-      </c>
-      <c r="E62">
-        <v>2.69208E-4</v>
-      </c>
-      <c r="F62">
-        <v>2.69208E-4</v>
-      </c>
-      <c r="G62">
-        <v>2.69208E-4</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>314</v>
-      </c>
-      <c r="B63">
-        <v>2022</v>
-      </c>
-      <c r="C63">
-        <v>5.1113500000000002E-4</v>
-      </c>
-      <c r="D63">
-        <v>5.1113500000000002E-4</v>
-      </c>
-      <c r="E63">
-        <v>5.1113500000000002E-4</v>
-      </c>
-      <c r="F63">
-        <v>5.1113500000000002E-4</v>
-      </c>
-      <c r="G63">
-        <v>5.1113500000000002E-4</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>314</v>
-      </c>
-      <c r="B64">
-        <v>2023</v>
-      </c>
-      <c r="C64">
-        <v>7.5173000000000004E-4</v>
-      </c>
-      <c r="D64">
-        <v>7.5173000000000004E-4</v>
-      </c>
-      <c r="E64">
-        <v>7.5173000000000004E-4</v>
-      </c>
-      <c r="F64">
-        <v>7.5173000000000004E-4</v>
-      </c>
-      <c r="G64">
-        <v>7.5173000000000004E-4</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>314</v>
-      </c>
-      <c r="B65">
-        <v>2024</v>
-      </c>
-      <c r="C65">
-        <v>9.8721599999999996E-4</v>
-      </c>
-      <c r="D65">
-        <v>9.8721599999999996E-4</v>
-      </c>
-      <c r="E65">
-        <v>9.8721599999999996E-4</v>
-      </c>
-      <c r="F65">
-        <v>2.2232290000000002E-3</v>
-      </c>
-      <c r="G65">
-        <v>2.2232290000000002E-3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>314</v>
-      </c>
-      <c r="B66">
-        <v>2025</v>
-      </c>
-      <c r="C66">
-        <v>1.2173970000000001E-3</v>
-      </c>
-      <c r="D66">
-        <v>1.2173970000000001E-3</v>
-      </c>
-      <c r="E66">
-        <v>1.2173970000000001E-3</v>
-      </c>
-      <c r="F66">
-        <v>6.3453590000000001E-3</v>
-      </c>
-      <c r="G66">
-        <v>6.3453590000000001E-3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>314</v>
-      </c>
-      <c r="B67">
-        <v>2026</v>
-      </c>
-      <c r="C67">
-        <v>1.4441510000000001E-3</v>
-      </c>
-      <c r="D67">
-        <v>1.4441510000000001E-3</v>
-      </c>
-      <c r="E67">
-        <v>1.4441510000000001E-3</v>
-      </c>
-      <c r="F67">
-        <v>1.1845461999999999E-2</v>
-      </c>
-      <c r="G67">
-        <v>1.1845461999999999E-2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>314</v>
-      </c>
-      <c r="B68">
-        <v>2027</v>
-      </c>
-      <c r="C68">
-        <v>1.664706E-3</v>
-      </c>
-      <c r="D68">
-        <v>1.664706E-3</v>
-      </c>
-      <c r="E68">
-        <v>1.664706E-3</v>
-      </c>
-      <c r="F68">
-        <v>1.9948430999999999E-2</v>
-      </c>
-      <c r="G68">
-        <v>1.9948430999999999E-2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>314</v>
-      </c>
-      <c r="B69">
-        <v>2028</v>
-      </c>
-      <c r="C69">
-        <v>1.879225E-3</v>
-      </c>
-      <c r="D69">
-        <v>1.879225E-3</v>
-      </c>
-      <c r="E69">
-        <v>1.879225E-3</v>
-      </c>
-      <c r="F69">
-        <v>3.1568299000000001E-2</v>
-      </c>
-      <c r="G69">
-        <v>3.1568299000000001E-2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>314</v>
-      </c>
-      <c r="B70">
-        <v>2029</v>
-      </c>
-      <c r="C70">
-        <v>2.0915529999999999E-3</v>
-      </c>
-      <c r="D70">
-        <v>2.0915529999999999E-3</v>
-      </c>
-      <c r="E70">
-        <v>2.0915529999999999E-3</v>
-      </c>
-      <c r="F70">
-        <v>4.6924004999999998E-2</v>
-      </c>
-      <c r="G70">
-        <v>4.6924004999999998E-2</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>314</v>
-      </c>
-      <c r="B71">
-        <v>2030</v>
-      </c>
-      <c r="C71">
-        <v>2.3018520000000001E-3</v>
-      </c>
-      <c r="D71">
-        <v>2.3018520000000001E-3</v>
-      </c>
-      <c r="E71">
-        <v>2.3018520000000001E-3</v>
-      </c>
-      <c r="F71">
-        <v>6.5785700000000003E-2</v>
-      </c>
-      <c r="G71">
-        <v>6.5785700000000003E-2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>314</v>
-      </c>
-      <c r="B72">
-        <v>2031</v>
-      </c>
-      <c r="C72">
-        <v>2.5109339999999998E-3</v>
-      </c>
-      <c r="D72">
-        <v>2.5109339999999998E-3</v>
-      </c>
-      <c r="E72">
-        <v>2.5109339999999998E-3</v>
-      </c>
-      <c r="F72">
-        <v>8.8363822999999994E-2</v>
-      </c>
-      <c r="G72">
-        <v>8.8363822999999994E-2</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>314</v>
-      </c>
-      <c r="B73">
-        <v>2032</v>
-      </c>
-      <c r="C73">
-        <v>2.7175649999999999E-3</v>
-      </c>
-      <c r="D73">
-        <v>2.7175649999999999E-3</v>
-      </c>
-      <c r="E73">
-        <v>2.7175649999999999E-3</v>
-      </c>
-      <c r="F73">
-        <v>0.112572854</v>
-      </c>
-      <c r="G73">
-        <v>0.112572854</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>314</v>
-      </c>
-      <c r="B74">
-        <v>2033</v>
-      </c>
-      <c r="C74">
-        <v>2.927851E-3</v>
-      </c>
-      <c r="D74">
-        <v>2.927851E-3</v>
-      </c>
-      <c r="E74">
-        <v>2.927851E-3</v>
-      </c>
-      <c r="F74">
-        <v>0.13861931199999999</v>
-      </c>
-      <c r="G74">
-        <v>0.13861931199999999</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>314</v>
-      </c>
-      <c r="B75">
-        <v>2034</v>
-      </c>
-      <c r="C75">
-        <v>3.1403939999999999E-3</v>
-      </c>
-      <c r="D75">
-        <v>3.1403939999999999E-3</v>
-      </c>
-      <c r="E75">
-        <v>3.1403939999999999E-3</v>
-      </c>
-      <c r="F75">
-        <v>0.16646481900000001</v>
-      </c>
-      <c r="G75">
-        <v>0.16646481900000001</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>314</v>
-      </c>
-      <c r="B76">
-        <v>2035</v>
-      </c>
-      <c r="C76">
-        <v>3.3537770000000001E-3</v>
-      </c>
-      <c r="D76">
-        <v>3.3537770000000001E-3</v>
-      </c>
-      <c r="E76">
-        <v>3.3537770000000001E-3</v>
-      </c>
-      <c r="F76">
-        <v>0.19560739399999999</v>
-      </c>
-      <c r="G76">
-        <v>0.19560739399999999</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>314</v>
-      </c>
-      <c r="B77">
-        <v>2036</v>
-      </c>
-      <c r="C77">
-        <v>3.5669400000000002E-3</v>
-      </c>
-      <c r="D77">
-        <v>3.5669400000000002E-3</v>
-      </c>
-      <c r="E77">
-        <v>3.5669400000000002E-3</v>
-      </c>
-      <c r="F77">
-        <v>0.224213724</v>
-      </c>
-      <c r="G77">
-        <v>0.224213724</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>314</v>
-      </c>
-      <c r="B78">
-        <v>2037</v>
-      </c>
-      <c r="C78">
-        <v>3.7814290000000002E-3</v>
-      </c>
-      <c r="D78">
-        <v>3.7814290000000002E-3</v>
-      </c>
-      <c r="E78">
-        <v>3.7814290000000002E-3</v>
-      </c>
-      <c r="F78">
-        <v>0.251758013</v>
-      </c>
-      <c r="G78">
-        <v>0.251758013</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>314</v>
-      </c>
-      <c r="B79">
-        <v>2038</v>
-      </c>
-      <c r="C79">
-        <v>3.9981180000000002E-3</v>
-      </c>
-      <c r="D79">
-        <v>3.9981180000000002E-3</v>
-      </c>
-      <c r="E79">
-        <v>3.9981180000000002E-3</v>
-      </c>
-      <c r="F79">
-        <v>0.27830375000000002</v>
-      </c>
-      <c r="G79">
-        <v>0.27830375000000002</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>314</v>
-      </c>
-      <c r="B80">
-        <v>2039</v>
-      </c>
-      <c r="C80">
-        <v>4.2198260000000003E-3</v>
-      </c>
-      <c r="D80">
-        <v>4.2198260000000003E-3</v>
-      </c>
-      <c r="E80">
-        <v>4.2198260000000003E-3</v>
-      </c>
-      <c r="F80">
-        <v>0.30357849199999998</v>
-      </c>
-      <c r="G80">
-        <v>0.30357849199999998</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>314</v>
-      </c>
-      <c r="B81">
-        <v>2040</v>
-      </c>
-      <c r="C81">
-        <v>4.448624E-3</v>
-      </c>
-      <c r="D81">
-        <v>4.448624E-3</v>
-      </c>
-      <c r="E81">
-        <v>4.448624E-3</v>
-      </c>
-      <c r="F81">
-        <v>0.32763684900000001</v>
-      </c>
-      <c r="G81">
-        <v>0.32763684900000001</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>314</v>
-      </c>
-      <c r="B82">
-        <v>2041</v>
-      </c>
-      <c r="C82">
-        <v>4.678415E-3</v>
-      </c>
-      <c r="D82">
-        <v>4.678415E-3</v>
-      </c>
-      <c r="E82">
-        <v>4.678415E-3</v>
-      </c>
-      <c r="F82">
-        <v>0.35042086</v>
-      </c>
-      <c r="G82">
-        <v>0.35042086</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>314</v>
-      </c>
-      <c r="B83">
-        <v>2042</v>
-      </c>
-      <c r="C83">
-        <v>4.910925E-3</v>
-      </c>
-      <c r="D83">
-        <v>4.910925E-3</v>
-      </c>
-      <c r="E83">
-        <v>4.910925E-3</v>
-      </c>
-      <c r="F83">
-        <v>0.371888357</v>
-      </c>
-      <c r="G83">
-        <v>0.371888357</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>314</v>
-      </c>
-      <c r="B84">
-        <v>2043</v>
-      </c>
-      <c r="C84">
-        <v>5.1371760000000002E-3</v>
-      </c>
-      <c r="D84">
-        <v>5.1371760000000002E-3</v>
-      </c>
-      <c r="E84">
-        <v>5.1371760000000002E-3</v>
-      </c>
-      <c r="F84">
-        <v>0.39163393099999999</v>
-      </c>
-      <c r="G84">
-        <v>0.39163393099999999</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>314</v>
-      </c>
-      <c r="B85">
-        <v>2044</v>
-      </c>
-      <c r="C85">
-        <v>5.3573889999999997E-3</v>
-      </c>
-      <c r="D85">
-        <v>5.3573889999999997E-3</v>
-      </c>
-      <c r="E85">
-        <v>5.3573889999999997E-3</v>
-      </c>
-      <c r="F85">
-        <v>0.41053531700000001</v>
-      </c>
-      <c r="G85">
-        <v>0.41053531700000001</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
-        <v>314</v>
-      </c>
-      <c r="B86">
-        <v>2045</v>
-      </c>
-      <c r="C86">
-        <v>5.5812450000000003E-3</v>
-      </c>
-      <c r="D86">
-        <v>5.5812450000000003E-3</v>
-      </c>
-      <c r="E86">
-        <v>5.5812450000000003E-3</v>
-      </c>
-      <c r="F86">
-        <v>0.427685765</v>
-      </c>
-      <c r="G86">
-        <v>0.427685765</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
-        <v>314</v>
-      </c>
-      <c r="B87">
-        <v>2046</v>
-      </c>
-      <c r="C87">
-        <v>5.811709E-3</v>
-      </c>
-      <c r="D87">
-        <v>5.811709E-3</v>
-      </c>
-      <c r="E87">
-        <v>5.811709E-3</v>
-      </c>
-      <c r="F87">
-        <v>0.443591191</v>
-      </c>
-      <c r="G87">
-        <v>0.443591191</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
-        <v>314</v>
-      </c>
-      <c r="B88">
-        <v>2047</v>
-      </c>
-      <c r="C88">
-        <v>6.0421320000000004E-3</v>
-      </c>
-      <c r="D88">
-        <v>6.0421320000000004E-3</v>
-      </c>
-      <c r="E88">
-        <v>6.0421320000000004E-3</v>
-      </c>
-      <c r="F88">
-        <v>0.45792830099999998</v>
-      </c>
-      <c r="G88">
-        <v>0.45792830099999998</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
-        <v>314</v>
-      </c>
-      <c r="B89">
-        <v>2048</v>
-      </c>
-      <c r="C89">
-        <v>6.2732539999999998E-3</v>
-      </c>
-      <c r="D89">
-        <v>6.2732539999999998E-3</v>
-      </c>
-      <c r="E89">
-        <v>6.2732539999999998E-3</v>
-      </c>
-      <c r="F89">
-        <v>0.47101606299999998</v>
-      </c>
-      <c r="G89">
-        <v>0.47101606299999998</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
-        <v>314</v>
-      </c>
-      <c r="B90">
-        <v>2049</v>
-      </c>
-      <c r="C90">
-        <v>6.5150909999999998E-3</v>
-      </c>
-      <c r="D90">
-        <v>6.5150909999999998E-3</v>
-      </c>
-      <c r="E90">
-        <v>6.5150909999999998E-3</v>
-      </c>
-      <c r="F90">
-        <v>0.48289326799999999</v>
-      </c>
-      <c r="G90">
-        <v>0.48289326799999999</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
-        <v>314</v>
-      </c>
-      <c r="B91">
-        <v>2050</v>
-      </c>
-      <c r="C91">
-        <v>6.767019E-3</v>
-      </c>
-      <c r="D91">
-        <v>6.767019E-3</v>
-      </c>
-      <c r="E91">
-        <v>6.767019E-3</v>
-      </c>
-      <c r="F91">
-        <v>0.49398055200000002</v>
-      </c>
-      <c r="G91">
-        <v>0.49398055200000002</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
-        <v>315</v>
-      </c>
-      <c r="B92">
-        <v>2021</v>
-      </c>
-      <c r="C92">
-        <v>1.2819571E-2</v>
-      </c>
-      <c r="D92">
-        <v>1.2819571E-2</v>
-      </c>
-      <c r="E92">
-        <v>1.2819571E-2</v>
-      </c>
-      <c r="F92">
-        <v>1.2819571E-2</v>
-      </c>
-      <c r="G92">
-        <v>1.2819571E-2</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
-        <v>315</v>
-      </c>
-      <c r="B93">
-        <v>2022</v>
-      </c>
-      <c r="C93">
-        <v>1.4978317E-2</v>
-      </c>
-      <c r="D93">
-        <v>3.2432076999999997E-2</v>
-      </c>
-      <c r="E93">
-        <v>2.3705197000000001E-2</v>
-      </c>
-      <c r="F93">
-        <v>2.3705197000000001E-2</v>
-      </c>
-      <c r="G93">
-        <v>3.2432076999999997E-2</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
-        <v>315</v>
-      </c>
-      <c r="B94">
-        <v>2023</v>
-      </c>
-      <c r="C94">
-        <v>1.7291666000000001E-2</v>
-      </c>
-      <c r="D94">
-        <v>5.2044582999999998E-2</v>
-      </c>
-      <c r="E94">
-        <v>3.4668124000000002E-2</v>
-      </c>
-      <c r="F94">
-        <v>3.4668124000000002E-2</v>
-      </c>
-      <c r="G94">
-        <v>5.2044582999999998E-2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
-        <v>315</v>
-      </c>
-      <c r="B95">
-        <v>2024</v>
-      </c>
-      <c r="C95">
-        <v>1.9724051999999999E-2</v>
-      </c>
-      <c r="D95">
-        <v>7.1657088999999993E-2</v>
-      </c>
-      <c r="E95">
-        <v>4.5690570999999999E-2</v>
-      </c>
-      <c r="F95">
-        <v>4.5690570999999999E-2</v>
-      </c>
-      <c r="G95">
-        <v>7.1657088999999993E-2</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
-        <v>315</v>
-      </c>
-      <c r="B96">
-        <v>2025</v>
-      </c>
-      <c r="C96">
-        <v>2.2165526000000001E-2</v>
-      </c>
-      <c r="D96">
-        <v>9.1269594999999995E-2</v>
-      </c>
-      <c r="E96">
-        <v>5.671756E-2</v>
-      </c>
-      <c r="F96">
-        <v>5.671756E-2</v>
-      </c>
-      <c r="G96">
-        <v>9.1269594999999995E-2</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
-        <v>315</v>
-      </c>
-      <c r="B97">
-        <v>2026</v>
-      </c>
-      <c r="C97">
-        <v>2.4657855999999999E-2</v>
-      </c>
-      <c r="D97">
-        <v>0.12079788800000001</v>
-      </c>
-      <c r="E97">
-        <v>7.2727871999999999E-2</v>
-      </c>
-      <c r="F97">
-        <v>7.2727871999999999E-2</v>
-      </c>
-      <c r="G97">
-        <v>0.12079788800000001</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
-        <v>315</v>
-      </c>
-      <c r="B98">
-        <v>2027</v>
-      </c>
-      <c r="C98">
-        <v>2.7184686999999999E-2</v>
-      </c>
-      <c r="D98">
-        <v>0.151904497</v>
-      </c>
-      <c r="E98">
-        <v>8.9544592000000006E-2</v>
-      </c>
-      <c r="F98">
-        <v>8.9544592000000006E-2</v>
-      </c>
-      <c r="G98">
-        <v>0.151904497</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>315</v>
-      </c>
-      <c r="B99">
-        <v>2028</v>
-      </c>
-      <c r="C99">
-        <v>2.9742540000000001E-2</v>
-      </c>
-      <c r="D99">
-        <v>0.18432768499999999</v>
-      </c>
-      <c r="E99">
-        <v>0.107035112</v>
-      </c>
-      <c r="F99">
-        <v>0.107035112</v>
-      </c>
-      <c r="G99">
-        <v>0.18432768499999999</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
-        <v>315</v>
-      </c>
-      <c r="B100">
-        <v>2029</v>
-      </c>
-      <c r="C100">
-        <v>3.2380491999999997E-2</v>
-      </c>
-      <c r="D100">
-        <v>0.22622346600000001</v>
-      </c>
-      <c r="E100">
-        <v>0.12930197900000001</v>
-      </c>
-      <c r="F100">
-        <v>0.12930197900000001</v>
-      </c>
-      <c r="G100">
-        <v>0.22622346600000001</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
-        <v>315</v>
-      </c>
-      <c r="B101">
-        <v>2030</v>
-      </c>
-      <c r="C101">
-        <v>3.5179580000000002E-2</v>
-      </c>
-      <c r="D101">
-        <v>0.27353129100000001</v>
-      </c>
-      <c r="E101">
-        <v>0.15435543600000001</v>
-      </c>
-      <c r="F101">
-        <v>0.15435543600000001</v>
-      </c>
-      <c r="G101">
-        <v>0.27353129100000001</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
-        <v>315</v>
-      </c>
-      <c r="B102">
-        <v>2031</v>
-      </c>
-      <c r="C102">
-        <v>3.8168565000000002E-2</v>
-      </c>
-      <c r="D102">
-        <v>0.32771400000000001</v>
-      </c>
-      <c r="E102">
-        <v>0.18294128300000001</v>
-      </c>
-      <c r="F102">
-        <v>0.18294128300000001</v>
-      </c>
-      <c r="G102">
-        <v>0.32771400000000001</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
-        <v>315</v>
-      </c>
-      <c r="B103">
-        <v>2032</v>
-      </c>
-      <c r="C103">
-        <v>4.1333373999999999E-2</v>
-      </c>
-      <c r="D103">
-        <v>0.38171043300000002</v>
-      </c>
-      <c r="E103">
-        <v>0.21152190400000001</v>
-      </c>
-      <c r="F103">
-        <v>0.21152190400000001</v>
-      </c>
-      <c r="G103">
-        <v>0.38171043300000002</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>315</v>
-      </c>
-      <c r="B104">
-        <v>2033</v>
-      </c>
-      <c r="C104">
-        <v>4.4657994999999999E-2</v>
-      </c>
-      <c r="D104">
-        <v>0.43484204300000001</v>
-      </c>
-      <c r="E104">
-        <v>0.23975001900000001</v>
-      </c>
-      <c r="F104">
-        <v>0.23975001900000001</v>
-      </c>
-      <c r="G104">
-        <v>0.43484204300000001</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>315</v>
-      </c>
-      <c r="B105">
-        <v>2034</v>
-      </c>
-      <c r="C105">
-        <v>4.8126879999999997E-2</v>
-      </c>
-      <c r="D105">
-        <v>0.48654755500000002</v>
-      </c>
-      <c r="E105">
-        <v>0.26733721799999999</v>
-      </c>
-      <c r="F105">
-        <v>0.26733721799999999</v>
-      </c>
-      <c r="G105">
-        <v>0.48654755500000002</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
-        <v>315</v>
-      </c>
-      <c r="B106">
-        <v>2035</v>
-      </c>
-      <c r="C106">
-        <v>5.1706859000000001E-2</v>
-      </c>
-      <c r="D106">
-        <v>0.53597180700000002</v>
-      </c>
-      <c r="E106">
-        <v>0.29383933299999998</v>
-      </c>
-      <c r="F106">
-        <v>0.29383933299999998</v>
-      </c>
-      <c r="G106">
-        <v>0.53597180700000002</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
-        <v>315</v>
-      </c>
-      <c r="B107">
-        <v>2036</v>
-      </c>
-      <c r="C107">
-        <v>5.5368675999999999E-2</v>
-      </c>
-      <c r="D107">
-        <v>0.58298080299999999</v>
-      </c>
-      <c r="E107">
-        <v>0.31917473899999999</v>
-      </c>
-      <c r="F107">
-        <v>0.31917473899999999</v>
-      </c>
-      <c r="G107">
-        <v>0.58298080299999999</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
-        <v>315</v>
-      </c>
-      <c r="B108">
-        <v>2037</v>
-      </c>
-      <c r="C108">
-        <v>5.9080055999999999E-2</v>
-      </c>
-      <c r="D108">
-        <v>0.62722744100000005</v>
-      </c>
-      <c r="E108">
-        <v>0.34315374799999998</v>
-      </c>
-      <c r="F108">
-        <v>0.34315374799999998</v>
-      </c>
-      <c r="G108">
-        <v>0.62722744100000005</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
-        <v>315</v>
-      </c>
-      <c r="B109">
-        <v>2038</v>
-      </c>
-      <c r="C109">
-        <v>6.2828703E-2</v>
-      </c>
-      <c r="D109">
-        <v>0.66866269899999997</v>
-      </c>
-      <c r="E109">
-        <v>0.36574570099999998</v>
-      </c>
-      <c r="F109">
-        <v>0.36574570099999998</v>
-      </c>
-      <c r="G109">
-        <v>0.66866269899999997</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
-        <v>315</v>
-      </c>
-      <c r="B110">
-        <v>2039</v>
-      </c>
-      <c r="C110">
-        <v>6.6573137000000004E-2</v>
-      </c>
-      <c r="D110">
-        <v>0.70719917499999996</v>
-      </c>
-      <c r="E110">
-        <v>0.38688615599999998</v>
-      </c>
-      <c r="F110">
-        <v>0.38688615599999998</v>
-      </c>
-      <c r="G110">
-        <v>0.70719917499999996</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
-        <v>315</v>
-      </c>
-      <c r="B111">
-        <v>2040</v>
-      </c>
-      <c r="C111">
-        <v>7.0318973000000007E-2</v>
-      </c>
-      <c r="D111">
-        <v>0.74286130100000003</v>
-      </c>
-      <c r="E111">
-        <v>0.40659013700000002</v>
-      </c>
-      <c r="F111">
-        <v>0.40659013700000002</v>
-      </c>
-      <c r="G111">
-        <v>0.74286130100000003</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
-        <v>315</v>
-      </c>
-      <c r="B112">
-        <v>2041</v>
-      </c>
-      <c r="C112">
-        <v>7.4044963000000005E-2</v>
-      </c>
-      <c r="D112">
-        <v>0.77541419899999997</v>
-      </c>
-      <c r="E112">
-        <v>0.42472958100000002</v>
-      </c>
-      <c r="F112">
-        <v>0.42472958100000002</v>
-      </c>
-      <c r="G112">
-        <v>0.77541419899999997</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
-        <v>315</v>
-      </c>
-      <c r="B113">
-        <v>2042</v>
-      </c>
-      <c r="C113">
-        <v>7.7742975000000006E-2</v>
-      </c>
-      <c r="D113">
-        <v>0.80508984299999997</v>
-      </c>
-      <c r="E113">
-        <v>0.44141640900000001</v>
-      </c>
-      <c r="F113">
-        <v>0.44141640900000001</v>
-      </c>
-      <c r="G113">
-        <v>0.80508984299999997</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A114" t="s">
-        <v>315</v>
-      </c>
-      <c r="B114">
-        <v>2043</v>
-      </c>
-      <c r="C114">
-        <v>8.1487271E-2</v>
-      </c>
-      <c r="D114">
-        <v>0.83183468400000005</v>
-      </c>
-      <c r="E114">
-        <v>0.456660978</v>
-      </c>
-      <c r="F114">
-        <v>0.456660978</v>
-      </c>
-      <c r="G114">
-        <v>0.83183468400000005</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A115" t="s">
-        <v>315</v>
-      </c>
-      <c r="B115">
-        <v>2044</v>
-      </c>
-      <c r="C115">
-        <v>8.5272758000000004E-2</v>
-      </c>
-      <c r="D115">
-        <v>0.85566570900000005</v>
-      </c>
-      <c r="E115">
-        <v>0.47046923400000001</v>
-      </c>
-      <c r="F115">
-        <v>0.47046923400000001</v>
-      </c>
-      <c r="G115">
-        <v>0.85566570900000005</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A116" t="s">
-        <v>315</v>
-      </c>
-      <c r="B116">
-        <v>2045</v>
-      </c>
-      <c r="C116">
-        <v>8.9111153999999998E-2</v>
-      </c>
-      <c r="D116">
-        <v>0.87680356800000003</v>
-      </c>
-      <c r="E116">
-        <v>0.48295736099999997</v>
-      </c>
-      <c r="F116">
-        <v>0.48295736099999997</v>
-      </c>
-      <c r="G116">
-        <v>0.87680356800000003</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A117" t="s">
-        <v>315</v>
-      </c>
-      <c r="B117">
-        <v>2046</v>
-      </c>
-      <c r="C117">
-        <v>9.3001159E-2</v>
-      </c>
-      <c r="D117">
-        <v>0.89522190400000001</v>
-      </c>
-      <c r="E117">
-        <v>0.49411153099999999</v>
-      </c>
-      <c r="F117">
-        <v>0.49411153099999999</v>
-      </c>
-      <c r="G117">
-        <v>0.89522190400000001</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A118" t="s">
-        <v>315</v>
-      </c>
-      <c r="B118">
-        <v>2047</v>
-      </c>
-      <c r="C118">
-        <v>9.6893360999999997E-2</v>
-      </c>
-      <c r="D118">
-        <v>0.91109814099999997</v>
-      </c>
-      <c r="E118">
-        <v>0.50399575100000005</v>
-      </c>
-      <c r="F118">
-        <v>0.50399575100000005</v>
-      </c>
-      <c r="G118">
-        <v>0.91109814099999997</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A119" t="s">
-        <v>315</v>
-      </c>
-      <c r="B119">
-        <v>2048</v>
-      </c>
-      <c r="C119">
-        <v>0.100758687</v>
-      </c>
-      <c r="D119">
-        <v>0.92468582899999996</v>
-      </c>
-      <c r="E119">
-        <v>0.51272225800000004</v>
-      </c>
-      <c r="F119">
-        <v>0.51272225800000004</v>
-      </c>
-      <c r="G119">
-        <v>0.92468582899999996</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A120" t="s">
-        <v>315</v>
-      </c>
-      <c r="B120">
-        <v>2049</v>
-      </c>
-      <c r="C120">
-        <v>0.104609438</v>
-      </c>
-      <c r="D120">
-        <v>0.93609858000000001</v>
-      </c>
-      <c r="E120">
-        <v>0.52035400899999995</v>
-      </c>
-      <c r="F120">
-        <v>0.52035400899999995</v>
-      </c>
-      <c r="G120">
-        <v>0.93609858000000001</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A121" t="s">
-        <v>315</v>
-      </c>
-      <c r="B121">
-        <v>2050</v>
-      </c>
-      <c r="C121">
-        <v>0.108448247</v>
-      </c>
-      <c r="D121">
-        <v>0.94575257999999995</v>
-      </c>
-      <c r="E121">
-        <v>0.52710000000000001</v>
-      </c>
-      <c r="F121">
-        <v>0.52710041399999996</v>
-      </c>
-      <c r="G121">
-        <v>0.94575257999999995</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C4DD4AF-DD0C-4218-BC59-541B179F4B4B}">
-  <dimension ref="A1:F52"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="3" max="3" width="14.6328125" customWidth="1"/>
-    <col min="4" max="4" width="19.90625" customWidth="1"/>
-    <col min="5" max="5" width="16.26953125" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>316</v>
-      </c>
-      <c r="D1" t="s">
-        <v>317</v>
-      </c>
-      <c r="E1" t="s">
-        <v>318</v>
-      </c>
-      <c r="F1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <v>2019</v>
-      </c>
-      <c r="C2">
-        <v>10150210</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>2019</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>2019</v>
-      </c>
-      <c r="C4">
-        <v>19763274</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>108918663</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>2019</v>
-      </c>
-      <c r="C5">
-        <v>6032563</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
-        <v>2019</v>
-      </c>
-      <c r="C6">
-        <v>2272320341</v>
-      </c>
-      <c r="D6">
-        <v>923680643</v>
-      </c>
-      <c r="E6">
-        <v>1964029505</v>
-      </c>
-      <c r="F6">
-        <v>931495117</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>2019</v>
-      </c>
-      <c r="C7">
-        <v>53601802</v>
-      </c>
-      <c r="D7">
-        <v>121331394</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>178266835</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>2019</v>
-      </c>
-      <c r="C8">
-        <v>362943581</v>
-      </c>
-      <c r="D8">
-        <v>16002355</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>2019</v>
-      </c>
-      <c r="C9">
-        <v>142291569</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10">
-        <v>2019</v>
-      </c>
-      <c r="C10">
-        <v>179525732</v>
-      </c>
-      <c r="D10">
-        <v>143756233</v>
-      </c>
-      <c r="E10">
-        <v>136546053</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11">
-        <v>2019</v>
-      </c>
-      <c r="C11">
-        <v>28108257</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>450023139</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>2019</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13">
-        <v>2019</v>
-      </c>
-      <c r="C13">
-        <v>1334134</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14">
-        <v>2019</v>
-      </c>
-      <c r="C14">
-        <v>936800351</v>
-      </c>
-      <c r="D14">
-        <v>1365137921</v>
-      </c>
-      <c r="E14">
-        <v>1378128437</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15">
-        <v>2019</v>
-      </c>
-      <c r="C15">
-        <v>23368372</v>
-      </c>
-      <c r="D15">
-        <v>108385897</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16">
-        <v>2019</v>
-      </c>
-      <c r="C16">
-        <v>10215072</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17">
-        <v>2019</v>
-      </c>
-      <c r="C17">
-        <v>9219926</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18">
-        <v>2019</v>
-      </c>
-      <c r="C18">
-        <v>1659634</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19">
-        <v>2019</v>
-      </c>
-      <c r="C19">
-        <v>34941975</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20">
-        <v>2019</v>
-      </c>
-      <c r="C20">
-        <v>66584121</v>
-      </c>
-      <c r="D20">
-        <v>44297074</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21">
-        <v>2019</v>
-      </c>
-      <c r="C21">
-        <v>403051904</v>
-      </c>
-      <c r="D21">
-        <v>271391388</v>
-      </c>
-      <c r="E21">
-        <v>32470539</v>
-      </c>
-      <c r="F21">
-        <v>39816955</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22">
-        <v>2019</v>
-      </c>
-      <c r="C22">
-        <v>686323124</v>
-      </c>
-      <c r="D22">
-        <v>653570994</v>
-      </c>
-      <c r="E22">
-        <v>572046325</v>
-      </c>
-      <c r="F22">
-        <v>137719112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23">
-        <v>2019</v>
-      </c>
-      <c r="C23">
-        <v>167317988</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24">
-        <v>2019</v>
-      </c>
-      <c r="C24">
-        <v>26177472</v>
-      </c>
-      <c r="D24">
-        <v>18965595</v>
-      </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-      <c r="F24">
-        <v>100499405</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25">
-        <v>2019</v>
-      </c>
-      <c r="C25">
-        <v>24330591</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26">
-        <v>2019</v>
-      </c>
-      <c r="C26">
-        <v>137330320</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <v>89068641</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27">
-        <v>2019</v>
-      </c>
-      <c r="C27">
-        <v>24070350</v>
-      </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28">
-        <v>2019</v>
-      </c>
-      <c r="C28">
-        <v>9853074</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29">
-        <v>2019</v>
-      </c>
-      <c r="C29">
-        <v>17645639</v>
-      </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-      <c r="E29">
-        <v>0</v>
-      </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30">
-        <v>2019</v>
-      </c>
-      <c r="C30">
-        <v>85722975</v>
-      </c>
-      <c r="D30">
-        <v>0</v>
-      </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31">
-        <v>2019</v>
-      </c>
-      <c r="C31">
-        <v>347590724</v>
-      </c>
-      <c r="D31">
-        <v>2006197776</v>
-      </c>
-      <c r="E31">
-        <v>546353547</v>
-      </c>
-      <c r="F31">
-        <v>73704102</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32">
-        <v>2019</v>
-      </c>
-      <c r="C32">
-        <v>23165058</v>
-      </c>
-      <c r="D32">
-        <v>35411192</v>
-      </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
-      <c r="F32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33">
-        <v>2019</v>
-      </c>
-      <c r="C33">
-        <v>2583207104</v>
-      </c>
-      <c r="D33">
-        <v>5964349570</v>
-      </c>
-      <c r="E33">
-        <v>10511005234</v>
-      </c>
-      <c r="F33">
-        <v>11971472</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>256</v>
-      </c>
-      <c r="B34">
-        <v>2019</v>
-      </c>
-      <c r="C34">
-        <v>184838466</v>
-      </c>
-      <c r="D34">
-        <v>0</v>
-      </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
-      <c r="F34">
-        <v>45024652</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>36</v>
-      </c>
-      <c r="B35">
-        <v>2019</v>
-      </c>
-      <c r="C35">
-        <v>20057435</v>
-      </c>
-      <c r="D35">
-        <v>0</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36">
-        <v>2019</v>
-      </c>
-      <c r="C36">
-        <v>26201671</v>
-      </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="E36">
-        <v>36529680</v>
-      </c>
-      <c r="F36">
-        <v>8974467</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37">
-        <v>2019</v>
-      </c>
-      <c r="C37">
-        <v>13968539</v>
-      </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38">
-        <v>2019</v>
-      </c>
-      <c r="C38">
-        <v>161077351</v>
-      </c>
-      <c r="D38">
-        <v>0</v>
-      </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <v>207967836</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>40</v>
-      </c>
-      <c r="B39">
-        <v>2019</v>
-      </c>
-      <c r="C39">
-        <v>1321007165</v>
-      </c>
-      <c r="D39">
-        <v>603541707</v>
-      </c>
-      <c r="E39">
-        <v>399537395</v>
-      </c>
-      <c r="F39">
-        <v>28888028</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>41</v>
-      </c>
-      <c r="B40">
-        <v>2019</v>
-      </c>
-      <c r="C40">
-        <v>195839815</v>
-      </c>
-      <c r="D40">
-        <v>0</v>
-      </c>
-      <c r="E40">
-        <v>0</v>
-      </c>
-      <c r="F40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>257</v>
-      </c>
-      <c r="B41">
-        <v>2019</v>
-      </c>
-      <c r="C41">
-        <v>35517998</v>
-      </c>
-      <c r="D41">
-        <v>0</v>
-      </c>
-      <c r="E41">
-        <v>0</v>
-      </c>
-      <c r="F41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42">
-        <v>2019</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42">
-        <v>0</v>
-      </c>
-      <c r="E42">
-        <v>0</v>
-      </c>
-      <c r="F42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43">
-        <v>2019</v>
-      </c>
-      <c r="C43">
-        <v>12774245</v>
-      </c>
-      <c r="D43">
-        <v>4544152</v>
-      </c>
-      <c r="E43">
-        <v>0</v>
-      </c>
-      <c r="F43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B44">
-        <v>2019</v>
-      </c>
-      <c r="C44">
-        <v>72175940</v>
-      </c>
-      <c r="D44">
-        <v>41940297</v>
-      </c>
-      <c r="E44">
-        <v>0</v>
-      </c>
-      <c r="F44">
-        <v>279333373</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>45</v>
-      </c>
-      <c r="B45">
-        <v>2019</v>
-      </c>
-      <c r="C45">
-        <v>11341330</v>
-      </c>
-      <c r="D45">
-        <v>133685517</v>
-      </c>
-      <c r="E45">
-        <v>0</v>
-      </c>
-      <c r="F45">
-        <v>83098538</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46">
-        <v>2019</v>
-      </c>
-      <c r="C46">
-        <v>18429934</v>
-      </c>
-      <c r="D46">
-        <v>0</v>
-      </c>
-      <c r="E46">
-        <v>0</v>
-      </c>
-      <c r="F46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>47</v>
-      </c>
-      <c r="B47">
-        <v>2019</v>
-      </c>
-      <c r="C47">
-        <v>306024295</v>
-      </c>
-      <c r="D47">
-        <v>135051068</v>
-      </c>
-      <c r="E47">
-        <v>0</v>
-      </c>
-      <c r="F47">
-        <v>4798117</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48">
-        <v>2019</v>
-      </c>
-      <c r="C48">
-        <v>258175574</v>
-      </c>
-      <c r="D48">
-        <v>116066343</v>
-      </c>
-      <c r="E48">
-        <v>0</v>
-      </c>
-      <c r="F48">
-        <v>163463700</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>11</v>
-      </c>
-      <c r="B49">
-        <v>2019</v>
-      </c>
-      <c r="C49">
-        <v>1032877444</v>
-      </c>
-      <c r="D49">
-        <v>0</v>
-      </c>
-      <c r="E49">
-        <v>1313511151</v>
-      </c>
-      <c r="F49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>2019</v>
-      </c>
-      <c r="C50">
-        <v>10228758</v>
-      </c>
-      <c r="D50">
-        <v>0</v>
-      </c>
-      <c r="E50">
-        <v>0</v>
-      </c>
-      <c r="F50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>50</v>
-      </c>
-      <c r="B51">
-        <v>2019</v>
-      </c>
-      <c r="C51">
-        <v>192765515</v>
-      </c>
-      <c r="D51">
-        <v>0</v>
-      </c>
-      <c r="E51">
-        <v>0</v>
-      </c>
-      <c r="F51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>51</v>
-      </c>
-      <c r="B52">
-        <v>2019</v>
-      </c>
-      <c r="C52">
-        <v>0</v>
-      </c>
-      <c r="D52">
-        <v>0</v>
-      </c>
-      <c r="E52">
-        <v>0</v>
-      </c>
-      <c r="F52">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8190302C-E34C-4DC7-B5A5-3449292AAE8F}">
-  <dimension ref="A1:E33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="33.26953125" customWidth="1"/>
-    <col min="4" max="4" width="33.453125" customWidth="1"/>
-    <col min="5" max="5" width="33" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>320</v>
-      </c>
-      <c r="C1" t="s">
-        <v>321</v>
-      </c>
-      <c r="D1" t="s">
-        <v>322</v>
-      </c>
-      <c r="E1" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>2019</v>
-      </c>
-      <c r="B2">
-        <v>1506</v>
-      </c>
-      <c r="C2">
-        <v>1583</v>
-      </c>
-      <c r="D2">
-        <v>851</v>
-      </c>
-      <c r="E2">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2020</v>
-      </c>
-      <c r="B3">
-        <v>1506</v>
-      </c>
-      <c r="C3">
-        <v>1583</v>
-      </c>
-      <c r="D3">
-        <v>851</v>
-      </c>
-      <c r="E3">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>2021</v>
-      </c>
-      <c r="B4">
-        <v>1506</v>
-      </c>
-      <c r="C4">
-        <v>1583</v>
-      </c>
-      <c r="D4">
-        <v>851</v>
-      </c>
-      <c r="E4">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>2022</v>
-      </c>
-      <c r="B5">
-        <v>1506</v>
-      </c>
-      <c r="C5">
-        <v>1583</v>
-      </c>
-      <c r="D5">
-        <v>851</v>
-      </c>
-      <c r="E5">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>2023</v>
-      </c>
-      <c r="B6">
-        <v>1506</v>
-      </c>
-      <c r="C6">
-        <v>1583</v>
-      </c>
-      <c r="D6">
-        <v>851</v>
-      </c>
-      <c r="E6">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>2024</v>
-      </c>
-      <c r="B7">
-        <v>1506</v>
-      </c>
-      <c r="C7">
-        <v>1583</v>
-      </c>
-      <c r="D7">
-        <v>851</v>
-      </c>
-      <c r="E7">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>2025</v>
-      </c>
-      <c r="B8">
-        <v>1506</v>
-      </c>
-      <c r="C8">
-        <v>1583</v>
-      </c>
-      <c r="D8">
-        <v>851</v>
-      </c>
-      <c r="E8">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>2026</v>
-      </c>
-      <c r="B9">
-        <v>1506</v>
-      </c>
-      <c r="C9">
-        <v>1583</v>
-      </c>
-      <c r="D9">
-        <v>851</v>
-      </c>
-      <c r="E9">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>2027</v>
-      </c>
-      <c r="B10">
-        <v>1506</v>
-      </c>
-      <c r="C10">
-        <v>1583</v>
-      </c>
-      <c r="D10">
-        <v>851</v>
-      </c>
-      <c r="E10">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>2028</v>
-      </c>
-      <c r="B11">
-        <v>1506</v>
-      </c>
-      <c r="C11">
-        <v>1583</v>
-      </c>
-      <c r="D11">
-        <v>851</v>
-      </c>
-      <c r="E11">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>2029</v>
-      </c>
-      <c r="B12">
-        <v>1506</v>
-      </c>
-      <c r="C12">
-        <v>1583</v>
-      </c>
-      <c r="D12">
-        <v>851</v>
-      </c>
-      <c r="E12">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>2030</v>
-      </c>
-      <c r="B13">
-        <v>1506</v>
-      </c>
-      <c r="C13">
-        <v>1583</v>
-      </c>
-      <c r="D13">
-        <v>851</v>
-      </c>
-      <c r="E13">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14">
-        <v>2031</v>
-      </c>
-      <c r="B14">
-        <v>1506</v>
-      </c>
-      <c r="C14">
-        <v>1583</v>
-      </c>
-      <c r="D14">
-        <v>851</v>
-      </c>
-      <c r="E14">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>2032</v>
-      </c>
-      <c r="B15">
-        <v>1506</v>
-      </c>
-      <c r="C15">
-        <v>1583</v>
-      </c>
-      <c r="D15">
-        <v>851</v>
-      </c>
-      <c r="E15">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>2033</v>
-      </c>
-      <c r="B16">
-        <v>1506</v>
-      </c>
-      <c r="C16">
-        <v>1583</v>
-      </c>
-      <c r="D16">
-        <v>851</v>
-      </c>
-      <c r="E16">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>2034</v>
-      </c>
-      <c r="B17">
-        <v>1506</v>
-      </c>
-      <c r="C17">
-        <v>1583</v>
-      </c>
-      <c r="D17">
-        <v>851</v>
-      </c>
-      <c r="E17">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <v>2035</v>
-      </c>
-      <c r="B18">
-        <v>1506</v>
-      </c>
-      <c r="C18">
-        <v>1583</v>
-      </c>
-      <c r="D18">
-        <v>851</v>
-      </c>
-      <c r="E18">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>2036</v>
-      </c>
-      <c r="B19">
-        <v>1506</v>
-      </c>
-      <c r="C19">
-        <v>1583</v>
-      </c>
-      <c r="D19">
-        <v>851</v>
-      </c>
-      <c r="E19">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>2037</v>
-      </c>
-      <c r="B20">
-        <v>1506</v>
-      </c>
-      <c r="C20">
-        <v>1583</v>
-      </c>
-      <c r="D20">
-        <v>851</v>
-      </c>
-      <c r="E20">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>2038</v>
-      </c>
-      <c r="B21">
-        <v>1506</v>
-      </c>
-      <c r="C21">
-        <v>1583</v>
-      </c>
-      <c r="D21">
-        <v>851</v>
-      </c>
-      <c r="E21">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>2039</v>
-      </c>
-      <c r="B22">
-        <v>1506</v>
-      </c>
-      <c r="C22">
-        <v>1583</v>
-      </c>
-      <c r="D22">
-        <v>851</v>
-      </c>
-      <c r="E22">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>2040</v>
-      </c>
-      <c r="B23">
-        <v>1506</v>
-      </c>
-      <c r="C23">
-        <v>1583</v>
-      </c>
-      <c r="D23">
-        <v>851</v>
-      </c>
-      <c r="E23">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <v>2041</v>
-      </c>
-      <c r="B24">
-        <v>1506</v>
-      </c>
-      <c r="C24">
-        <v>1583</v>
-      </c>
-      <c r="D24">
-        <v>851</v>
-      </c>
-      <c r="E24">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>2042</v>
-      </c>
-      <c r="B25">
-        <v>1506</v>
-      </c>
-      <c r="C25">
-        <v>1583</v>
-      </c>
-      <c r="D25">
-        <v>851</v>
-      </c>
-      <c r="E25">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>2043</v>
-      </c>
-      <c r="B26">
-        <v>1506</v>
-      </c>
-      <c r="C26">
-        <v>1583</v>
-      </c>
-      <c r="D26">
-        <v>851</v>
-      </c>
-      <c r="E26">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>2044</v>
-      </c>
-      <c r="B27">
-        <v>1506</v>
-      </c>
-      <c r="C27">
-        <v>1583</v>
-      </c>
-      <c r="D27">
-        <v>851</v>
-      </c>
-      <c r="E27">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>2045</v>
-      </c>
-      <c r="B28">
-        <v>1506</v>
-      </c>
-      <c r="C28">
-        <v>1583</v>
-      </c>
-      <c r="D28">
-        <v>851</v>
-      </c>
-      <c r="E28">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>2046</v>
-      </c>
-      <c r="B29">
-        <v>1506</v>
-      </c>
-      <c r="C29">
-        <v>1583</v>
-      </c>
-      <c r="D29">
-        <v>851</v>
-      </c>
-      <c r="E29">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30">
-        <v>2047</v>
-      </c>
-      <c r="B30">
-        <v>1506</v>
-      </c>
-      <c r="C30">
-        <v>1583</v>
-      </c>
-      <c r="D30">
-        <v>851</v>
-      </c>
-      <c r="E30">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31">
-        <v>2048</v>
-      </c>
-      <c r="B31">
-        <v>1506</v>
-      </c>
-      <c r="C31">
-        <v>1583</v>
-      </c>
-      <c r="D31">
-        <v>851</v>
-      </c>
-      <c r="E31">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32">
-        <v>2049</v>
-      </c>
-      <c r="B32">
-        <v>1506</v>
-      </c>
-      <c r="C32">
-        <v>1583</v>
-      </c>
-      <c r="D32">
-        <v>851</v>
-      </c>
-      <c r="E32">
-        <v>851</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33">
-        <v>2050</v>
-      </c>
-      <c r="B33">
-        <v>1506</v>
-      </c>
-      <c r="C33">
-        <v>1583</v>
-      </c>
-      <c r="D33">
-        <v>851</v>
-      </c>
-      <c r="E33">
-        <v>851</v>
       </c>
     </row>
   </sheetData>
@@ -63997,12 +59221,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>259</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
       <c r="G2" s="17">
         <f>SUM([1]AEO_VMT_Base!$B$6:$B$7)/[1]AEO_VMT_Base!$B$10</f>
         <v>0.90535164725664219</v>
@@ -87030,6 +82254,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -87211,15 +82444,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -87227,6 +82451,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -87244,14 +82476,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
added GLV stuff back to head of branch + moved VMT_Forecast
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gvendemiatti\Documents\TEACART\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="13_ncr:1_{12930437-8380-4A20-BC55-0F37E67B4891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50E4F9C-DABB-43FD-8AD4-600C041CDCCA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB20FA56-547F-4994-BA6C-8847E6EFC8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="821" firstSheet="14" activeTab="19" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="821" firstSheet="8" activeTab="12" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8660" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8661" uniqueCount="335">
   <si>
     <t>state</t>
   </si>
@@ -1094,6 +1094,9 @@
   </si>
   <si>
     <t>FR_million_tonmiles</t>
+  </si>
+  <si>
+    <t>hd_weight</t>
   </si>
 </sst>
 </file>
@@ -2154,10 +2157,10 @@
       <sheetName val="Key Inputs"/>
       <sheetName val="Baseline Parameters"/>
       <sheetName val="Custom Project Inputs"/>
-      <sheetName val="Capital Project Inputs"/>
       <sheetName val="Strategy Parameters"/>
       <sheetName val="Cost Parameters"/>
       <sheetName val="Scenario Testing"/>
+      <sheetName val="Capital Project Inputs"/>
       <sheetName val="Baseline GHG Forecast"/>
       <sheetName val="Scenario and Strategy Summary"/>
       <sheetName val="Cost Effectiveness"/>
@@ -2872,9 +2875,9 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{62EC80A7-DBC4-4CDB-B48F-50BC0B39765B}" name="Fuel_Factors" displayName="Fuel_Factors" ref="A1:M17" totalsRowShown="0">
-  <autoFilter ref="A1:M17" xr:uid="{62EC80A7-DBC4-4CDB-B48F-50BC0B39765B}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{62EC80A7-DBC4-4CDB-B48F-50BC0B39765B}" name="Fuel_Factors" displayName="Fuel_Factors" ref="A1:N17" totalsRowShown="0">
+  <autoFilter ref="A1:N17" xr:uid="{62EC80A7-DBC4-4CDB-B48F-50BC0B39765B}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{E103189A-4DA6-4377-AB4E-1DF5ED210431}" name="fuel_type"/>
     <tableColumn id="2" xr3:uid="{BC39F391-E563-4290-B1C5-823855FBBC20}" name="veh_type"/>
     <tableColumn id="3" xr3:uid="{FD2A91EE-A109-4BD3-84CC-9749CB0A60C2}" name="CH4_g_per_mi"/>
@@ -2888,6 +2891,7 @@
     <tableColumn id="11" xr3:uid="{73BC4852-3891-426D-A214-0862821D25F8}" name="NOx_g_per_veh_mi"/>
     <tableColumn id="12" xr3:uid="{04D5835E-A6BD-487D-9B3F-FF56081E7557}" name="PM25_exhaust"/>
     <tableColumn id="13" xr3:uid="{CF8E75C3-B9AF-493B-A8E2-B1380D26348F}" name="PM25_tires_brakes"/>
+    <tableColumn id="14" xr3:uid="{D60EC766-3E83-47B4-B9D6-3DFBE1E830BC}" name="hd_weight"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -19239,7 +19243,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F0F21F-CF6E-40C9-A121-647FA35A90C3}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.453125" bestFit="1" customWidth="1"/>
@@ -19252,7 +19256,7 @@
     <col min="8" max="8" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -19292,8 +19296,11 @@
       <c r="M1" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>182</v>
       </c>
@@ -19312,7 +19319,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>182</v>
       </c>
@@ -19343,7 +19350,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>182</v>
       </c>
@@ -19373,8 +19380,12 @@
       <c r="M4">
         <v>8.0000000000000002E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <f>2/3</f>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>156</v>
       </c>
@@ -19396,7 +19407,7 @@
         <v>5.7215999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>156</v>
       </c>
@@ -19418,7 +19429,7 @@
         <v>6.3771999999999993</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>156</v>
       </c>
@@ -19448,8 +19459,12 @@
       <c r="M7">
         <v>1.2999999999999999E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N7">
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>66</v>
       </c>
@@ -19471,7 +19486,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>66</v>
       </c>
@@ -19493,7 +19508,7 @@
         <v>0.29799999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>183</v>
       </c>
@@ -19515,7 +19530,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>183</v>
       </c>
@@ -19537,7 +19552,7 @@
         <v>8.3439999999999994</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -19559,7 +19574,7 @@
         <v>10.132000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>184</v>
       </c>
@@ -19581,7 +19596,7 @@
         <v>0.29799999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>156</v>
       </c>
@@ -19614,7 +19629,7 @@
         <v>1.2907268133754085E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>182</v>
       </c>
@@ -19633,7 +19648,7 @@
         <v>9.6666666666666672E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>156</v>
       </c>
@@ -87798,18 +87813,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -87831,18 +87846,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates to VMT issues
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gvendemiatti\Documents\TEACART\TEACART\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB20FA56-547F-4994-BA6C-8847E6EFC8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{701D4D3F-2980-4D84-8D38-2F82969068E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89F73685-F2ED-4A3E-886D-4D3420F11A80}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="821" firstSheet="8" activeTab="12" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView minimized="1" xWindow="42420" yWindow="-80190" windowWidth="4275" windowHeight="2175" tabRatio="821" firstSheet="6" activeTab="15" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8661" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8657" uniqueCount="335">
   <si>
     <t>state</t>
   </si>
@@ -3040,8 +3040,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}" name="AEO_VMT_Base" displayName="AEO_VMT_Base" ref="A1:C125" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
-  <autoFilter ref="A1:C125" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}" name="AEO_VMT_Base" displayName="AEO_VMT_Base" ref="A1:C121" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+  <autoFilter ref="A1:C121" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{51DE3611-329C-41B0-A4DB-52AE83C97AC8}" name="veh_type" dataDxfId="37"/>
     <tableColumn id="2" xr3:uid="{591F901E-48BF-4AA2-83C5-3ABFD077C4E7}" name="year" dataDxfId="36"/>
@@ -46173,7 +46173,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54720949-FCA8-4E91-97C8-758F882F64C3}">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -46196,10 +46196,10 @@
         <v>193</v>
       </c>
       <c r="B2" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
+        <v>175905.05869999999</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -46207,10 +46207,10 @@
         <v>192</v>
       </c>
       <c r="B3" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C3" s="1">
-        <v>0</v>
+        <v>1453415.709</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -46218,10 +46218,10 @@
         <v>222</v>
       </c>
       <c r="B4" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C4" s="1">
-        <v>0</v>
+        <v>120902.86599999999</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -46229,10 +46229,10 @@
         <v>204</v>
       </c>
       <c r="B5" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C5" s="1">
-        <v>0</v>
+        <v>1385678.007</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -46240,10 +46240,10 @@
         <v>193</v>
       </c>
       <c r="B6" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C6" s="1">
-        <v>175905.05869999999</v>
+        <v>180087.62419999999</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -46251,10 +46251,10 @@
         <v>192</v>
       </c>
       <c r="B7" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C7" s="1">
-        <v>1453415.709</v>
+        <v>1587379.9620000001</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -46262,10 +46262,10 @@
         <v>222</v>
       </c>
       <c r="B8" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C8" s="1">
-        <v>120902.86599999999</v>
+        <v>124146.145</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -46273,10 +46273,10 @@
         <v>204</v>
       </c>
       <c r="B9" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C9" s="1">
-        <v>1385678.007</v>
+        <v>1293781.5649999999</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -46284,10 +46284,10 @@
         <v>193</v>
       </c>
       <c r="B10" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C10" s="1">
-        <v>180087.62419999999</v>
+        <v>182482.29639999999</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -46295,10 +46295,10 @@
         <v>192</v>
       </c>
       <c r="B11" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>1587379.9620000001</v>
+        <v>1697480.8940000001</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -46306,10 +46306,10 @@
         <v>222</v>
       </c>
       <c r="B12" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C12" s="1">
-        <v>124146.145</v>
+        <v>126453.22</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -46317,10 +46317,10 @@
         <v>204</v>
       </c>
       <c r="B13" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C13" s="1">
-        <v>1293781.5649999999</v>
+        <v>1314686.4809999999</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -46328,10 +46328,10 @@
         <v>193</v>
       </c>
       <c r="B14" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C14" s="1">
-        <v>182482.29639999999</v>
+        <v>184146.29070000001</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -46339,10 +46339,10 @@
         <v>192</v>
       </c>
       <c r="B15" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C15" s="1">
-        <v>1697480.8940000001</v>
+        <v>1797010.4129999999</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -46350,10 +46350,10 @@
         <v>222</v>
       </c>
       <c r="B16" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C16" s="1">
-        <v>126453.22</v>
+        <v>128525.497</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -46361,10 +46361,10 @@
         <v>204</v>
       </c>
       <c r="B17" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C17" s="1">
-        <v>1314686.4809999999</v>
+        <v>1316350.733</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -46372,10 +46372,10 @@
         <v>193</v>
       </c>
       <c r="B18" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C18" s="1">
-        <v>184146.29070000001</v>
+        <v>185937.74249999999</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -46383,10 +46383,10 @@
         <v>192</v>
       </c>
       <c r="B19" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C19" s="1">
-        <v>1797010.4129999999</v>
+        <v>1871423.4709999999</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -46394,10 +46394,10 @@
         <v>222</v>
       </c>
       <c r="B20" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C20" s="1">
-        <v>128525.497</v>
+        <v>130945.202</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -46405,10 +46405,10 @@
         <v>204</v>
       </c>
       <c r="B21" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C21" s="1">
-        <v>1316350.733</v>
+        <v>1290550.6950000001</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -46416,10 +46416,10 @@
         <v>193</v>
       </c>
       <c r="B22" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C22" s="1">
-        <v>185937.74249999999</v>
+        <v>187153.3437</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -46427,10 +46427,10 @@
         <v>192</v>
       </c>
       <c r="B23" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C23" s="1">
-        <v>1871423.4709999999</v>
+        <v>1946860.6070000001</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -46438,10 +46438,10 @@
         <v>222</v>
       </c>
       <c r="B24" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C24" s="1">
-        <v>130945.202</v>
+        <v>133322.02499999999</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -46449,10 +46449,10 @@
         <v>204</v>
       </c>
       <c r="B25" s="1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C25" s="1">
-        <v>1290550.6950000001</v>
+        <v>1260452.5419999999</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -46460,10 +46460,10 @@
         <v>193</v>
       </c>
       <c r="B26" s="1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C26" s="1">
-        <v>187153.3437</v>
+        <v>187637.05809999999</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -46471,10 +46471,10 @@
         <v>192</v>
       </c>
       <c r="B27" s="1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C27" s="1">
-        <v>1946860.6070000001</v>
+        <v>2019509.8770000001</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -46482,10 +46482,10 @@
         <v>222</v>
       </c>
       <c r="B28" s="1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C28" s="1">
-        <v>133322.02499999999</v>
+        <v>135653.24100000001</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -46493,10 +46493,10 @@
         <v>204</v>
       </c>
       <c r="B29" s="1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="C29" s="1">
-        <v>1260452.5419999999</v>
+        <v>1224924.429</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -46504,10 +46504,10 @@
         <v>193</v>
       </c>
       <c r="B30" s="1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="C30" s="1">
-        <v>187637.05809999999</v>
+        <v>188223.3774</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -46515,10 +46515,10 @@
         <v>192</v>
       </c>
       <c r="B31" s="1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="C31" s="1">
-        <v>2019509.8770000001</v>
+        <v>2086422.263</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -46526,10 +46526,10 @@
         <v>222</v>
       </c>
       <c r="B32" s="1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="C32" s="1">
-        <v>135653.24100000001</v>
+        <v>138483.856</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
@@ -46537,10 +46537,10 @@
         <v>204</v>
       </c>
       <c r="B33" s="1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="C33" s="1">
-        <v>1224924.429</v>
+        <v>1184882.7139999999</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -46548,10 +46548,10 @@
         <v>193</v>
       </c>
       <c r="B34" s="1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="C34" s="1">
-        <v>188223.3774</v>
+        <v>188772.98740000001</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
@@ -46559,10 +46559,10 @@
         <v>192</v>
       </c>
       <c r="B35" s="1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="C35" s="1">
-        <v>2086422.263</v>
+        <v>2150056.2030000002</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -46570,10 +46570,10 @@
         <v>222</v>
       </c>
       <c r="B36" s="1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="C36" s="1">
-        <v>138483.856</v>
+        <v>141633.06</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -46581,10 +46581,10 @@
         <v>204</v>
       </c>
       <c r="B37" s="1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="C37" s="1">
-        <v>1184882.7139999999</v>
+        <v>1143207.7690000001</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -46592,10 +46592,10 @@
         <v>193</v>
       </c>
       <c r="B38" s="1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C38" s="1">
-        <v>188772.98740000001</v>
+        <v>189083.60569999999</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
@@ -46603,10 +46603,10 @@
         <v>192</v>
       </c>
       <c r="B39" s="1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C39" s="1">
-        <v>2150056.2030000002</v>
+        <v>2211753.6189999999</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
@@ -46614,10 +46614,10 @@
         <v>222</v>
       </c>
       <c r="B40" s="1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C40" s="1">
-        <v>141633.06</v>
+        <v>144797.84</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
@@ -46625,10 +46625,10 @@
         <v>204</v>
       </c>
       <c r="B41" s="1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="C41" s="1">
-        <v>1143207.7690000001</v>
+        <v>1102584.8289999999</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -46636,10 +46636,10 @@
         <v>193</v>
       </c>
       <c r="B42" s="1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="C42" s="1">
-        <v>189083.60569999999</v>
+        <v>189308.39300000001</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -46647,10 +46647,10 @@
         <v>192</v>
       </c>
       <c r="B43" s="1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="C43" s="1">
-        <v>2211753.6189999999</v>
+        <v>2271951.747</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -46658,10 +46658,10 @@
         <v>222</v>
       </c>
       <c r="B44" s="1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="C44" s="1">
-        <v>144797.84</v>
+        <v>148003.883</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
@@ -46669,10 +46669,10 @@
         <v>204</v>
       </c>
       <c r="B45" s="1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="C45" s="1">
-        <v>1102584.8289999999</v>
+        <v>1064723.162</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
@@ -46680,10 +46680,10 @@
         <v>193</v>
       </c>
       <c r="B46" s="1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="C46" s="1">
-        <v>189308.39300000001</v>
+        <v>189464.01329999999</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -46691,10 +46691,10 @@
         <v>192</v>
       </c>
       <c r="B47" s="1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="C47" s="1">
-        <v>2271951.747</v>
+        <v>2329925.5959999999</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -46702,10 +46702,10 @@
         <v>222</v>
       </c>
       <c r="B48" s="1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="C48" s="1">
-        <v>148003.883</v>
+        <v>151342.39999999999</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -46713,10 +46713,10 @@
         <v>204</v>
       </c>
       <c r="B49" s="1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="C49" s="1">
-        <v>1064723.162</v>
+        <v>1029644.0429999999</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
@@ -46724,10 +46724,10 @@
         <v>193</v>
       </c>
       <c r="B50" s="1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="C50" s="1">
-        <v>189464.01329999999</v>
+        <v>189539.73</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
@@ -46735,10 +46735,10 @@
         <v>192</v>
       </c>
       <c r="B51" s="1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="C51" s="1">
-        <v>2329925.5959999999</v>
+        <v>2381138.9350000001</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -46746,10 +46746,10 @@
         <v>222</v>
       </c>
       <c r="B52" s="1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="C52" s="1">
-        <v>151342.39999999999</v>
+        <v>154675.133</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -46757,10 +46757,10 @@
         <v>204</v>
       </c>
       <c r="B53" s="1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="C53" s="1">
-        <v>1029644.0429999999</v>
+        <v>996160.41799999995</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
@@ -46768,10 +46768,10 @@
         <v>193</v>
       </c>
       <c r="B54" s="1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="C54" s="1">
-        <v>189539.73</v>
+        <v>189592.37040000001</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
@@ -46779,10 +46779,10 @@
         <v>192</v>
       </c>
       <c r="B55" s="1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="C55" s="1">
-        <v>2381138.9350000001</v>
+        <v>2429660.1639999999</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
@@ -46790,10 +46790,10 @@
         <v>222</v>
       </c>
       <c r="B56" s="1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="C56" s="1">
-        <v>154675.133</v>
+        <v>157937.71400000001</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
@@ -46801,10 +46801,10 @@
         <v>204</v>
       </c>
       <c r="B57" s="1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="C57" s="1">
-        <v>996160.41799999995</v>
+        <v>966278.76100000006</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
@@ -46812,10 +46812,10 @@
         <v>193</v>
       </c>
       <c r="B58" s="1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="C58" s="1">
-        <v>189592.37040000001</v>
+        <v>189671.37849999999</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
@@ -46823,10 +46823,10 @@
         <v>192</v>
       </c>
       <c r="B59" s="1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="C59" s="1">
-        <v>2429660.1639999999</v>
+        <v>2473313.2650000001</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
@@ -46834,10 +46834,10 @@
         <v>222</v>
       </c>
       <c r="B60" s="1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="C60" s="1">
-        <v>157937.71400000001</v>
+        <v>161310.57800000001</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
@@ -46845,10 +46845,10 @@
         <v>204</v>
       </c>
       <c r="B61" s="1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="C61" s="1">
-        <v>966278.76100000006</v>
+        <v>939809.076</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
@@ -46856,10 +46856,10 @@
         <v>193</v>
       </c>
       <c r="B62" s="1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="C62" s="1">
-        <v>189671.37849999999</v>
+        <v>189741.73389999999</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
@@ -46867,10 +46867,10 @@
         <v>192</v>
       </c>
       <c r="B63" s="1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="C63" s="1">
-        <v>2473313.2650000001</v>
+        <v>2512835.2769999998</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
@@ -46878,10 +46878,10 @@
         <v>222</v>
       </c>
       <c r="B64" s="1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="C64" s="1">
-        <v>161310.57800000001</v>
+        <v>164760.88699999999</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
@@ -46889,10 +46889,10 @@
         <v>204</v>
       </c>
       <c r="B65" s="1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="C65" s="1">
-        <v>939809.076</v>
+        <v>916837.32799999998</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
@@ -46900,10 +46900,10 @@
         <v>193</v>
       </c>
       <c r="B66" s="1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="C66" s="1">
-        <v>189741.73389999999</v>
+        <v>190016.35509999999</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
@@ -46911,10 +46911,10 @@
         <v>192</v>
       </c>
       <c r="B67" s="1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="C67" s="1">
-        <v>2512835.2769999998</v>
+        <v>2549580.1340000001</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
@@ -46922,10 +46922,10 @@
         <v>222</v>
       </c>
       <c r="B68" s="1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="C68" s="1">
-        <v>164760.88699999999</v>
+        <v>168423.584</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
@@ -46933,10 +46933,10 @@
         <v>204</v>
       </c>
       <c r="B69" s="1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="C69" s="1">
-        <v>916837.32799999998</v>
+        <v>897685.51599999995</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
@@ -46944,10 +46944,10 @@
         <v>193</v>
       </c>
       <c r="B70" s="1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="C70" s="1">
-        <v>190016.35509999999</v>
+        <v>190293.97640000001</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
@@ -46955,10 +46955,10 @@
         <v>192</v>
       </c>
       <c r="B71" s="1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="C71" s="1">
-        <v>2549580.1340000001</v>
+        <v>2583804.2710000002</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
@@ -46966,10 +46966,10 @@
         <v>222</v>
       </c>
       <c r="B72" s="1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="C72" s="1">
-        <v>168423.584</v>
+        <v>172034.745</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
@@ -46977,10 +46977,10 @@
         <v>204</v>
       </c>
       <c r="B73" s="1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="C73" s="1">
-        <v>897685.51599999995</v>
+        <v>882476.03300000005</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
@@ -46988,10 +46988,10 @@
         <v>193</v>
       </c>
       <c r="B74" s="1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="C74" s="1">
-        <v>190293.97640000001</v>
+        <v>190610.7175</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
@@ -46999,10 +46999,10 @@
         <v>192</v>
       </c>
       <c r="B75" s="1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="C75" s="1">
-        <v>2583804.2710000002</v>
+        <v>2615314.9619999998</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
@@ -47010,10 +47010,10 @@
         <v>222</v>
       </c>
       <c r="B76" s="1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="C76" s="1">
-        <v>172034.745</v>
+        <v>175634.46799999999</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
@@ -47021,10 +47021,10 @@
         <v>204</v>
       </c>
       <c r="B77" s="1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="C77" s="1">
-        <v>882476.03300000005</v>
+        <v>870383.95499999996</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
@@ -47032,10 +47032,10 @@
         <v>193</v>
       </c>
       <c r="B78" s="1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="C78" s="1">
-        <v>190610.7175</v>
+        <v>190970.98680000001</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
@@ -47043,10 +47043,10 @@
         <v>192</v>
       </c>
       <c r="B79" s="1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="C79" s="1">
-        <v>2615314.9619999998</v>
+        <v>2646150.2910000002</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
@@ -47054,10 +47054,10 @@
         <v>222</v>
       </c>
       <c r="B80" s="1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="C80" s="1">
-        <v>175634.46799999999</v>
+        <v>179230.97200000001</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
@@ -47065,10 +47065,10 @@
         <v>204</v>
       </c>
       <c r="B81" s="1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="C81" s="1">
-        <v>870383.95499999996</v>
+        <v>861964.58</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
@@ -47076,10 +47076,10 @@
         <v>193</v>
       </c>
       <c r="B82" s="1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="C82" s="1">
-        <v>190970.98680000001</v>
+        <v>191453.59779999999</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
@@ -47087,10 +47087,10 @@
         <v>192</v>
       </c>
       <c r="B83" s="1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="C83" s="1">
-        <v>2646150.2910000002</v>
+        <v>2674284.6540000001</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
@@ -47098,10 +47098,10 @@
         <v>222</v>
       </c>
       <c r="B84" s="1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="C84" s="1">
-        <v>179230.97200000001</v>
+        <v>183064.33100000001</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
@@ -47109,10 +47109,10 @@
         <v>204</v>
       </c>
       <c r="B85" s="1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="C85" s="1">
-        <v>861964.58</v>
+        <v>855630.73400000005</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
@@ -47120,10 +47120,10 @@
         <v>193</v>
       </c>
       <c r="B86" s="1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="C86" s="1">
-        <v>191453.59779999999</v>
+        <v>192054.36309999999</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
@@ -47131,10 +47131,10 @@
         <v>192</v>
       </c>
       <c r="B87" s="1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="C87" s="1">
-        <v>2674284.6540000001</v>
+        <v>2699678.19</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
@@ -47142,10 +47142,10 @@
         <v>222</v>
       </c>
       <c r="B88" s="1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="C88" s="1">
-        <v>183064.33100000001</v>
+        <v>186996.95600000001</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
@@ -47153,10 +47153,10 @@
         <v>204</v>
       </c>
       <c r="B89" s="1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="C89" s="1">
-        <v>855630.73400000005</v>
+        <v>850804.74699999997</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
@@ -47164,10 +47164,10 @@
         <v>193</v>
       </c>
       <c r="B90" s="1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="C90" s="1">
-        <v>192054.36309999999</v>
+        <v>192587.74789999999</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.35">
@@ -47175,10 +47175,10 @@
         <v>192</v>
       </c>
       <c r="B91" s="1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="C91" s="1">
-        <v>2699678.19</v>
+        <v>2724653.0090000001</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.35">
@@ -47186,10 +47186,10 @@
         <v>222</v>
       </c>
       <c r="B92" s="1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="C92" s="1">
-        <v>186996.95600000001</v>
+        <v>190871.391</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.35">
@@ -47197,10 +47197,10 @@
         <v>204</v>
       </c>
       <c r="B93" s="1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="C93" s="1">
-        <v>850804.74699999997</v>
+        <v>847901.91799999995</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.35">
@@ -47208,10 +47208,10 @@
         <v>193</v>
       </c>
       <c r="B94" s="1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="C94" s="1">
-        <v>192587.74789999999</v>
+        <v>193047.80609999999</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.35">
@@ -47219,10 +47219,10 @@
         <v>192</v>
       </c>
       <c r="B95" s="1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="C95" s="1">
-        <v>2724653.0090000001</v>
+        <v>2748073.8020000001</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.35">
@@ -47230,10 +47230,10 @@
         <v>222</v>
       </c>
       <c r="B96" s="1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="C96" s="1">
-        <v>190871.391</v>
+        <v>194784.18700000001</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.35">
@@ -47241,10 +47241,10 @@
         <v>204</v>
       </c>
       <c r="B97" s="1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="C97" s="1">
-        <v>847901.91799999995</v>
+        <v>846015.01699999999</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.35">
@@ -47252,10 +47252,10 @@
         <v>193</v>
       </c>
       <c r="B98" s="1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="C98" s="1">
-        <v>193047.80609999999</v>
+        <v>193394.29629999999</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.35">
@@ -47263,10 +47263,10 @@
         <v>192</v>
       </c>
       <c r="B99" s="1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="C99" s="1">
-        <v>2748073.8020000001</v>
+        <v>2770397.1660000002</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.35">
@@ -47274,10 +47274,10 @@
         <v>222</v>
       </c>
       <c r="B100" s="1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="C100" s="1">
-        <v>194784.18700000001</v>
+        <v>198765.693</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.35">
@@ -47285,10 +47285,10 @@
         <v>204</v>
       </c>
       <c r="B101" s="1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="C101" s="1">
-        <v>846015.01699999999</v>
+        <v>844884.71200000006</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.35">
@@ -47296,10 +47296,10 @@
         <v>193</v>
       </c>
       <c r="B102" s="1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="C102" s="1">
-        <v>193394.29629999999</v>
+        <v>193830.55290000001</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.35">
@@ -47307,10 +47307,10 @@
         <v>192</v>
       </c>
       <c r="B103" s="1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="C103" s="1">
-        <v>2770397.1660000002</v>
+        <v>2793342.4109999998</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.35">
@@ -47318,10 +47318,10 @@
         <v>222</v>
       </c>
       <c r="B104" s="1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="C104" s="1">
-        <v>198765.693</v>
+        <v>202974.114</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.35">
@@ -47329,10 +47329,10 @@
         <v>204</v>
       </c>
       <c r="B105" s="1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="C105" s="1">
-        <v>844884.71200000006</v>
+        <v>845135.25600000005</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.35">
@@ -47340,10 +47340,10 @@
         <v>193</v>
       </c>
       <c r="B106" s="1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="C106" s="1">
-        <v>193830.55290000001</v>
+        <v>193839.5312</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
@@ -47351,10 +47351,10 @@
         <v>192</v>
       </c>
       <c r="B107" s="1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="C107" s="1">
-        <v>2793342.4109999998</v>
+        <v>2817418.2620000001</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
@@ -47362,10 +47362,10 @@
         <v>222</v>
       </c>
       <c r="B108" s="1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="C108" s="1">
-        <v>202974.114</v>
+        <v>206951.79</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
@@ -47373,10 +47373,10 @@
         <v>204</v>
       </c>
       <c r="B109" s="1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="C109" s="1">
-        <v>845135.25600000005</v>
+        <v>845825.82200000004</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
@@ -47384,10 +47384,10 @@
         <v>193</v>
       </c>
       <c r="B110" s="1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="C110" s="1">
-        <v>193839.5312</v>
+        <v>193480.38269999999</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
@@ -47395,10 +47395,10 @@
         <v>192</v>
       </c>
       <c r="B111" s="1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="C111" s="1">
-        <v>2817418.2620000001</v>
+        <v>2841721.6919999998</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
@@ -47406,10 +47406,10 @@
         <v>222</v>
       </c>
       <c r="B112" s="1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="C112" s="1">
-        <v>206951.79</v>
+        <v>210744.30100000001</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
@@ -47417,10 +47417,10 @@
         <v>204</v>
       </c>
       <c r="B113" s="1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="C113" s="1">
-        <v>845825.82200000004</v>
+        <v>846651.25100000005</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
@@ -47428,10 +47428,10 @@
         <v>193</v>
       </c>
       <c r="B114" s="1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="C114" s="1">
-        <v>193480.38269999999</v>
+        <v>193608.07459999999</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
@@ -47439,10 +47439,10 @@
         <v>192</v>
       </c>
       <c r="B115" s="1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="C115" s="1">
-        <v>2841721.6919999998</v>
+        <v>2866483.3050000002</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
@@ -47450,10 +47450,10 @@
         <v>222</v>
       </c>
       <c r="B116" s="1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="C116" s="1">
-        <v>210744.30100000001</v>
+        <v>215131.821</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
@@ -47461,10 +47461,10 @@
         <v>204</v>
       </c>
       <c r="B117" s="1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="C117" s="1">
-        <v>846651.25100000005</v>
+        <v>847708.85499999998</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
@@ -47472,10 +47472,10 @@
         <v>193</v>
       </c>
       <c r="B118" s="1">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="C118" s="1">
-        <v>193608.07459999999</v>
+        <v>194188.55050000001</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
@@ -47483,10 +47483,10 @@
         <v>192</v>
       </c>
       <c r="B119" s="1">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="C119" s="1">
-        <v>2866483.3050000002</v>
+        <v>2892942.5290000001</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
@@ -47494,10 +47494,10 @@
         <v>222</v>
       </c>
       <c r="B120" s="1">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="C120" s="1">
-        <v>215131.821</v>
+        <v>220055.75599999999</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
@@ -47505,53 +47505,9 @@
         <v>204</v>
       </c>
       <c r="B121" s="1">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="C121" s="1">
-        <v>847708.85499999998</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A122" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B122" s="1">
-        <v>2050</v>
-      </c>
-      <c r="C122" s="1">
-        <v>194188.55050000001</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A123" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="B123" s="1">
-        <v>2050</v>
-      </c>
-      <c r="C123" s="1">
-        <v>2892942.5290000001</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A124" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="B124" s="1">
-        <v>2050</v>
-      </c>
-      <c r="C124" s="1">
-        <v>220055.75599999999</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A125" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="B125" s="1">
-        <v>2050</v>
-      </c>
-      <c r="C125" s="1">
         <v>849019.72380000004</v>
       </c>
     </row>
@@ -87631,6 +87587,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -87812,22 +87783,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -87843,21 +87816,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
work on the processing transit elect code.
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qsi\Documents\GitHub\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4305A78-079E-471F-828D-7A4C18A27982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FCBA56-380B-40FA-BB8C-4A368AB940DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-24" windowWidth="23256" windowHeight="12252" tabRatio="955" firstSheet="6" activeTab="15" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
@@ -1107,7 +1107,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -1230,10 +1230,10 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -19467,7 +19467,7 @@
       <c r="D7">
         <v>4.3099999999999999E-2</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="21">
         <f>Fuel_Factors[[#This Row],[CH4_g_per_mi]]*INDEX(GWP[GWP], 1)</f>
         <v>0.23749999999999999</v>
       </c>
@@ -20391,7 +20391,7 @@
         <v>61</v>
       </c>
       <c r="C8">
-        <v>5.4399999999999997E-2</v>
+        <v>5.4440000000000002E-2</v>
       </c>
       <c r="D8" t="s">
         <v>290</v>
@@ -20776,7 +20776,7 @@
         <v>61</v>
       </c>
       <c r="C19">
-        <v>5.4399999999999997E-2</v>
+        <v>5.4440000000000002E-2</v>
       </c>
       <c r="D19" t="s">
         <v>290</v>
@@ -21021,7 +21021,7 @@
         <v>66</v>
       </c>
       <c r="C26">
-        <v>5.4399999999999997E-2</v>
+        <v>5.4440000000000002E-2</v>
       </c>
       <c r="D26" t="s">
         <v>290</v>
@@ -21301,7 +21301,7 @@
         <v>66</v>
       </c>
       <c r="C34">
-        <v>5.4399999999999997E-2</v>
+        <v>5.4440000000000002E-2</v>
       </c>
       <c r="D34" t="s">
         <v>290</v>
@@ -64831,12 +64831,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
       <c r="G2" s="17">
         <f>SUM([1]AEO_VMT_Base!$B$6:$B$7)/[1]AEO_VMT_Base!$B$10</f>
         <v>0.90535164725664219</v>
@@ -87864,6 +87864,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -88045,22 +88060,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -88076,21 +88093,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add cost to bikeped
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qsi\Documents\GitHub\TEACART\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4409B169-60DF-4627-92F1-3418E514A04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-24" windowWidth="23256" windowHeight="12252" tabRatio="955" firstSheet="11" activeTab="19" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="-23148" yWindow="-24" windowWidth="23256" windowHeight="12252" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -34,11 +34,12 @@
     <sheet name="Passenger_Rail_State_Mileage" sheetId="25" r:id="rId19"/>
     <sheet name="Passenger_Rail_FuelFactors" sheetId="26" r:id="rId20"/>
     <sheet name="Freight_Rail_Data" sheetId="27" r:id="rId21"/>
+    <sheet name="Public_Transit_data" sheetId="29" r:id="rId22"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId22"/>
     <externalReference r:id="rId23"/>
     <externalReference r:id="rId24"/>
+    <externalReference r:id="rId25"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">AEO_VMT_Base!$A$1:$C$1</definedName>
@@ -93,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8688" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8749" uniqueCount="340">
   <si>
     <t>state</t>
   </si>
@@ -1096,6 +1097,24 @@
   <si>
     <t>upstream_life_cycle_factor</t>
   </si>
+  <si>
+    <t>State Abbreviation</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>CB</t>
+  </si>
+  <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>MB</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
 </sst>
 </file>
 
@@ -1206,7 +1225,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1231,10 +1250,16 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -3000,9 +3025,9 @@
   <autoFilter ref="A1:E33" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6059561D-B144-44A4-BD42-8A6CB47AE110}" name="year"/>
-    <tableColumn id="2" xr3:uid="{D8A3ABC2-F1D5-4278-9FC5-76DED278C85F}" name="amtrak_Energy_Intensity_BTUPerPaxMil" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{D8A3ABC2-F1D5-4278-9FC5-76DED278C85F}" name="amtrak_Energy_Intensity_BTUPerPaxMil" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{E65C9314-C120-4F4A-B346-84C59D802685}" name="CR_Energy_Intensity_BTUPerPaxMil" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{425B37B1-3EA8-495D-91F4-852DA9CC3D68}" name="HR_Energy_Intensity_BTUPerPaxMil" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{425B37B1-3EA8-495D-91F4-852DA9CC3D68}" name="HR_Energy_Intensity_BTUPerPaxMil" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{88F33EA8-F37C-4417-AC3E-4ECBF4C7F327}" name="LR_Energy_Intensity_BTUPerPaxMil"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -41478,16 +41503,16 @@
       <c r="A2">
         <v>2019</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C2" s="23">
+      <c r="C2" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D2" s="23">
+      <c r="D2" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41495,16 +41520,16 @@
       <c r="A3">
         <v>2020</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C3" s="23">
+      <c r="C3" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D3" s="23">
+      <c r="D3" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41512,16 +41537,16 @@
       <c r="A4">
         <v>2021</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C4" s="23">
+      <c r="C4" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41529,16 +41554,16 @@
       <c r="A5">
         <v>2022</v>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41546,16 +41571,16 @@
       <c r="A6">
         <v>2023</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41563,16 +41588,16 @@
       <c r="A7">
         <v>2024</v>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41580,16 +41605,16 @@
       <c r="A8">
         <v>2025</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41597,16 +41622,16 @@
       <c r="A9">
         <v>2026</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41614,16 +41639,16 @@
       <c r="A10">
         <v>2027</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41631,16 +41656,16 @@
       <c r="A11">
         <v>2028</v>
       </c>
-      <c r="B11" s="23">
+      <c r="B11" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41648,16 +41673,16 @@
       <c r="A12">
         <v>2029</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41665,16 +41690,16 @@
       <c r="A13">
         <v>2030</v>
       </c>
-      <c r="B13" s="23">
+      <c r="B13" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41682,16 +41707,16 @@
       <c r="A14">
         <v>2031</v>
       </c>
-      <c r="B14" s="23">
+      <c r="B14" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41699,16 +41724,16 @@
       <c r="A15">
         <v>2032</v>
       </c>
-      <c r="B15" s="23">
+      <c r="B15" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D15" s="23">
+      <c r="D15" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41716,16 +41741,16 @@
       <c r="A16">
         <v>2033</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D16" s="23">
+      <c r="D16" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41733,16 +41758,16 @@
       <c r="A17">
         <v>2034</v>
       </c>
-      <c r="B17" s="23">
+      <c r="B17" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41750,16 +41775,16 @@
       <c r="A18">
         <v>2035</v>
       </c>
-      <c r="B18" s="23">
+      <c r="B18" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41767,16 +41792,16 @@
       <c r="A19">
         <v>2036</v>
       </c>
-      <c r="B19" s="23">
+      <c r="B19" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41784,16 +41809,16 @@
       <c r="A20">
         <v>2037</v>
       </c>
-      <c r="B20" s="23">
+      <c r="B20" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41801,16 +41826,16 @@
       <c r="A21">
         <v>2038</v>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41818,16 +41843,16 @@
       <c r="A22">
         <v>2039</v>
       </c>
-      <c r="B22" s="23">
+      <c r="B22" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41835,16 +41860,16 @@
       <c r="A23">
         <v>2040</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41852,16 +41877,16 @@
       <c r="A24">
         <v>2041</v>
       </c>
-      <c r="B24" s="23">
+      <c r="B24" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D24" s="23">
+      <c r="D24" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41869,16 +41894,16 @@
       <c r="A25">
         <v>2042</v>
       </c>
-      <c r="B25" s="23">
+      <c r="B25" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D25" s="23">
+      <c r="D25" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41886,16 +41911,16 @@
       <c r="A26">
         <v>2043</v>
       </c>
-      <c r="B26" s="23">
+      <c r="B26" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D26" s="23">
+      <c r="D26" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41903,16 +41928,16 @@
       <c r="A27">
         <v>2044</v>
       </c>
-      <c r="B27" s="23">
+      <c r="B27" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41920,16 +41945,16 @@
       <c r="A28">
         <v>2045</v>
       </c>
-      <c r="B28" s="23">
+      <c r="B28" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D28" s="23">
+      <c r="D28" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41937,16 +41962,16 @@
       <c r="A29">
         <v>2046</v>
       </c>
-      <c r="B29" s="23">
+      <c r="B29" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D29" s="23">
+      <c r="D29" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E29" s="23">
+      <c r="E29" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41954,16 +41979,16 @@
       <c r="A30">
         <v>2047</v>
       </c>
-      <c r="B30" s="23">
+      <c r="B30" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D30" s="23">
+      <c r="D30" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E30" s="23">
+      <c r="E30" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41971,16 +41996,16 @@
       <c r="A31">
         <v>2048</v>
       </c>
-      <c r="B31" s="23">
+      <c r="B31" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D31" s="23">
+      <c r="D31" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E31" s="23">
+      <c r="E31" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -41988,16 +42013,16 @@
       <c r="A32">
         <v>2049</v>
       </c>
-      <c r="B32" s="23">
+      <c r="B32" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C32" s="23">
+      <c r="C32" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D32" s="23">
+      <c r="D32" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E32" s="23">
+      <c r="E32" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -42005,16 +42030,16 @@
       <c r="A33">
         <v>2050</v>
       </c>
-      <c r="B33" s="23">
+      <c r="B33" s="22">
         <v>1506.0564783587499</v>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="22">
         <v>1582.5116758178201</v>
       </c>
-      <c r="D33" s="23">
+      <c r="D33" s="22">
         <v>850.593849448794</v>
       </c>
-      <c r="E33" s="23">
+      <c r="E33" s="22">
         <v>850.593849448794</v>
       </c>
     </row>
@@ -42601,6 +42626,1147 @@
       </c>
       <c r="C52">
         <v>3863.6778559999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C856A2-2644-45CE-8C61-85605A6B28DC}">
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>334</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>335</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>336</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>337</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>338</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="25" t="str">
+        <f>VLOOKUP(A2, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Alaska</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25">
+        <v>1820969</v>
+      </c>
+      <c r="E2" s="25">
+        <v>4544203</v>
+      </c>
+      <c r="F2" s="25">
+        <v>6365172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="25" t="str">
+        <f>VLOOKUP(A3, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Alabama</v>
+      </c>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25">
+        <v>10146650</v>
+      </c>
+      <c r="E3" s="25">
+        <v>6650385</v>
+      </c>
+      <c r="F3" s="25">
+        <v>16797035</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="25" t="str">
+        <f>VLOOKUP(A4, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Arkansas</v>
+      </c>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25">
+        <v>13251409</v>
+      </c>
+      <c r="E4" s="25">
+        <v>4668133</v>
+      </c>
+      <c r="F4" s="25">
+        <v>17919542</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="25" t="e">
+        <f>VLOOKUP(A5, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25">
+        <v>128251</v>
+      </c>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25">
+        <v>128251</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="25" t="str">
+        <f>VLOOKUP(A6, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Arizona</v>
+      </c>
+      <c r="C6" s="25">
+        <v>686829</v>
+      </c>
+      <c r="D6" s="25">
+        <v>8850838</v>
+      </c>
+      <c r="E6" s="25">
+        <v>49557933</v>
+      </c>
+      <c r="F6" s="25">
+        <v>59095600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="25" t="str">
+        <f>VLOOKUP(A7, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>California</v>
+      </c>
+      <c r="C7" s="25">
+        <v>17653453</v>
+      </c>
+      <c r="D7" s="25">
+        <v>88205270</v>
+      </c>
+      <c r="E7" s="25">
+        <v>330675119</v>
+      </c>
+      <c r="F7" s="25">
+        <v>436533842</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="25" t="str">
+        <f>VLOOKUP(A8, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Colorado</v>
+      </c>
+      <c r="C8" s="25">
+        <v>3275162</v>
+      </c>
+      <c r="D8" s="25">
+        <v>18116638</v>
+      </c>
+      <c r="E8" s="25">
+        <v>49855214</v>
+      </c>
+      <c r="F8" s="25">
+        <v>71247014</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="25" t="str">
+        <f>VLOOKUP(A9, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Connecticut</v>
+      </c>
+      <c r="C9" s="25">
+        <v>1302927</v>
+      </c>
+      <c r="D9" s="25">
+        <v>9462995</v>
+      </c>
+      <c r="E9" s="25">
+        <v>23037923</v>
+      </c>
+      <c r="F9" s="25">
+        <v>33803845</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="25" t="str">
+        <f>VLOOKUP(A10, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>District of Columbia</v>
+      </c>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25">
+        <v>19685883</v>
+      </c>
+      <c r="E10" s="25">
+        <v>38872603</v>
+      </c>
+      <c r="F10" s="25">
+        <v>58558486</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" s="25" t="str">
+        <f>VLOOKUP(A11, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Delaware</v>
+      </c>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25">
+        <v>8098492</v>
+      </c>
+      <c r="E11" s="25">
+        <v>8984139</v>
+      </c>
+      <c r="F11" s="25">
+        <v>17082631</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="25" t="str">
+        <f>VLOOKUP(A12, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Florida</v>
+      </c>
+      <c r="C12" s="25">
+        <v>1206534</v>
+      </c>
+      <c r="D12" s="25">
+        <v>80295496</v>
+      </c>
+      <c r="E12" s="25">
+        <v>124877739</v>
+      </c>
+      <c r="F12" s="25">
+        <v>206379769</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="25" t="str">
+        <f>VLOOKUP(A13, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Georgia</v>
+      </c>
+      <c r="C13" s="25">
+        <v>3708274</v>
+      </c>
+      <c r="D13" s="25">
+        <v>28298863</v>
+      </c>
+      <c r="E13" s="25">
+        <v>40629519</v>
+      </c>
+      <c r="F13" s="25">
+        <v>72636656</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="25" t="e">
+        <f>VLOOKUP(A14, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25">
+        <v>372212</v>
+      </c>
+      <c r="E14" s="25">
+        <v>422892</v>
+      </c>
+      <c r="F14" s="25">
+        <v>795104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="25" t="str">
+        <f>VLOOKUP(A15, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Hawaii</v>
+      </c>
+      <c r="C15" s="25">
+        <v>1888935</v>
+      </c>
+      <c r="D15" s="25">
+        <v>9218028</v>
+      </c>
+      <c r="E15" s="25">
+        <v>20454917</v>
+      </c>
+      <c r="F15" s="25">
+        <v>31561880</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="25" t="str">
+        <f>VLOOKUP(A16, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Iowa</v>
+      </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25">
+        <v>16204926</v>
+      </c>
+      <c r="E16" s="25">
+        <v>11203459</v>
+      </c>
+      <c r="F16" s="25">
+        <v>27408385</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="25" t="str">
+        <f>VLOOKUP(A17, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Idaho</v>
+      </c>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25">
+        <v>1792488</v>
+      </c>
+      <c r="E17" s="25">
+        <v>4418282</v>
+      </c>
+      <c r="F17" s="25">
+        <v>6210770</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="25" t="str">
+        <f>VLOOKUP(A18, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Illinois</v>
+      </c>
+      <c r="C18" s="25">
+        <v>316684</v>
+      </c>
+      <c r="D18" s="25">
+        <v>51817490</v>
+      </c>
+      <c r="E18" s="25">
+        <v>103734267</v>
+      </c>
+      <c r="F18" s="25">
+        <v>155868441</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="25" t="str">
+        <f>VLOOKUP(A19, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Indiana</v>
+      </c>
+      <c r="C19" s="25">
+        <v>450990</v>
+      </c>
+      <c r="D19" s="25">
+        <v>18241770</v>
+      </c>
+      <c r="E19" s="25">
+        <v>19286019</v>
+      </c>
+      <c r="F19" s="25">
+        <v>37978779</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="25" t="str">
+        <f>VLOOKUP(A20, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Kansas</v>
+      </c>
+      <c r="C20" s="25">
+        <v>366540</v>
+      </c>
+      <c r="D20" s="25">
+        <v>7847064</v>
+      </c>
+      <c r="E20" s="25">
+        <v>7512599</v>
+      </c>
+      <c r="F20" s="25">
+        <v>15726203</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="25" t="str">
+        <f>VLOOKUP(A21, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Kentucky</v>
+      </c>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25">
+        <v>35520308</v>
+      </c>
+      <c r="E21" s="25">
+        <v>14087087</v>
+      </c>
+      <c r="F21" s="25">
+        <v>49607395</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" s="25" t="str">
+        <f>VLOOKUP(A22, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Louisiana</v>
+      </c>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25">
+        <v>10323437</v>
+      </c>
+      <c r="E22" s="25">
+        <v>15649937</v>
+      </c>
+      <c r="F22" s="25">
+        <v>25973374</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="25" t="str">
+        <f>VLOOKUP(A23, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Massachusetts</v>
+      </c>
+      <c r="C23" s="25">
+        <v>3104521</v>
+      </c>
+      <c r="D23" s="25">
+        <v>31031514</v>
+      </c>
+      <c r="E23" s="25">
+        <v>43374617</v>
+      </c>
+      <c r="F23" s="25">
+        <v>77510652</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="25" t="str">
+        <f>VLOOKUP(A24, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Maryland</v>
+      </c>
+      <c r="C24" s="25">
+        <v>6636014</v>
+      </c>
+      <c r="D24" s="25">
+        <v>26146936</v>
+      </c>
+      <c r="E24" s="25">
+        <v>48391900</v>
+      </c>
+      <c r="F24" s="25">
+        <v>81174850</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" s="25" t="str">
+        <f>VLOOKUP(A25, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Maine</v>
+      </c>
+      <c r="C25" s="25">
+        <v>265210</v>
+      </c>
+      <c r="D25" s="25">
+        <v>10826516</v>
+      </c>
+      <c r="E25" s="25">
+        <v>4137861</v>
+      </c>
+      <c r="F25" s="25">
+        <v>15229587</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="25" t="str">
+        <f>VLOOKUP(A26, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Michigan</v>
+      </c>
+      <c r="C26" s="25">
+        <v>432546</v>
+      </c>
+      <c r="D26" s="25">
+        <v>50261455</v>
+      </c>
+      <c r="E26" s="25">
+        <v>49939298</v>
+      </c>
+      <c r="F26" s="25">
+        <v>100633299</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="25" t="str">
+        <f>VLOOKUP(A27, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Minnesota</v>
+      </c>
+      <c r="C27" s="25">
+        <v>217003</v>
+      </c>
+      <c r="D27" s="25">
+        <v>37519099</v>
+      </c>
+      <c r="E27" s="25">
+        <v>44630214</v>
+      </c>
+      <c r="F27" s="25">
+        <v>82366316</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" s="25" t="str">
+        <f>VLOOKUP(A28, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Missouri</v>
+      </c>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25">
+        <v>25977732</v>
+      </c>
+      <c r="E28" s="25">
+        <v>29294533</v>
+      </c>
+      <c r="F28" s="25">
+        <v>55272265</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="25" t="str">
+        <f>VLOOKUP(A29, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Mississippi</v>
+      </c>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25">
+        <v>10355411</v>
+      </c>
+      <c r="E29" s="25">
+        <v>3281232</v>
+      </c>
+      <c r="F29" s="25">
+        <v>13636643</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="25" t="str">
+        <f>VLOOKUP(A30, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Montana</v>
+      </c>
+      <c r="C30" s="25">
+        <v>145031</v>
+      </c>
+      <c r="D30" s="25">
+        <v>2994570</v>
+      </c>
+      <c r="E30" s="25">
+        <v>3791255</v>
+      </c>
+      <c r="F30" s="25">
+        <v>6930856</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="25" t="str">
+        <f>VLOOKUP(A31, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>North Carolina</v>
+      </c>
+      <c r="C31" s="25">
+        <v>2548230</v>
+      </c>
+      <c r="D31" s="25">
+        <v>49037696</v>
+      </c>
+      <c r="E31" s="25">
+        <v>37124123</v>
+      </c>
+      <c r="F31" s="25">
+        <v>88710049</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" s="25" t="str">
+        <f>VLOOKUP(A32, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>North Dakota</v>
+      </c>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25">
+        <v>4584891</v>
+      </c>
+      <c r="E32" s="25">
+        <v>1934311</v>
+      </c>
+      <c r="F32" s="25">
+        <v>6519202</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" s="25" t="str">
+        <f>VLOOKUP(A33, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Nebraska</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25">
+        <v>4815160</v>
+      </c>
+      <c r="E33" s="25">
+        <v>6276073</v>
+      </c>
+      <c r="F33" s="25">
+        <v>11091233</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" s="25" t="str">
+        <f>VLOOKUP(A34, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>New Hampshire</v>
+      </c>
+      <c r="C34" s="25">
+        <v>3969821</v>
+      </c>
+      <c r="D34" s="25">
+        <v>875174</v>
+      </c>
+      <c r="E34" s="25">
+        <v>2401459</v>
+      </c>
+      <c r="F34" s="25">
+        <v>7246454</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" s="25" t="str">
+        <f>VLOOKUP(A35, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>New Jersey</v>
+      </c>
+      <c r="C35" s="25">
+        <v>30328896</v>
+      </c>
+      <c r="D35" s="25">
+        <v>22632079</v>
+      </c>
+      <c r="E35" s="25">
+        <v>85248950</v>
+      </c>
+      <c r="F35" s="25">
+        <v>138209925</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B36" s="25" t="str">
+        <f>VLOOKUP(A36, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>New Mexico</v>
+      </c>
+      <c r="C36" s="25">
+        <v>331362</v>
+      </c>
+      <c r="D36" s="25">
+        <v>4270615</v>
+      </c>
+      <c r="E36" s="25">
+        <v>11058565</v>
+      </c>
+      <c r="F36" s="25">
+        <v>15660542</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="25" t="str">
+        <f>VLOOKUP(A37, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Nevada</v>
+      </c>
+      <c r="C37" s="25">
+        <v>410090</v>
+      </c>
+      <c r="D37" s="25">
+        <v>13795616</v>
+      </c>
+      <c r="E37" s="25">
+        <v>22752296</v>
+      </c>
+      <c r="F37" s="25">
+        <v>36958002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B38" s="25" t="str">
+        <f>VLOOKUP(A38, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>New York</v>
+      </c>
+      <c r="C38" s="25">
+        <v>18162255</v>
+      </c>
+      <c r="D38" s="25">
+        <v>62282351</v>
+      </c>
+      <c r="E38" s="25">
+        <v>182735062</v>
+      </c>
+      <c r="F38" s="25">
+        <v>263179668</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="B39" s="25" t="str">
+        <f>VLOOKUP(A39, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Ohio</v>
+      </c>
+      <c r="C39" s="25">
+        <v>515002</v>
+      </c>
+      <c r="D39" s="25">
+        <v>37821824</v>
+      </c>
+      <c r="E39" s="25">
+        <v>56939993</v>
+      </c>
+      <c r="F39" s="25">
+        <v>95276819</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="25" t="str">
+        <f>VLOOKUP(A40, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Oklahoma</v>
+      </c>
+      <c r="C40" s="25">
+        <v>92708</v>
+      </c>
+      <c r="D40" s="25">
+        <v>19161183</v>
+      </c>
+      <c r="E40" s="25">
+        <v>7918742</v>
+      </c>
+      <c r="F40" s="25">
+        <v>27172633</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="B41" s="25" t="str">
+        <f>VLOOKUP(A41, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Oregon</v>
+      </c>
+      <c r="C41" s="25">
+        <v>3750422</v>
+      </c>
+      <c r="D41" s="25">
+        <v>13160147</v>
+      </c>
+      <c r="E41" s="25">
+        <v>33429198</v>
+      </c>
+      <c r="F41" s="25">
+        <v>50339767</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B42" s="25" t="str">
+        <f>VLOOKUP(A42, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Pennsylvania</v>
+      </c>
+      <c r="C42" s="25">
+        <v>4926331</v>
+      </c>
+      <c r="D42" s="25">
+        <v>44238102</v>
+      </c>
+      <c r="E42" s="25">
+        <v>88986984</v>
+      </c>
+      <c r="F42" s="25">
+        <v>138151417</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B43" s="25" t="str">
+        <f>VLOOKUP(A43, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Puerto Rico</v>
+      </c>
+      <c r="C43" s="25"/>
+      <c r="D43" s="25">
+        <v>1401597</v>
+      </c>
+      <c r="E43" s="25">
+        <v>5328065</v>
+      </c>
+      <c r="F43" s="25">
+        <v>6729662</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" s="25" t="str">
+        <f>VLOOKUP(A44, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Rhode Island</v>
+      </c>
+      <c r="C44" s="25"/>
+      <c r="D44" s="25">
+        <v>2424533</v>
+      </c>
+      <c r="E44" s="25">
+        <v>8922598</v>
+      </c>
+      <c r="F44" s="25">
+        <v>11347131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="B45" s="25" t="str">
+        <f>VLOOKUP(A45, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>South Carolina</v>
+      </c>
+      <c r="C45" s="25">
+        <v>701719</v>
+      </c>
+      <c r="D45" s="25">
+        <v>9490872</v>
+      </c>
+      <c r="E45" s="25">
+        <v>10435969</v>
+      </c>
+      <c r="F45" s="25">
+        <v>20628560</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B46" s="25" t="str">
+        <f>VLOOKUP(A46, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>South Dakota</v>
+      </c>
+      <c r="C46" s="25"/>
+      <c r="D46" s="25">
+        <v>5071774</v>
+      </c>
+      <c r="E46" s="25">
+        <v>1450451</v>
+      </c>
+      <c r="F46" s="25">
+        <v>6522225</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47" s="25" t="str">
+        <f>VLOOKUP(A47, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Tennessee</v>
+      </c>
+      <c r="C47" s="25">
+        <v>326460</v>
+      </c>
+      <c r="D47" s="25">
+        <v>31402928</v>
+      </c>
+      <c r="E47" s="25">
+        <v>21251959</v>
+      </c>
+      <c r="F47" s="25">
+        <v>52981347</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="B48" s="25" t="str">
+        <f>VLOOKUP(A48, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Texas</v>
+      </c>
+      <c r="C48" s="25">
+        <v>14830278</v>
+      </c>
+      <c r="D48" s="25">
+        <v>75039448</v>
+      </c>
+      <c r="E48" s="25">
+        <v>140051617</v>
+      </c>
+      <c r="F48" s="25">
+        <v>229921343</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="B49" s="25" t="str">
+        <f>VLOOKUP(A49, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Utah</v>
+      </c>
+      <c r="C49" s="25">
+        <v>904101</v>
+      </c>
+      <c r="D49" s="25">
+        <v>3319266</v>
+      </c>
+      <c r="E49" s="25">
+        <v>20872218</v>
+      </c>
+      <c r="F49" s="25">
+        <v>25095585</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B50" s="25" t="str">
+        <f>VLOOKUP(A50, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Virginia</v>
+      </c>
+      <c r="C50" s="25">
+        <v>4031352</v>
+      </c>
+      <c r="D50" s="25">
+        <v>13200660</v>
+      </c>
+      <c r="E50" s="25">
+        <v>44091053</v>
+      </c>
+      <c r="F50" s="25">
+        <v>61323065</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="B51" s="25" t="str">
+        <f>VLOOKUP(A51, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Virgin Islands</v>
+      </c>
+      <c r="C51" s="25"/>
+      <c r="D51" s="25">
+        <v>349850</v>
+      </c>
+      <c r="E51" s="25">
+        <v>291988</v>
+      </c>
+      <c r="F51" s="25">
+        <v>641838</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" s="25" t="str">
+        <f>VLOOKUP(A52, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Vermont</v>
+      </c>
+      <c r="C52" s="25">
+        <v>2005605</v>
+      </c>
+      <c r="D52" s="25">
+        <v>13420628</v>
+      </c>
+      <c r="E52" s="25">
+        <v>3731759</v>
+      </c>
+      <c r="F52" s="25">
+        <v>19157992</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="25" t="str">
+        <f>VLOOKUP(A53, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Washington</v>
+      </c>
+      <c r="C53" s="25">
+        <v>15447471</v>
+      </c>
+      <c r="D53" s="25">
+        <v>28877650</v>
+      </c>
+      <c r="E53" s="25">
+        <v>83332487</v>
+      </c>
+      <c r="F53" s="25">
+        <v>127657608</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="B54" s="25" t="str">
+        <f>VLOOKUP(A54, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Wisconsin</v>
+      </c>
+      <c r="C54" s="25">
+        <v>880327</v>
+      </c>
+      <c r="D54" s="25">
+        <v>16792018</v>
+      </c>
+      <c r="E54" s="25">
+        <v>33284438</v>
+      </c>
+      <c r="F54" s="25">
+        <v>50956783</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="25" t="s">
+        <v>151</v>
+      </c>
+      <c r="B55" s="25" t="str">
+        <f>VLOOKUP(A55, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>West Virginia</v>
+      </c>
+      <c r="C55" s="25"/>
+      <c r="D55" s="25">
+        <v>2671749</v>
+      </c>
+      <c r="E55" s="25">
+        <v>9309564</v>
+      </c>
+      <c r="F55" s="25">
+        <v>11981313</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="B56" s="25" t="str">
+        <f>VLOOKUP(A56, [1]Lookups!$N$5:$O$57, 2, FALSE)</f>
+        <v>Wyoming</v>
+      </c>
+      <c r="C56" s="25"/>
+      <c r="D56" s="25">
+        <v>1673521</v>
+      </c>
+      <c r="E56" s="25">
+        <v>2044125</v>
+      </c>
+      <c r="F56" s="25">
+        <v>3717646</v>
       </c>
     </row>
   </sheetData>
@@ -64874,12 +66040,12 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="23" t="s">
         <v>247</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
       <c r="G2" s="17">
         <f>SUM([1]AEO_VMT_Base!$B$6:$B$7)/[1]AEO_VMT_Base!$B$10</f>
         <v>0.90535164725664219</v>
@@ -87907,6 +89073,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -88088,22 +89269,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -88119,21 +89302,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
First Draft for Baseline
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C40857C8-DB94-490D-B801-0577F9A83C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51A45467-8339-4845-8290-F195DF3AAA88}"/>
   <bookViews>
     <workbookView xWindow="270" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8747" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8748" uniqueCount="339">
   <si>
     <t>state</t>
   </si>
@@ -1266,7 +1266,10 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="93">
+  <dxfs count="94">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2896,19 +2899,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADE72E7A-0DB0-4383-8DA6-330004A96BD0}" name="State_Populations" displayName="State_Populations" ref="A1:C154" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADE72E7A-0DB0-4383-8DA6-330004A96BD0}" name="State_Populations" displayName="State_Populations" ref="A1:C154" totalsRowShown="0" headerRowDxfId="93" dataDxfId="92">
   <autoFilter ref="A1:C154" xr:uid="{ADE72E7A-0DB0-4383-8DA6-330004A96BD0}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F73397ED-6858-4813-B93E-2A498EEFD6E3}" name="state" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{EAD47E40-4750-4C1A-A537-F6E5EF6A8690}" name="year" dataDxfId="89"/>
-    <tableColumn id="3" xr3:uid="{4E1E205E-B487-4A34-A35C-C243A187E68E}" name="population" dataDxfId="88"/>
+    <tableColumn id="1" xr3:uid="{F73397ED-6858-4813-B93E-2A498EEFD6E3}" name="state" dataDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{EAD47E40-4750-4C1A-A537-F6E5EF6A8690}" name="year" dataDxfId="90"/>
+    <tableColumn id="3" xr3:uid="{4E1E205E-B487-4A34-A35C-C243A187E68E}" name="population" dataDxfId="89"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{B4795AAF-4610-425F-8F68-4147C1C92E9B}" name="Transit_Costs" displayName="Transit_Costs" ref="A1:F194" totalsRowShown="0" headerRowDxfId="19" headerRowCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{B4795AAF-4610-425F-8F68-4147C1C92E9B}" name="Transit_Costs" displayName="Transit_Costs" ref="A1:F194" totalsRowShown="0" headerRowDxfId="20" headerRowCellStyle="Percent">
   <autoFilter ref="A1:F194" xr:uid="{B4795AAF-4610-425F-8F68-4147C1C92E9B}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3700977E-9911-44C0-B2F1-15979A419435}" name="state_code"/>
@@ -2937,12 +2940,12 @@
     <tableColumn id="5" xr3:uid="{751366A9-9305-492E-A769-B802C8C7CC10}" name="total_mode_VOMS"/>
     <tableColumn id="6" xr3:uid="{7858DD05-7D70-4987-8F3C-55ACAC76303F}" name="total_vehicle_rev_miles"/>
     <tableColumn id="7" xr3:uid="{688BA74D-9B8A-495A-9C38-87B84285B3A5}" name="total_unlinked_trips"/>
-    <tableColumn id="9" xr3:uid="{F47DAB7E-0908-4873-B99E-FC544AA9407F}" name="total_miles_per_veh" dataDxfId="18">
+    <tableColumn id="9" xr3:uid="{F47DAB7E-0908-4873-B99E-FC544AA9407F}" name="total_miles_per_veh" dataDxfId="19">
       <calculatedColumnFormula>F2/E2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D8D93C7A-8CA9-4D72-844F-B335D2C20C19}" name="total_pass_miles" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{F5AEBFD2-08D8-4868-BAFE-9688429964B0}" name="load_factor" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{05EF0C75-B302-4BAB-8F15-9D21DC18BA9D}" name="avg_trip_length" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{D8D93C7A-8CA9-4D72-844F-B335D2C20C19}" name="total_pass_miles" dataDxfId="18"/>
+    <tableColumn id="10" xr3:uid="{F5AEBFD2-08D8-4868-BAFE-9688429964B0}" name="load_factor" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{05EF0C75-B302-4BAB-8F15-9D21DC18BA9D}" name="avg_trip_length" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2956,12 +2959,12 @@
     <tableColumn id="2" xr3:uid="{BC39F391-E563-4290-B1C5-823855FBBC20}" name="veh_type"/>
     <tableColumn id="3" xr3:uid="{FD2A91EE-A109-4BD3-84CC-9749CB0A60C2}" name="CH4_g_per_mi"/>
     <tableColumn id="4" xr3:uid="{555E7F06-1A67-40BE-A12E-4388C018C1D8}" name="N20_g_per_mi"/>
-    <tableColumn id="5" xr3:uid="{510D765C-5A91-4829-963B-B311F21E7164}" name="GWP_CH4_g_per_mi" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{E24522AC-FEF6-4CF1-A652-CD1CACE1519C}" name="GWP_N20_g_per_mi" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{510D765C-5A91-4829-963B-B311F21E7164}" name="GWP_CH4_g_per_mi" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{E24522AC-FEF6-4CF1-A652-CD1CACE1519C}" name="GWP_N20_g_per_mi" dataDxfId="14"/>
     <tableColumn id="7" xr3:uid="{BDE6D434-E061-4642-81E8-F626242F89AD}" name="CH4_g_per_gallon"/>
     <tableColumn id="8" xr3:uid="{D768C14D-D955-4B79-A3AF-B0DAB187B3AE}" name="N20_g_per_gallon"/>
-    <tableColumn id="9" xr3:uid="{9302FD96-30DA-4894-98D7-E14FC261340C}" name="GWP_CH4_g_per_gallon" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{236B1E85-CD34-4728-A85A-22981CBD37AD}" name="GWP_N20_g_per_gallon" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{9302FD96-30DA-4894-98D7-E14FC261340C}" name="GWP_CH4_g_per_gallon" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{236B1E85-CD34-4728-A85A-22981CBD37AD}" name="GWP_N20_g_per_gallon" dataDxfId="12"/>
     <tableColumn id="11" xr3:uid="{73BC4852-3891-426D-A214-0862821D25F8}" name="NOx_g_per_veh_mi"/>
     <tableColumn id="12" xr3:uid="{04D5835E-A6BD-487D-9B3F-FF56081E7557}" name="PM25_exhaust"/>
     <tableColumn id="13" xr3:uid="{CF8E75C3-B9AF-493B-A8E2-B1380D26348F}" name="PM25_tires_brakes"/>
@@ -3050,7 +3053,7 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9A86A176-CF61-4734-9BAD-94713ADA77C0}" name="state"/>
     <tableColumn id="2" xr3:uid="{D0619388-12F1-4E6B-B22A-CA319BB3CE1F}" name="year"/>
-    <tableColumn id="3" xr3:uid="{221E64F0-9F3D-4CEE-B8D8-C755259DAA15}" name="amtrak_riders" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{221E64F0-9F3D-4CEE-B8D8-C755259DAA15}" name="amtrak_riders" dataDxfId="11"/>
     <tableColumn id="4" xr3:uid="{550AFC65-8E32-4A03-A47B-4AC1D0B32575}" name="commuterrail_miles"/>
     <tableColumn id="5" xr3:uid="{9BA83566-C962-4C2F-BE54-7DE70FFB175B}" name="heavyrail_miles"/>
     <tableColumn id="6" xr3:uid="{B314656D-75E6-48B6-8E62-F682D6C1A8C2}" name="lightrail_miles"/>
@@ -3064,9 +3067,9 @@
   <autoFilter ref="A1:E33" xr:uid="{72909F37-32CC-4777-BAF8-56EF443400DD}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{6059561D-B144-44A4-BD42-8A6CB47AE110}" name="year"/>
-    <tableColumn id="2" xr3:uid="{D8A3ABC2-F1D5-4278-9FC5-76DED278C85F}" name="amtrak_Energy_Intensity_BTUPerPaxMil" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{E65C9314-C120-4F4A-B346-84C59D802685}" name="CR_Energy_Intensity_BTUPerPaxMil" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{425B37B1-3EA8-495D-91F4-852DA9CC3D68}" name="HR_Energy_Intensity_BTUPerPaxMil" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D8A3ABC2-F1D5-4278-9FC5-76DED278C85F}" name="amtrak_Energy_Intensity_BTUPerPaxMil" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{E65C9314-C120-4F4A-B346-84C59D802685}" name="CR_Energy_Intensity_BTUPerPaxMil" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{425B37B1-3EA8-495D-91F4-852DA9CC3D68}" name="HR_Energy_Intensity_BTUPerPaxMil" dataDxfId="8"/>
     <tableColumn id="5" xr3:uid="{88F33EA8-F37C-4417-AC3E-4ECBF4C7F327}" name="LR_Energy_Intensity_BTUPerPaxMil"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3074,13 +3077,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{582D4DAA-0A5B-4D25-ABF1-823CB17290ED}" name="Fuel_Econs" displayName="Fuel_Econs" ref="A1:D1141" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{582D4DAA-0A5B-4D25-ABF1-823CB17290ED}" name="Fuel_Econs" displayName="Fuel_Econs" ref="A1:D1141" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
   <autoFilter ref="A1:D1141" xr:uid="{582D4DAA-0A5B-4D25-ABF1-823CB17290ED}"/>
   <tableColumns count="4">
-    <tableColumn id="2" xr3:uid="{A9C8722C-57C5-40ED-81D2-F9D452B57E3E}" name="veh_type" dataDxfId="85"/>
-    <tableColumn id="1" xr3:uid="{3C2D67BB-3546-42C7-9841-AE339E1104FD}" name="veh_subtype" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{0DD6F3F8-56C6-4110-A8A5-7C8CD018E715}" name="year" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{753CDE3B-EF5E-47F8-951F-924B91E92EDB}" name="mpg_gasoline_eq" dataDxfId="82"/>
+    <tableColumn id="2" xr3:uid="{A9C8722C-57C5-40ED-81D2-F9D452B57E3E}" name="veh_type" dataDxfId="86"/>
+    <tableColumn id="1" xr3:uid="{3C2D67BB-3546-42C7-9841-AE339E1104FD}" name="veh_subtype" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{0DD6F3F8-56C6-4110-A8A5-7C8CD018E715}" name="year" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{753CDE3B-EF5E-47F8-951F-924B91E92EDB}" name="mpg_gasoline_eq" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3092,20 +3095,21 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3BDF347B-2D3A-4649-97A7-2FA4EC519A2D}" name="state"/>
     <tableColumn id="2" xr3:uid="{6F628BBE-20DC-4499-BFB8-A1A5CC1B6D82}" name="year"/>
-    <tableColumn id="3" xr3:uid="{27339B8C-01F5-4D0E-A0DE-81D38807DD4F}" name="FR_million_tonmiles" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{27339B8C-01F5-4D0E-A0DE-81D38807DD4F}" name="FR_million_tonmiles" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{C901F22A-A043-4FE0-8C77-891B5FA3758C}" name="Table21" displayName="Table21" ref="A1:D56" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:D56" xr:uid="{C901F22A-A043-4FE0-8C77-891B5FA3758C}"/>
-  <tableColumns count="4">
-    <tableColumn id="2" xr3:uid="{F5A4F286-87E2-4E79-8A9B-680A1C2FAED3}" name="State" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{180BA1B0-69F9-4548-A8B9-F87BA72BD396}" name="CB" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{8161DDC3-4000-4841-89A1-08C8420F7E4E}" name="DR" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{9E575DE0-C23F-4F23-AC43-20D0423FD10F}" name="MB" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{C901F22A-A043-4FE0-8C77-891B5FA3758C}" name="Table21" displayName="Table21" ref="A1:E56" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E56" xr:uid="{C901F22A-A043-4FE0-8C77-891B5FA3758C}"/>
+  <tableColumns count="5">
+    <tableColumn id="2" xr3:uid="{F5A4F286-87E2-4E79-8A9B-680A1C2FAED3}" name="State" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{933F9A1A-A0A7-4F3E-8987-E1DBBEA5652B}" name="year" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{180BA1B0-69F9-4548-A8B9-F87BA72BD396}" name="CB" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{8161DDC3-4000-4841-89A1-08C8420F7E4E}" name="DR" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{9E575DE0-C23F-4F23-AC43-20D0423FD10F}" name="MB" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3116,66 +3120,66 @@
   <autoFilter ref="A1:AF39" xr:uid="{26DFE3D8-BF1F-4FA6-907B-327B6B0CEDAC}"/>
   <tableColumns count="32">
     <tableColumn id="1" xr3:uid="{62053B8D-9C72-4701-9AF7-43D88B9B22A4}" name="veh_type"/>
-    <tableColumn id="2" xr3:uid="{66DC8B15-DBCD-4BB7-A766-A8DB844E878B}" name="veh_subtype" dataDxfId="81"/>
-    <tableColumn id="3" xr3:uid="{5494E6D8-5555-4D07-A136-D2F095F89A0D}" name="2021" dataDxfId="80"/>
-    <tableColumn id="4" xr3:uid="{CB4CDFAB-90E2-419E-8EE6-8088731A718B}" name="2022" dataDxfId="79"/>
-    <tableColumn id="5" xr3:uid="{BC7EE75F-AFCD-4529-B49D-65B37D50E18B}" name="2023" dataDxfId="78"/>
-    <tableColumn id="6" xr3:uid="{2623A818-04D3-4CB7-9536-20CF33F0B445}" name="2024" dataDxfId="77"/>
-    <tableColumn id="7" xr3:uid="{C39B458D-DADB-4DC8-8072-5961431A9CC2}" name="2025" dataDxfId="76"/>
-    <tableColumn id="8" xr3:uid="{948F76BF-D2B4-4121-B3D8-5EDC8BE89BBD}" name="2026" dataDxfId="75"/>
-    <tableColumn id="9" xr3:uid="{86DCCC54-C9B2-482B-A28E-FB136851756A}" name="2027" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{1F24E1A2-102B-4F50-B2EF-531364FD506A}" name="2028" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{B5BD79DC-374C-41E2-BBE0-C4FA5CA7266B}" name="2029" dataDxfId="72"/>
-    <tableColumn id="12" xr3:uid="{6040F6C0-728F-4F56-82FA-8F335B346240}" name="2030" dataDxfId="71"/>
-    <tableColumn id="13" xr3:uid="{777D8B44-0C5D-412C-83B4-00F03632ECF9}" name="2031" dataDxfId="70"/>
-    <tableColumn id="14" xr3:uid="{9EC73B4B-E136-4AB8-B77D-C1FE60128A72}" name="2032" dataDxfId="69"/>
-    <tableColumn id="15" xr3:uid="{87DBED95-4E40-4F35-AC1E-B196183A1426}" name="2033" dataDxfId="68"/>
-    <tableColumn id="16" xr3:uid="{F1439027-BBF2-49AA-A591-3632F24804A1}" name="2034" dataDxfId="67"/>
-    <tableColumn id="17" xr3:uid="{F7968730-192F-404F-9B45-308DDE081907}" name="2035" dataDxfId="66"/>
-    <tableColumn id="18" xr3:uid="{7A7C733C-F5A6-49A9-BFF2-A495AEEB66C2}" name="2036" dataDxfId="65"/>
-    <tableColumn id="19" xr3:uid="{58026119-8B8F-4A3D-83CA-4C8B006005FF}" name="2037" dataDxfId="64"/>
-    <tableColumn id="20" xr3:uid="{0DC2964A-45E1-4675-9A45-6F69DA155672}" name="2038" dataDxfId="63"/>
-    <tableColumn id="21" xr3:uid="{84BBC27E-E152-41D2-9036-587EF7DB9FF2}" name="2039" dataDxfId="62"/>
-    <tableColumn id="22" xr3:uid="{3807A9C4-C050-4A3A-952A-5859AD2AE874}" name="2040" dataDxfId="61"/>
-    <tableColumn id="23" xr3:uid="{FF9A5B48-C7D9-4B91-84E5-63297F2C4FEC}" name="2041" dataDxfId="60"/>
-    <tableColumn id="24" xr3:uid="{8B5085CD-A302-4A03-B5EA-F22DABEA8C34}" name="2042" dataDxfId="59"/>
-    <tableColumn id="25" xr3:uid="{136F35CC-46CA-4CB2-AA82-25188F53F90B}" name="2043" dataDxfId="58"/>
-    <tableColumn id="26" xr3:uid="{D9C87554-6CC8-4B3B-873C-8198436EB206}" name="2044" dataDxfId="57"/>
-    <tableColumn id="27" xr3:uid="{A5A1C6D2-F476-404B-8688-89130BE3DF0D}" name="2045" dataDxfId="56"/>
-    <tableColumn id="28" xr3:uid="{88296D41-DBE1-4E61-96BF-AEF8FC13BE35}" name="2046" dataDxfId="55"/>
-    <tableColumn id="29" xr3:uid="{CE07A51A-2B10-4EA2-ACE8-6F4BE2476DCE}" name="2047" dataDxfId="54"/>
-    <tableColumn id="30" xr3:uid="{1DAC48BA-1924-498D-8FC3-861C248885FC}" name="2048" dataDxfId="53"/>
-    <tableColumn id="31" xr3:uid="{B688E9DA-A549-42F4-AB8B-FDE0EFCB9009}" name="2049" dataDxfId="52"/>
-    <tableColumn id="32" xr3:uid="{24389340-B3AB-4C24-8D9C-A0BD7675F042}" name="2050" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{66DC8B15-DBCD-4BB7-A766-A8DB844E878B}" name="veh_subtype" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{5494E6D8-5555-4D07-A136-D2F095F89A0D}" name="2021" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{CB4CDFAB-90E2-419E-8EE6-8088731A718B}" name="2022" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{BC7EE75F-AFCD-4529-B49D-65B37D50E18B}" name="2023" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{2623A818-04D3-4CB7-9536-20CF33F0B445}" name="2024" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{C39B458D-DADB-4DC8-8072-5961431A9CC2}" name="2025" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{948F76BF-D2B4-4121-B3D8-5EDC8BE89BBD}" name="2026" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{86DCCC54-C9B2-482B-A28E-FB136851756A}" name="2027" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{1F24E1A2-102B-4F50-B2EF-531364FD506A}" name="2028" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{B5BD79DC-374C-41E2-BBE0-C4FA5CA7266B}" name="2029" dataDxfId="73"/>
+    <tableColumn id="12" xr3:uid="{6040F6C0-728F-4F56-82FA-8F335B346240}" name="2030" dataDxfId="72"/>
+    <tableColumn id="13" xr3:uid="{777D8B44-0C5D-412C-83B4-00F03632ECF9}" name="2031" dataDxfId="71"/>
+    <tableColumn id="14" xr3:uid="{9EC73B4B-E136-4AB8-B77D-C1FE60128A72}" name="2032" dataDxfId="70"/>
+    <tableColumn id="15" xr3:uid="{87DBED95-4E40-4F35-AC1E-B196183A1426}" name="2033" dataDxfId="69"/>
+    <tableColumn id="16" xr3:uid="{F1439027-BBF2-49AA-A591-3632F24804A1}" name="2034" dataDxfId="68"/>
+    <tableColumn id="17" xr3:uid="{F7968730-192F-404F-9B45-308DDE081907}" name="2035" dataDxfId="67"/>
+    <tableColumn id="18" xr3:uid="{7A7C733C-F5A6-49A9-BFF2-A495AEEB66C2}" name="2036" dataDxfId="66"/>
+    <tableColumn id="19" xr3:uid="{58026119-8B8F-4A3D-83CA-4C8B006005FF}" name="2037" dataDxfId="65"/>
+    <tableColumn id="20" xr3:uid="{0DC2964A-45E1-4675-9A45-6F69DA155672}" name="2038" dataDxfId="64"/>
+    <tableColumn id="21" xr3:uid="{84BBC27E-E152-41D2-9036-587EF7DB9FF2}" name="2039" dataDxfId="63"/>
+    <tableColumn id="22" xr3:uid="{3807A9C4-C050-4A3A-952A-5859AD2AE874}" name="2040" dataDxfId="62"/>
+    <tableColumn id="23" xr3:uid="{FF9A5B48-C7D9-4B91-84E5-63297F2C4FEC}" name="2041" dataDxfId="61"/>
+    <tableColumn id="24" xr3:uid="{8B5085CD-A302-4A03-B5EA-F22DABEA8C34}" name="2042" dataDxfId="60"/>
+    <tableColumn id="25" xr3:uid="{136F35CC-46CA-4CB2-AA82-25188F53F90B}" name="2043" dataDxfId="59"/>
+    <tableColumn id="26" xr3:uid="{D9C87554-6CC8-4B3B-873C-8198436EB206}" name="2044" dataDxfId="58"/>
+    <tableColumn id="27" xr3:uid="{A5A1C6D2-F476-404B-8688-89130BE3DF0D}" name="2045" dataDxfId="57"/>
+    <tableColumn id="28" xr3:uid="{88296D41-DBE1-4E61-96BF-AEF8FC13BE35}" name="2046" dataDxfId="56"/>
+    <tableColumn id="29" xr3:uid="{CE07A51A-2B10-4EA2-ACE8-6F4BE2476DCE}" name="2047" dataDxfId="55"/>
+    <tableColumn id="30" xr3:uid="{1DAC48BA-1924-498D-8FC3-861C248885FC}" name="2048" dataDxfId="54"/>
+    <tableColumn id="31" xr3:uid="{B688E9DA-A549-42F4-AB8B-FDE0EFCB9009}" name="2049" dataDxfId="53"/>
+    <tableColumn id="32" xr3:uid="{24389340-B3AB-4C24-8D9C-A0BD7675F042}" name="2050" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}" name="AEO_VMT_Base" displayName="AEO_VMT_Base" ref="A1:C125" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}" name="AEO_VMT_Base" displayName="AEO_VMT_Base" ref="A1:C125" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="A1:C125" xr:uid="{3CAC199F-1E44-400D-AE49-2DF031458F28}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{51DE3611-329C-41B0-A4DB-52AE83C97AC8}" name="veh_type" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{591F901E-48BF-4AA2-83C5-3ABFD077C4E7}" name="year" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{68ED531E-CBD1-4FD0-B6FE-39DCA60A2D35}" name="VMT_AEO" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{51DE3611-329C-41B0-A4DB-52AE83C97AC8}" name="veh_type" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{591F901E-48BF-4AA2-83C5-3ABFD077C4E7}" name="year" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{68ED531E-CBD1-4FD0-B6FE-39DCA60A2D35}" name="VMT_AEO" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1316E024-4D78-4E5E-A3BE-D1D66BF710F0}" name="HPMS" displayName="HPMS" ref="A1:H743" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{1316E024-4D78-4E5E-A3BE-D1D66BF710F0}" name="HPMS" displayName="HPMS" ref="A1:H743" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A1:H743" xr:uid="{1316E024-4D78-4E5E-A3BE-D1D66BF710F0}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{8197FE9A-A39C-4187-B5AC-62137B98FA8C}" name="state" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{33E598CD-870F-42AB-891F-120C293216E4}" name="road_class" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{497DF0FF-D0A2-4A0F-AFE6-132C97C1B5AD}" name="area_type" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{776B704E-54DA-4B36-942C-A38CD577374B}" name="VMT" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{BDC6225D-BEFD-46A2-B173-8338BF6CD1D9}" name="ln_mile" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{24DAA4FA-2524-49F1-8BF5-F7D985D4CF64}" name="cntrln_mile" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{08E78B07-AE22-4A69-BADE-9D39986335D3}" name="AADT" dataDxfId="37"/>
-    <tableColumn id="7" xr3:uid="{863F524C-50D9-4550-847E-504CEE40EC23}" name="VMT_perln" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{8197FE9A-A39C-4187-B5AC-62137B98FA8C}" name="state" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{33E598CD-870F-42AB-891F-120C293216E4}" name="road_class" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{497DF0FF-D0A2-4A0F-AFE6-132C97C1B5AD}" name="area_type" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{776B704E-54DA-4B36-942C-A38CD577374B}" name="VMT" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{BDC6225D-BEFD-46A2-B173-8338BF6CD1D9}" name="ln_mile" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{24DAA4FA-2524-49F1-8BF5-F7D985D4CF64}" name="cntrln_mile" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{08E78B07-AE22-4A69-BADE-9D39986335D3}" name="AADT" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{863F524C-50D9-4550-847E-504CEE40EC23}" name="VMT_perln" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3186,8 +3190,8 @@
   <autoFilter ref="A1:D52" xr:uid="{AF7C35B9-8FE5-4041-A7B8-E1A84CB12C3D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{45CA7A43-AA6B-4C86-8B4D-AAB410C7E1C6}" name="state"/>
-    <tableColumn id="2" xr3:uid="{5CF42C05-08A7-42B5-BC47-0AEEE4AC6C72}" name="year" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{FEC27B6E-BBC0-45E0-8D54-901A00210403}" name="CO2eq_lbs_MWh" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{5CF42C05-08A7-42B5-BC47-0AEEE4AC6C72}" name="year" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{FEC27B6E-BBC0-45E0-8D54-901A00210403}" name="CO2eq_lbs_MWh" dataDxfId="35"/>
     <tableColumn id="4" xr3:uid="{2895651D-5EC8-4717-945D-3D007960FE15}" name="CO2eq_g_kWh"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3195,7 +3199,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7A91E0A4-8964-4E3A-BC3C-267B3185BA1C}" name="VMT_State_Allocation" displayName="VMT_State_Allocation" ref="A1:C1531" totalsRowShown="0" headerRowDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7A91E0A4-8964-4E3A-BC3C-267B3185BA1C}" name="VMT_State_Allocation" displayName="VMT_State_Allocation" ref="A1:C1531" totalsRowShown="0" headerRowDxfId="34">
   <autoFilter ref="A1:C1531" xr:uid="{365B7AAA-443F-4721-B58B-59C0701739EE}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{EEC20DE1-59BC-461D-9870-944562F1E1BA}" name="state"/>
@@ -3207,26 +3211,26 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{8F71A607-355D-4561-B371-DF64A33BAB60}" name="State_Prices" displayName="State_Prices" ref="A1:J52" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{8F71A607-355D-4561-B371-DF64A33BAB60}" name="State_Prices" displayName="State_Prices" ref="A1:J52" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A1:J52" xr:uid="{8F71A607-355D-4561-B371-DF64A33BAB60}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{FCA1C28F-7FB1-4E75-ABE4-772AFC6C788B}" name="source" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{8F610959-9FEF-4037-AD50-D15004FDEC97}" name="state " dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{DC14385D-FE79-4EBC-B031-AAF6DF063175}" name="gas_regular" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{30495008-5280-426E-A40F-3CBF7D9B9A92}" name="gas_mid" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{66FA34E8-985C-461A-9962-D27A2E7BC3B6}" name="gas_premium" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{9B04AF70-034B-4C94-AFF3-98D10D1FD236}" name="gas_diesel" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{2118497B-7145-40BC-9331-03F557AA7959}" name="electricity_retail_avg" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{ACAB8D01-5214-4549-830E-B7BF39440F10}" name="electricity_summer_capacity" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{E2BC6161-14F8-44FD-9F20-BBB936BC725E}" name="electricity_net_generation" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{EBA42203-1B14-46B5-AF40-8E9C9B3EBA3C}" name="electricity_retail_sales" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{FCA1C28F-7FB1-4E75-ABE4-772AFC6C788B}" name="source" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{8F610959-9FEF-4037-AD50-D15004FDEC97}" name="state " dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{DC14385D-FE79-4EBC-B031-AAF6DF063175}" name="gas_regular" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{30495008-5280-426E-A40F-3CBF7D9B9A92}" name="gas_mid" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{66FA34E8-985C-461A-9962-D27A2E7BC3B6}" name="gas_premium" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{9B04AF70-034B-4C94-AFF3-98D10D1FD236}" name="gas_diesel" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{2118497B-7145-40BC-9331-03F557AA7959}" name="electricity_retail_avg" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{ACAB8D01-5214-4549-830E-B7BF39440F10}" name="electricity_summer_capacity" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{E2BC6161-14F8-44FD-9F20-BBB936BC725E}" name="electricity_net_generation" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{EBA42203-1B14-46B5-AF40-8E9C9B3EBA3C}" name="electricity_retail_sales" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8B4E7E83-799B-427A-A3DA-A7D8C89C054B}" name="Bike_Ped" displayName="Bike_Ped" ref="A1:E22" totalsRowShown="0" headerRowDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8B4E7E83-799B-427A-A3DA-A7D8C89C054B}" name="Bike_Ped" displayName="Bike_Ped" ref="A1:E22" totalsRowShown="0" headerRowDxfId="21">
   <autoFilter ref="A1:E22" xr:uid="{8B4E7E83-799B-427A-A3DA-A7D8C89C054B}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{16080A00-286A-46F0-B3AC-AB7A89FB70FC}" name="facility_type"/>
@@ -42707,790 +42711,958 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C856A2-2644-45CE-8C61-85605A6B28DC}">
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
         <v>334</v>
       </c>
       <c r="B1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="23" t="s">
         <v>335</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="D1" s="23" t="s">
         <v>336</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="E1" s="23" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C2" s="24">
         <v>0</v>
       </c>
-      <c r="C2" s="24">
+      <c r="D2" s="24">
         <v>1820969</v>
       </c>
-      <c r="D2" s="24">
+      <c r="E2" s="24">
         <v>4544203</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C3" s="24">
         <v>0</v>
       </c>
-      <c r="C3" s="24">
+      <c r="D3" s="24">
         <v>10146650</v>
       </c>
-      <c r="D3" s="24">
+      <c r="E3" s="24">
         <v>6650385</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="24" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C4" s="24">
         <v>0</v>
       </c>
-      <c r="C4" s="24">
+      <c r="D4" s="24">
         <v>13251409</v>
       </c>
-      <c r="D4" s="24">
+      <c r="E4" s="24">
         <v>4668133</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="24" t="s">
         <v>100</v>
       </c>
       <c r="B5" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C5" s="24">
         <v>0</v>
       </c>
-      <c r="C5" s="24">
+      <c r="D5" s="24">
         <v>128251</v>
       </c>
-      <c r="D5" s="24">
+      <c r="E5" s="24">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C6" s="24">
         <v>686829</v>
       </c>
-      <c r="C6" s="24">
+      <c r="D6" s="24">
         <v>8850838</v>
       </c>
-      <c r="D6" s="24">
+      <c r="E6" s="24">
         <v>49557933</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="24" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C7" s="24">
         <v>17653453</v>
       </c>
-      <c r="C7" s="24">
+      <c r="D7" s="24">
         <v>88205270</v>
       </c>
-      <c r="D7" s="24">
+      <c r="E7" s="24">
         <v>330675119</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="24" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C8" s="24">
         <v>3275162</v>
       </c>
-      <c r="C8" s="24">
+      <c r="D8" s="24">
         <v>18116638</v>
       </c>
-      <c r="D8" s="24">
+      <c r="E8" s="24">
         <v>49855214</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="24" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C9" s="24">
         <v>1302927</v>
       </c>
-      <c r="C9" s="24">
+      <c r="D9" s="24">
         <v>9462995</v>
       </c>
-      <c r="D9" s="24">
+      <c r="E9" s="24">
         <v>23037923</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="24" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C10" s="24">
         <v>0</v>
       </c>
-      <c r="C10" s="24">
+      <c r="D10" s="24">
         <v>19685883</v>
       </c>
-      <c r="D10" s="24">
+      <c r="E10" s="24">
         <v>38872603</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="24" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C11" s="24">
         <v>0</v>
       </c>
-      <c r="C11" s="24">
+      <c r="D11" s="24">
         <v>8098492</v>
       </c>
-      <c r="D11" s="24">
+      <c r="E11" s="24">
         <v>8984139</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C12" s="24">
         <v>1206534</v>
       </c>
-      <c r="C12" s="24">
+      <c r="D12" s="24">
         <v>80295496</v>
       </c>
-      <c r="D12" s="24">
+      <c r="E12" s="24">
         <v>124877739</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="24" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C13" s="24">
         <v>3708274</v>
       </c>
-      <c r="C13" s="24">
+      <c r="D13" s="24">
         <v>28298863</v>
       </c>
-      <c r="D13" s="24">
+      <c r="E13" s="24">
         <v>40629519</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="24" t="s">
         <v>110</v>
       </c>
       <c r="B14" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C14" s="24">
         <v>0</v>
       </c>
-      <c r="C14" s="24">
+      <c r="D14" s="24">
         <v>372212</v>
       </c>
-      <c r="D14" s="24">
+      <c r="E14" s="24">
         <v>422892</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="24" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C15" s="24">
         <v>1888935</v>
       </c>
-      <c r="C15" s="24">
+      <c r="D15" s="24">
         <v>9218028</v>
       </c>
-      <c r="D15" s="24">
+      <c r="E15" s="24">
         <v>20454917</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="24" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C16" s="24">
         <v>0</v>
       </c>
-      <c r="C16" s="24">
+      <c r="D16" s="24">
         <v>16204926</v>
       </c>
-      <c r="D16" s="24">
+      <c r="E16" s="24">
         <v>11203459</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="24" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C17" s="24">
         <v>0</v>
       </c>
-      <c r="C17" s="24">
+      <c r="D17" s="24">
         <v>1792488</v>
       </c>
-      <c r="D17" s="24">
+      <c r="E17" s="24">
         <v>4418282</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="24" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C18" s="24">
         <v>316684</v>
       </c>
-      <c r="C18" s="24">
+      <c r="D18" s="24">
         <v>51817490</v>
       </c>
-      <c r="D18" s="24">
+      <c r="E18" s="24">
         <v>103734267</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="24" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C19" s="24">
         <v>450990</v>
       </c>
-      <c r="C19" s="24">
+      <c r="D19" s="24">
         <v>18241770</v>
       </c>
-      <c r="D19" s="24">
+      <c r="E19" s="24">
         <v>19286019</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="24" t="s">
         <v>19</v>
       </c>
       <c r="B20" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C20" s="24">
         <v>366540</v>
       </c>
-      <c r="C20" s="24">
+      <c r="D20" s="24">
         <v>7847064</v>
       </c>
-      <c r="D20" s="24">
+      <c r="E20" s="24">
         <v>7512599</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="24" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C21" s="24">
         <v>0</v>
       </c>
-      <c r="C21" s="24">
+      <c r="D21" s="24">
         <v>35520308</v>
       </c>
-      <c r="D21" s="24">
+      <c r="E21" s="24">
         <v>14087087</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="24" t="s">
         <v>21</v>
       </c>
       <c r="B22" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C22" s="24">
         <v>0</v>
       </c>
-      <c r="C22" s="24">
+      <c r="D22" s="24">
         <v>10323437</v>
       </c>
-      <c r="D22" s="24">
+      <c r="E22" s="24">
         <v>15649937</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="24" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C23" s="24">
         <v>3104521</v>
       </c>
-      <c r="C23" s="24">
+      <c r="D23" s="24">
         <v>31031514</v>
       </c>
-      <c r="D23" s="24">
+      <c r="E23" s="24">
         <v>43374617</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="24" t="s">
         <v>23</v>
       </c>
       <c r="B24" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C24" s="24">
         <v>6636014</v>
       </c>
-      <c r="C24" s="24">
+      <c r="D24" s="24">
         <v>26146936</v>
       </c>
-      <c r="D24" s="24">
+      <c r="E24" s="24">
         <v>48391900</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="24" t="s">
         <v>22</v>
       </c>
       <c r="B25" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C25" s="24">
         <v>265210</v>
       </c>
-      <c r="C25" s="24">
+      <c r="D25" s="24">
         <v>10826516</v>
       </c>
-      <c r="D25" s="24">
+      <c r="E25" s="24">
         <v>4137861</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="24" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C26" s="24">
         <v>432546</v>
       </c>
-      <c r="C26" s="24">
+      <c r="D26" s="24">
         <v>50261455</v>
       </c>
-      <c r="D26" s="24">
+      <c r="E26" s="24">
         <v>49939298</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="24" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C27" s="24">
         <v>217003</v>
       </c>
-      <c r="C27" s="24">
+      <c r="D27" s="24">
         <v>37519099</v>
       </c>
-      <c r="D27" s="24">
+      <c r="E27" s="24">
         <v>44630214</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="24" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C28" s="24">
         <v>0</v>
       </c>
-      <c r="C28" s="24">
+      <c r="D28" s="24">
         <v>25977732</v>
       </c>
-      <c r="D28" s="24">
+      <c r="E28" s="24">
         <v>29294533</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="24" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C29" s="24">
         <v>0</v>
       </c>
-      <c r="C29" s="24">
+      <c r="D29" s="24">
         <v>10355411</v>
       </c>
-      <c r="D29" s="24">
+      <c r="E29" s="24">
         <v>3281232</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="24" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C30" s="24">
         <v>145031</v>
       </c>
-      <c r="C30" s="24">
+      <c r="D30" s="24">
         <v>2994570</v>
       </c>
-      <c r="D30" s="24">
+      <c r="E30" s="24">
         <v>3791255</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="24" t="s">
         <v>244</v>
       </c>
       <c r="B31" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C31" s="24">
         <v>2548230</v>
       </c>
-      <c r="C31" s="24">
+      <c r="D31" s="24">
         <v>49037696</v>
       </c>
-      <c r="D31" s="24">
+      <c r="E31" s="24">
         <v>37124123</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="24" t="s">
         <v>36</v>
       </c>
       <c r="B32" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C32" s="24">
         <v>0</v>
       </c>
-      <c r="C32" s="24">
+      <c r="D32" s="24">
         <v>4584891</v>
       </c>
-      <c r="D32" s="24">
+      <c r="E32" s="24">
         <v>1934311</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="24" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C33" s="24">
         <v>0</v>
       </c>
-      <c r="C33" s="24">
+      <c r="D33" s="24">
         <v>4815160</v>
       </c>
-      <c r="D33" s="24">
+      <c r="E33" s="24">
         <v>6276073</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="24" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C34" s="24">
         <v>3969821</v>
       </c>
-      <c r="C34" s="24">
+      <c r="D34" s="24">
         <v>875174</v>
       </c>
-      <c r="D34" s="24">
+      <c r="E34" s="24">
         <v>2401459</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="24" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C35" s="24">
         <v>30328896</v>
       </c>
-      <c r="C35" s="24">
+      <c r="D35" s="24">
         <v>22632079</v>
       </c>
-      <c r="D35" s="24">
+      <c r="E35" s="24">
         <v>85248950</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="24" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C36" s="24">
         <v>331362</v>
       </c>
-      <c r="C36" s="24">
+      <c r="D36" s="24">
         <v>4270615</v>
       </c>
-      <c r="D36" s="24">
+      <c r="E36" s="24">
         <v>11058565</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="24" t="s">
         <v>31</v>
       </c>
       <c r="B37" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C37" s="24">
         <v>410090</v>
       </c>
-      <c r="C37" s="24">
+      <c r="D37" s="24">
         <v>13795616</v>
       </c>
-      <c r="D37" s="24">
+      <c r="E37" s="24">
         <v>22752296</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="24" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C38" s="24">
         <v>18162255</v>
       </c>
-      <c r="C38" s="24">
+      <c r="D38" s="24">
         <v>62282351</v>
       </c>
-      <c r="D38" s="24">
+      <c r="E38" s="24">
         <v>182735062</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="24" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C39" s="24">
         <v>515002</v>
       </c>
-      <c r="C39" s="24">
+      <c r="D39" s="24">
         <v>37821824</v>
       </c>
-      <c r="D39" s="24">
+      <c r="E39" s="24">
         <v>56939993</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="24" t="s">
         <v>38</v>
       </c>
       <c r="B40" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C40" s="24">
         <v>92708</v>
       </c>
-      <c r="C40" s="24">
+      <c r="D40" s="24">
         <v>19161183</v>
       </c>
-      <c r="D40" s="24">
+      <c r="E40" s="24">
         <v>7918742</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="24" t="s">
         <v>39</v>
       </c>
       <c r="B41" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C41" s="24">
         <v>3750422</v>
       </c>
-      <c r="C41" s="24">
+      <c r="D41" s="24">
         <v>13160147</v>
       </c>
-      <c r="D41" s="24">
+      <c r="E41" s="24">
         <v>33429198</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="24" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C42" s="24">
         <v>4926331</v>
       </c>
-      <c r="C42" s="24">
+      <c r="D42" s="24">
         <v>44238102</v>
       </c>
-      <c r="D42" s="24">
+      <c r="E42" s="24">
         <v>88986984</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="24" t="s">
         <v>87</v>
       </c>
       <c r="B43" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C43" s="24">
         <v>0</v>
       </c>
-      <c r="C43" s="24">
+      <c r="D43" s="24">
         <v>1401597</v>
       </c>
-      <c r="D43" s="24">
+      <c r="E43" s="24">
         <v>5328065</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="24" t="s">
         <v>41</v>
       </c>
       <c r="B44" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C44" s="24">
         <v>0</v>
       </c>
-      <c r="C44" s="24">
+      <c r="D44" s="24">
         <v>2424533</v>
       </c>
-      <c r="D44" s="24">
+      <c r="E44" s="24">
         <v>8922598</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="24" t="s">
         <v>245</v>
       </c>
       <c r="B45" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C45" s="24">
         <v>701719</v>
       </c>
-      <c r="C45" s="24">
+      <c r="D45" s="24">
         <v>9490872</v>
       </c>
-      <c r="D45" s="24">
+      <c r="E45" s="24">
         <v>10435969</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="24" t="s">
         <v>42</v>
       </c>
       <c r="B46" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C46" s="24">
         <v>0</v>
       </c>
-      <c r="C46" s="24">
+      <c r="D46" s="24">
         <v>5071774</v>
       </c>
-      <c r="D46" s="24">
+      <c r="E46" s="24">
         <v>1450451</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="24" t="s">
         <v>43</v>
       </c>
       <c r="B47" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C47" s="24">
         <v>326460</v>
       </c>
-      <c r="C47" s="24">
+      <c r="D47" s="24">
         <v>31402928</v>
       </c>
-      <c r="D47" s="24">
+      <c r="E47" s="24">
         <v>21251959</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="24" t="s">
         <v>44</v>
       </c>
       <c r="B48" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C48" s="24">
         <v>14830278</v>
       </c>
-      <c r="C48" s="24">
+      <c r="D48" s="24">
         <v>75039448</v>
       </c>
-      <c r="D48" s="24">
+      <c r="E48" s="24">
         <v>140051617</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="24" t="s">
         <v>45</v>
       </c>
       <c r="B49" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C49" s="24">
         <v>904101</v>
       </c>
-      <c r="C49" s="24">
+      <c r="D49" s="24">
         <v>3319266</v>
       </c>
-      <c r="D49" s="24">
+      <c r="E49" s="24">
         <v>20872218</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="24" t="s">
         <v>47</v>
       </c>
       <c r="B50" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C50" s="24">
         <v>4031352</v>
       </c>
-      <c r="C50" s="24">
+      <c r="D50" s="24">
         <v>13200660</v>
       </c>
-      <c r="D50" s="24">
+      <c r="E50" s="24">
         <v>44091053</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="24" t="s">
         <v>338</v>
       </c>
       <c r="B51" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C51" s="24">
         <v>0</v>
       </c>
-      <c r="C51" s="24">
+      <c r="D51" s="24">
         <v>349850</v>
       </c>
-      <c r="D51" s="24">
+      <c r="E51" s="24">
         <v>291988</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="24" t="s">
         <v>46</v>
       </c>
       <c r="B52" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C52" s="24">
         <v>2005605</v>
       </c>
-      <c r="C52" s="24">
+      <c r="D52" s="24">
         <v>13420628</v>
       </c>
-      <c r="D52" s="24">
+      <c r="E52" s="24">
         <v>3731759</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="24" t="s">
         <v>48</v>
       </c>
       <c r="B53" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C53" s="24">
         <v>15447471</v>
       </c>
-      <c r="C53" s="24">
+      <c r="D53" s="24">
         <v>28877650</v>
       </c>
-      <c r="D53" s="24">
+      <c r="E53" s="24">
         <v>83332487</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="24" t="s">
         <v>50</v>
       </c>
       <c r="B54" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C54" s="24">
         <v>880327</v>
       </c>
-      <c r="C54" s="24">
+      <c r="D54" s="24">
         <v>16792018</v>
       </c>
-      <c r="D54" s="24">
+      <c r="E54" s="24">
         <v>33284438</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="24" t="s">
         <v>49</v>
       </c>
       <c r="B55" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C55" s="24">
         <v>0</v>
       </c>
-      <c r="C55" s="24">
+      <c r="D55" s="24">
         <v>2671749</v>
       </c>
-      <c r="D55" s="24">
+      <c r="E55" s="24">
         <v>9309564</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="24" t="s">
         <v>51</v>
       </c>
       <c r="B56" s="24">
+        <v>2019</v>
+      </c>
+      <c r="C56" s="24">
         <v>0</v>
       </c>
-      <c r="C56" s="24">
+      <c r="D56" s="24">
         <v>1673521</v>
       </c>
-      <c r="D56" s="24">
+      <c r="E56" s="24">
         <v>2044125</v>
       </c>
     </row>
@@ -88801,6 +88973,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -88982,22 +89169,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -89013,28 +89209,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pushing my fixes to minor things
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51A45467-8339-4845-8290-F195DF3AAA88}"/>
   <bookViews>
-    <workbookView xWindow="270" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="29070" yWindow="-14715" windowWidth="16440" windowHeight="29040" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
     <definedName name="up_lpg">'[1]Baseline Parameters'!$C$67</definedName>
     <definedName name="ViewMode">'[2]Project Inputs'!$B$299:$B$300</definedName>
   </definedNames>
-  <calcPr calcId="191028" calcOnSave="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3106,10 +3106,10 @@
   <autoFilter ref="A1:E56" xr:uid="{C901F22A-A043-4FE0-8C77-891B5FA3758C}"/>
   <tableColumns count="5">
     <tableColumn id="2" xr3:uid="{F5A4F286-87E2-4E79-8A9B-680A1C2FAED3}" name="State" dataDxfId="4"/>
-    <tableColumn id="1" xr3:uid="{933F9A1A-A0A7-4F3E-8987-E1DBBEA5652B}" name="year" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{180BA1B0-69F9-4548-A8B9-F87BA72BD396}" name="CB" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{8161DDC3-4000-4841-89A1-08C8420F7E4E}" name="DR" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{9E575DE0-C23F-4F23-AC43-20D0423FD10F}" name="MB" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{933F9A1A-A0A7-4F3E-8987-E1DBBEA5652B}" name="year" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{180BA1B0-69F9-4548-A8B9-F87BA72BD396}" name="CB" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{8161DDC3-4000-4841-89A1-08C8420F7E4E}" name="DR" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{9E575DE0-C23F-4F23-AC43-20D0423FD10F}" name="MB" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -88973,21 +88973,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -89169,31 +89154,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -89209,4 +89185,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AD81DBB-41E8-4D5D-9C32-6323A696B3D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Small Fixes smoothing things out
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51A45467-8339-4845-8290-F195DF3AAA88}"/>
   <bookViews>
-    <workbookView xWindow="29070" yWindow="-14715" windowWidth="16440" windowHeight="29040" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -2234,6 +2234,7 @@
       <sheetName val="Key Inputs"/>
       <sheetName val="Baseline Parameters"/>
       <sheetName val="Custom Project Inputs"/>
+      <sheetName val="Custom"/>
       <sheetName val="Strategy Parameters"/>
       <sheetName val="Cost Parameters"/>
       <sheetName val="Scenario Testing"/>
@@ -2274,7 +2275,6 @@
       <sheetName val="Freight"/>
       <sheetName val="EVSE"/>
       <sheetName val="RoadwayExp"/>
-      <sheetName val="Custom"/>
       <sheetName val="HPMS_Data"/>
       <sheetName val="FuelPrices"/>
       <sheetName val="EmRate_Multipliers"/>
@@ -2322,7 +2322,8 @@
       <sheetData sheetId="15"/>
       <sheetData sheetId="16"/>
       <sheetData sheetId="17"/>
-      <sheetData sheetId="18">
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19">
         <row r="6">
           <cell r="B6">
             <v>1385678.0070000002</v>
@@ -2339,7 +2340,6 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="19"/>
       <sheetData sheetId="20"/>
       <sheetData sheetId="21"/>
       <sheetData sheetId="22"/>
@@ -88973,6 +88973,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -89154,15 +89163,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -89170,6 +89170,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -89183,14 +89191,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fixed NHS and Tech Frac issue
</commit_message>
<xml_diff>
--- a/data/1.Raw_Data.xlsx
+++ b/data/1.Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camsys-my.sharepoint.com/personal/slarue_camsys_com/Documents/Documents/idot_github_puller/TEACART/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51A45467-8339-4845-8290-F195DF3AAA88}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{1FBCA57C-6DC9-49DB-92F9-9F72A168ADC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF5A304C-F499-4F31-8C49-1CFB71281F4F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="955" firstSheet="14" activeTab="21" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
+    <workbookView xWindow="29070" yWindow="-14715" windowWidth="16440" windowHeight="29040" tabRatio="955" firstSheet="12" activeTab="17" xr2:uid="{426A841F-B111-4A0D-9E3D-FA64A226CE83}"/>
   </bookViews>
   <sheets>
     <sheet name="State_Populations" sheetId="1" r:id="rId1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8748" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8748" uniqueCount="335">
   <si>
     <t>state</t>
   </si>
@@ -1018,18 +1018,6 @@
   </si>
   <si>
     <t>percEVstock_ACCIIACT</t>
-  </si>
-  <si>
-    <t>Heavy Duty Truck</t>
-  </si>
-  <si>
-    <t>Light Duty Truck</t>
-  </si>
-  <si>
-    <t>Medium Duty Truck</t>
-  </si>
-  <si>
-    <t>Passenger Car</t>
   </si>
   <si>
     <t>amtrak_riders</t>
@@ -5261,7 +5249,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>78</v>
@@ -5278,10 +5266,10 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B2" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C2">
         <v>327</v>
@@ -5295,7 +5283,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B3" t="s">
         <v>90</v>
@@ -5312,7 +5300,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B4" t="s">
         <v>157</v>
@@ -5329,7 +5317,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B5" t="s">
         <v>80</v>
@@ -5346,10 +5334,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B6" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C6">
         <v>150</v>
@@ -5363,7 +5351,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B7" t="s">
         <v>90</v>
@@ -5380,7 +5368,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B8" t="s">
         <v>157</v>
@@ -5397,7 +5385,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B9" t="s">
         <v>80</v>
@@ -5414,10 +5402,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>321</v>
+      </c>
+      <c r="B10" t="s">
         <v>325</v>
-      </c>
-      <c r="B10" t="s">
-        <v>329</v>
       </c>
       <c r="C10">
         <v>203.25</v>
@@ -5431,7 +5419,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B11" t="s">
         <v>90</v>
@@ -5448,7 +5436,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B12" t="s">
         <v>157</v>
@@ -5465,7 +5453,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B13" t="s">
         <v>80</v>
@@ -5482,10 +5470,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B14" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -5499,7 +5487,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B15" t="s">
         <v>90</v>
@@ -5516,7 +5504,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B16" t="s">
         <v>157</v>
@@ -5533,7 +5521,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B17" t="s">
         <v>80</v>
@@ -5550,10 +5538,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B18" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C18">
         <v>150</v>
@@ -5567,7 +5555,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B19" t="s">
         <v>90</v>
@@ -5584,7 +5572,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B20" t="s">
         <v>157</v>
@@ -5601,7 +5589,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B21" t="s">
         <v>157</v>
@@ -5618,7 +5606,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B22" t="s">
         <v>80</v>
@@ -19413,7 +19401,7 @@
         <v>198</v>
       </c>
       <c r="N1" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
@@ -19875,10 +19863,10 @@
         <v>197</v>
       </c>
       <c r="D1" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E1" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -19951,7 +19939,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B6" t="s">
         <v>210</v>
@@ -20099,7 +20087,7 @@
         <v>174</v>
       </c>
       <c r="B6" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C6">
         <v>0.24</v>
@@ -20110,7 +20098,7 @@
         <v>156</v>
       </c>
       <c r="B7" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C7">
         <v>0.21</v>
@@ -20121,7 +20109,7 @@
         <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C8">
         <v>0.28999999999999998</v>
@@ -20132,7 +20120,7 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -20143,7 +20131,7 @@
         <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -20154,7 +20142,7 @@
         <v>298</v>
       </c>
       <c r="B11" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -21689,7 +21677,7 @@
   <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.6328125" customWidth="1"/>
     <col min="4" max="4" width="18.54296875" customWidth="1"/>
     <col min="5" max="5" width="17.453125" customWidth="1"/>
@@ -21722,7 +21710,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B2">
         <v>2021</v>
@@ -21745,7 +21733,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B3">
         <v>2022</v>
@@ -21768,7 +21756,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B4">
         <v>2023</v>
@@ -21791,7 +21779,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B5">
         <v>2024</v>
@@ -21814,7 +21802,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B6">
         <v>2025</v>
@@ -21837,7 +21825,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B7">
         <v>2026</v>
@@ -21860,7 +21848,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B8">
         <v>2027</v>
@@ -21883,7 +21871,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B9">
         <v>2028</v>
@@ -21906,7 +21894,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B10">
         <v>2029</v>
@@ -21929,7 +21917,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B11">
         <v>2030</v>
@@ -21952,7 +21940,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B12">
         <v>2031</v>
@@ -21975,7 +21963,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B13">
         <v>2032</v>
@@ -21998,7 +21986,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B14">
         <v>2033</v>
@@ -22021,7 +22009,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B15">
         <v>2034</v>
@@ -22044,7 +22032,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B16">
         <v>2035</v>
@@ -22067,7 +22055,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B17">
         <v>2036</v>
@@ -22090,7 +22078,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B18">
         <v>2037</v>
@@ -22113,7 +22101,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B19">
         <v>2038</v>
@@ -22136,7 +22124,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B20">
         <v>2039</v>
@@ -22159,7 +22147,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B21">
         <v>2040</v>
@@ -22182,7 +22170,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B22">
         <v>2041</v>
@@ -22205,7 +22193,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B23">
         <v>2042</v>
@@ -22228,7 +22216,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B24">
         <v>2043</v>
@@ -22251,7 +22239,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B25">
         <v>2044</v>
@@ -22274,7 +22262,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B26">
         <v>2045</v>
@@ -22297,7 +22285,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B27">
         <v>2046</v>
@@ -22320,7 +22308,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B28">
         <v>2047</v>
@@ -22343,7 +22331,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B29">
         <v>2048</v>
@@ -22366,7 +22354,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B30">
         <v>2049</v>
@@ -22389,7 +22377,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>308</v>
+        <v>185</v>
       </c>
       <c r="B31">
         <v>2050</v>
@@ -22412,7 +22400,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B32">
         <v>2021</v>
@@ -22435,7 +22423,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B33">
         <v>2022</v>
@@ -22458,7 +22446,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B34">
         <v>2023</v>
@@ -22481,7 +22469,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B35">
         <v>2024</v>
@@ -22504,7 +22492,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B36">
         <v>2025</v>
@@ -22527,7 +22515,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B37">
         <v>2026</v>
@@ -22550,7 +22538,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B38">
         <v>2027</v>
@@ -22573,7 +22561,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B39">
         <v>2028</v>
@@ -22596,7 +22584,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B40">
         <v>2029</v>
@@ -22619,7 +22607,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B41">
         <v>2030</v>
@@ -22642,7 +22630,7 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B42">
         <v>2031</v>
@@ -22665,7 +22653,7 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B43">
         <v>2032</v>
@@ -22688,7 +22676,7 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B44">
         <v>2033</v>
@@ -22711,7 +22699,7 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B45">
         <v>2034</v>
@@ -22734,7 +22722,7 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B46">
         <v>2035</v>
@@ -22757,7 +22745,7 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B47">
         <v>2036</v>
@@ -22780,7 +22768,7 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B48">
         <v>2037</v>
@@ -22803,7 +22791,7 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B49">
         <v>2038</v>
@@ -22826,7 +22814,7 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B50">
         <v>2039</v>
@@ -22849,7 +22837,7 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B51">
         <v>2040</v>
@@ -22872,7 +22860,7 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B52">
         <v>2041</v>
@@ -22895,7 +22883,7 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B53">
         <v>2042</v>
@@ -22918,7 +22906,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B54">
         <v>2043</v>
@@ -22941,7 +22929,7 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B55">
         <v>2044</v>
@@ -22964,7 +22952,7 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B56">
         <v>2045</v>
@@ -22987,7 +22975,7 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B57">
         <v>2046</v>
@@ -23010,7 +22998,7 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B58">
         <v>2047</v>
@@ -23033,7 +23021,7 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B59">
         <v>2048</v>
@@ -23056,7 +23044,7 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B60">
         <v>2049</v>
@@ -23079,7 +23067,7 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>309</v>
+        <v>184</v>
       </c>
       <c r="B61">
         <v>2050</v>
@@ -23102,7 +23090,7 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B62">
         <v>2021</v>
@@ -23125,7 +23113,7 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B63">
         <v>2022</v>
@@ -23148,7 +23136,7 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B64">
         <v>2023</v>
@@ -23171,7 +23159,7 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B65">
         <v>2024</v>
@@ -23194,7 +23182,7 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B66">
         <v>2025</v>
@@ -23217,7 +23205,7 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B67">
         <v>2026</v>
@@ -23240,7 +23228,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B68">
         <v>2027</v>
@@ -23263,7 +23251,7 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B69">
         <v>2028</v>
@@ -23286,7 +23274,7 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B70">
         <v>2029</v>
@@ -23309,7 +23297,7 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B71">
         <v>2030</v>
@@ -23332,7 +23320,7 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B72">
         <v>2031</v>
@@ -23355,7 +23343,7 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B73">
         <v>2032</v>
@@ -23378,7 +23366,7 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B74">
         <v>2033</v>
@@ -23401,7 +23389,7 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B75">
         <v>2034</v>
@@ -23424,7 +23412,7 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B76">
         <v>2035</v>
@@ -23447,7 +23435,7 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B77">
         <v>2036</v>
@@ -23470,7 +23458,7 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B78">
         <v>2037</v>
@@ -23493,7 +23481,7 @@
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B79">
         <v>2038</v>
@@ -23516,7 +23504,7 @@
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B80">
         <v>2039</v>
@@ -23539,7 +23527,7 @@
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B81">
         <v>2040</v>
@@ -23562,7 +23550,7 @@
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B82">
         <v>2041</v>
@@ -23585,7 +23573,7 @@
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B83">
         <v>2042</v>
@@ -23608,7 +23596,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B84">
         <v>2043</v>
@@ -23631,7 +23619,7 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B85">
         <v>2044</v>
@@ -23654,7 +23642,7 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B86">
         <v>2045</v>
@@ -23677,7 +23665,7 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B87">
         <v>2046</v>
@@ -23700,7 +23688,7 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B88">
         <v>2047</v>
@@ -23723,7 +23711,7 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B89">
         <v>2048</v>
@@ -23746,7 +23734,7 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B90">
         <v>2049</v>
@@ -23769,7 +23757,7 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>310</v>
+        <v>210</v>
       </c>
       <c r="B91">
         <v>2050</v>
@@ -23792,7 +23780,7 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B92">
         <v>2021</v>
@@ -23815,7 +23803,7 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B93">
         <v>2022</v>
@@ -23838,7 +23826,7 @@
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B94">
         <v>2023</v>
@@ -23861,7 +23849,7 @@
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B95">
         <v>2024</v>
@@ -23884,7 +23872,7 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B96">
         <v>2025</v>
@@ -23907,7 +23895,7 @@
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B97">
         <v>2026</v>
@@ -23930,7 +23918,7 @@
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B98">
         <v>2027</v>
@@ -23953,7 +23941,7 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B99">
         <v>2028</v>
@@ -23976,7 +23964,7 @@
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B100">
         <v>2029</v>
@@ -23999,7 +23987,7 @@
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B101">
         <v>2030</v>
@@ -24022,7 +24010,7 @@
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B102">
         <v>2031</v>
@@ -24045,7 +24033,7 @@
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B103">
         <v>2032</v>
@@ -24068,7 +24056,7 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B104">
         <v>2033</v>
@@ -24091,7 +24079,7 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B105">
         <v>2034</v>
@@ -24114,7 +24102,7 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B106">
         <v>2035</v>
@@ -24137,7 +24125,7 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B107">
         <v>2036</v>
@@ -24160,7 +24148,7 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B108">
         <v>2037</v>
@@ -24183,7 +24171,7 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B109">
         <v>2038</v>
@@ -24206,7 +24194,7 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B110">
         <v>2039</v>
@@ -24229,7 +24217,7 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B111">
         <v>2040</v>
@@ -24252,7 +24240,7 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B112">
         <v>2041</v>
@@ -24275,7 +24263,7 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B113">
         <v>2042</v>
@@ -24298,7 +24286,7 @@
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B114">
         <v>2043</v>
@@ -24321,7 +24309,7 @@
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B115">
         <v>2044</v>
@@ -24344,7 +24332,7 @@
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B116">
         <v>2045</v>
@@ -24367,7 +24355,7 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B117">
         <v>2046</v>
@@ -24390,7 +24378,7 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B118">
         <v>2047</v>
@@ -24413,7 +24401,7 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B119">
         <v>2048</v>
@@ -24436,7 +24424,7 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B120">
         <v>2049</v>
@@ -24459,7 +24447,7 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>311</v>
+        <v>196</v>
       </c>
       <c r="B121">
         <v>2050</v>
@@ -24507,16 +24495,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D1" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="E1" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F1" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -41555,16 +41543,16 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C1" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D1" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E1" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -42137,7 +42125,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -42716,19 +42704,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="D1" s="23" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -43566,7 +43554,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="24" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="B51" s="24">
         <v>2019</v>
@@ -88973,15 +88961,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010074FD77E8DF26214E8A3D3B6DC2CB3456" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="540a33700147f10daa2148a31047025c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc9650b-f3ad-4a63-850f-e6e893a434d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="78fd43bcea03852b8aad0c2a75101358" ns2:_="">
     <xsd:import namespace="1bc9650b-f3ad-4a63-850f-e6e893a434d8"/>
@@ -89163,6 +89142,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -89170,14 +89158,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F87EEF9A-64DD-4C94-AADA-3FA669138FEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -89191,6 +89171,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{697D3734-930B-466A-983E-167E66A51EE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>